<commit_message>
perf: JPEG screenshots from the capture session (about 2.5x faster), parity compare reads JPEG
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-info.report.xlsx
+++ b/tools/importer/reports/import-info.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="954" uniqueCount="562">
   <si>
     <t>_reportFile</t>
   </si>
@@ -646,6 +646,36 @@
     <t>https://www.lufthansa.com/de/en/bid-upgrade</t>
   </si>
   <si>
+    <t>de/en/boarding.report.json</t>
+  </si>
+  <si>
+    <t>de/en/boarding</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:41:47.048Z</t>
+  </si>
+  <si>
+    <t>Boarding | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/boarding</t>
+  </si>
+  <si>
+    <t>de/en/business-class.report.json</t>
+  </si>
+  <si>
+    <t>de/en/business-class</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:48:53.691Z</t>
+  </si>
+  <si>
+    <t>Business Class | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/business-class</t>
+  </si>
+  <si>
     <t>de/en/children-on-board.report.json</t>
   </si>
   <si>
@@ -1216,6 +1246,24 @@
     <t>https://www.lufthansa.com/at/de/homepage#payment-social</t>
   </si>
   <si>
+    <t>de/de/discover-lufthansa/new-onboard-experience.report.json</t>
+  </si>
+  <si>
+    <t>["hero-campaign","hero-campaign","hero-campaign","hero-campaign","hero-campaign","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>de/de/discover-lufthansa/new-onboard-experience</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:18:27.478Z</t>
+  </si>
+  <si>
+    <t>New Onboard Experience | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/de/discover-lufthansa/new-onboard-experience</t>
+  </si>
+  <si>
     <t>de/de/during-your-trip/lhg-wifi.report.json</t>
   </si>
   <si>
@@ -1243,6 +1291,48 @@
     <t>https://www.lufthansa.com/de/de/homepage#payment-social</t>
   </si>
   <si>
+    <t>de/en/book-and-manage/pax-receipt.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/pax-receipt</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:48:40.390Z</t>
+  </si>
+  <si>
+    <t>Passenger receipt | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/pax-receipt</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/rebook.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/rebook</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:48:46.117Z</t>
+  </si>
+  <si>
+    <t>Flight Rebooking | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/rebook</t>
+  </si>
+  <si>
+    <t>de/en/discover-lufthansa/new-onboard-experience.report.json</t>
+  </si>
+  <si>
+    <t>de/en/discover-lufthansa/new-onboard-experience</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:18:19.974Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/discover-lufthansa/new-onboard-experience</t>
+  </si>
+  <si>
     <t>de/en/during-your-trip/lhg-wifi.report.json</t>
   </si>
   <si>
@@ -1300,6 +1390,39 @@
     <t>https://www.lufthansa.com/lhg/de/en/zz-test</t>
   </si>
   <si>
+    <t>de/de/100-years/history/menu-on-board.report.json</t>
+  </si>
+  <si>
+    <t>["hero-campaign","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
+  </si>
+  <si>
+    <t>de/de/100-years/history/menu-on-board</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:18:24.361Z</t>
+  </si>
+  <si>
+    <t>Menüs an Board | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/de/100-years/history/menu-on-board</t>
+  </si>
+  <si>
+    <t>de/en/100-years/history/menu-on-board.report.json</t>
+  </si>
+  <si>
+    <t>de/en/100-years/history/menu-on-board</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:18:17.824Z</t>
+  </si>
+  <si>
+    <t>Menus on Board | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/100-years/history/menu-on-board</t>
+  </si>
+  <si>
     <t>de/en/articles/explore-the-world/eat-see-do-berlin.report.json</t>
   </si>
   <si>
@@ -1316,6 +1439,210 @@
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/articles/explore-the-world/eat-see-do-berlin</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/additional-services/get-your-guide.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/additional-services/get-your-guide</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:41:49.789Z</t>
+  </si>
+  <si>
+    <t>Unforgettable travel experiences—GetYourGuide | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/additional-services/get-your-guide</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/additional-services/travel-insurances.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/additional-services/travel-insurances</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:41:51.782Z</t>
+  </si>
+  <si>
+    <t>Travel Care | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/additional-services/travel-insurances</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/digital-self-services/airline-apps.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/digital-self-services/airline-apps</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:41:54.185Z</t>
+  </si>
+  <si>
+    <t>Simply travel smarter | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/digital-self-services/airline-apps</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/air-baltic.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/air-baltic</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:41:56.300Z</t>
+  </si>
+  <si>
+    <t>Your Lufthansa flight with airBaltic | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/flights/air-baltic</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/ana.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/ana</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:41:58.144Z</t>
+  </si>
+  <si>
+    <t>ANA | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/flights/ana</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/giftvoucher.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-columns","carousel-cards","carousel-cards"]</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/giftvoucher</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:48:31.410Z</t>
+  </si>
+  <si>
+    <t>Buy a Lufthansa Gift Card &amp; give a flight as a gift | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/flights/giftvoucher</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/helvetic.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/helvetic</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:48:33.522Z</t>
+  </si>
+  <si>
+    <t>Helvetic | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/flights/helvetic</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/lufthansa-voucher.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/lufthansa-voucher</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:48:35.591Z</t>
+  </si>
+  <si>
+    <t>Terms of use for the purchase of Gift Vouchers | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/flights/lufthansa-voucher</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/wetlease-hub.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/wetlease-hub</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:48:37.711Z</t>
+  </si>
+  <si>
+    <t>Wet lease flights | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/flights/wetlease-hub</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/pax-receipt/invoices-different-countries.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/pax-receipt/invoices-different-countries</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:48:43.197Z</t>
+  </si>
+  <si>
+    <t>Invoices for different countries | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/pax-receipt/invoices-different-countries</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/rebook/involuntary-rebooking.report.json</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/rebook/involuntary-rebooking</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:48:49.236Z</t>
+  </si>
+  <si>
+    <t>Flight cancellation | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/rebook/involuntary-rebooking</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/rebook/voluntary-rebooking.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-columns","accordion-columns"]</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/rebook/voluntary-rebooking</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:48:51.326Z</t>
+  </si>
+  <si>
+    <t>Change flight | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/rebook/voluntary-rebooking</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/ana/faq.report.json</t>
+  </si>
+  <si>
+    <t>["accordion-columns","accordion-columns","accordion-columns","accordion-columns","accordion-columns","accordion-columns"]</t>
+  </si>
+  <si>
+    <t>de/en/book-and-manage/flights/ana/faq</t>
+  </si>
+  <si>
+    <t>2026-10-21T20:42:00.121Z</t>
+  </si>
+  <si>
+    <t>FAQs on travel with Lufthansa and ANA | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/book-and-manage/flights/ana/faq</t>
   </si>
   <si>
     <t>de/en/during-your-trip/food-and-beverages/onboard-delights/faq.report.json</t>
@@ -1758,7 +2085,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:I106"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
@@ -2876,7 +3203,7 @@
         <v>211</v>
       </c>
       <c r="B39" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="C39" t="s">
         <v>10</v>
@@ -2946,7 +3273,7 @@
         <v>13</v>
       </c>
       <c r="F41" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="G41" t="s">
         <v>223</v>
@@ -2963,7 +3290,7 @@
         <v>226</v>
       </c>
       <c r="B42" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="C42" t="s">
         <v>10</v>
@@ -3004,24 +3331,24 @@
         <v>13</v>
       </c>
       <c r="F43" t="s">
-        <v>31</v>
+        <v>98</v>
       </c>
       <c r="G43" t="s">
         <v>233</v>
       </c>
       <c r="H43" t="s">
-        <v>39</v>
+        <v>234</v>
       </c>
       <c r="I43" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B44" t="s">
-        <v>236</v>
+        <v>29</v>
       </c>
       <c r="C44" t="s">
         <v>10</v>
@@ -3033,21 +3360,21 @@
         <v>13</v>
       </c>
       <c r="F44" t="s">
+        <v>31</v>
+      </c>
+      <c r="G44" t="s">
         <v>238</v>
       </c>
-      <c r="G44" t="s">
+      <c r="H44" t="s">
         <v>239</v>
       </c>
-      <c r="H44" t="s">
+      <c r="I44" t="s">
         <v>240</v>
-      </c>
-      <c r="I44" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B45" t="s">
         <v>36</v>
@@ -3056,88 +3383,88 @@
         <v>10</v>
       </c>
       <c r="D45" t="s">
+        <v>242</v>
+      </c>
+      <c r="E45" t="s">
+        <v>13</v>
+      </c>
+      <c r="F45" t="s">
+        <v>31</v>
+      </c>
+      <c r="G45" t="s">
         <v>243</v>
       </c>
-      <c r="E45" t="s">
-        <v>13</v>
-      </c>
-      <c r="F45" t="s">
-        <v>31</v>
-      </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
+        <v>39</v>
+      </c>
+      <c r="I45" t="s">
         <v>244</v>
-      </c>
-      <c r="H45" t="s">
-        <v>245</v>
-      </c>
-      <c r="I45" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>245</v>
+      </c>
+      <c r="B46" t="s">
+        <v>246</v>
+      </c>
+      <c r="C46" t="s">
+        <v>10</v>
+      </c>
+      <c r="D46" t="s">
         <v>247</v>
       </c>
-      <c r="B46" t="s">
+      <c r="E46" t="s">
+        <v>13</v>
+      </c>
+      <c r="F46" t="s">
         <v>248</v>
       </c>
-      <c r="C46" t="s">
-        <v>10</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="G46" t="s">
         <v>249</v>
       </c>
-      <c r="E46" t="s">
-        <v>13</v>
-      </c>
-      <c r="F46" t="s">
-        <v>98</v>
-      </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>250</v>
       </c>
-      <c r="H46" t="s">
+      <c r="I46" t="s">
         <v>251</v>
-      </c>
-      <c r="I46" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
+        <v>252</v>
+      </c>
+      <c r="B47" t="s">
+        <v>36</v>
+      </c>
+      <c r="C47" t="s">
+        <v>10</v>
+      </c>
+      <c r="D47" t="s">
         <v>253</v>
       </c>
-      <c r="B47" t="s">
-        <v>29</v>
-      </c>
-      <c r="C47" t="s">
-        <v>10</v>
-      </c>
-      <c r="D47" t="s">
+      <c r="E47" t="s">
+        <v>13</v>
+      </c>
+      <c r="F47" t="s">
+        <v>31</v>
+      </c>
+      <c r="G47" t="s">
         <v>254</v>
       </c>
-      <c r="E47" t="s">
-        <v>13</v>
-      </c>
-      <c r="F47" t="s">
-        <v>31</v>
-      </c>
-      <c r="G47" t="s">
+      <c r="H47" t="s">
         <v>255</v>
       </c>
-      <c r="H47" t="s">
+      <c r="I47" t="s">
         <v>256</v>
-      </c>
-      <c r="I47" t="s">
-        <v>257</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>257</v>
+      </c>
+      <c r="B48" t="s">
         <v>258</v>
-      </c>
-      <c r="B48" t="s">
-        <v>103</v>
       </c>
       <c r="C48" t="s">
         <v>10</v>
@@ -3166,10 +3493,10 @@
         <v>263</v>
       </c>
       <c r="B49" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="C49" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D49" t="s">
         <v>264</v>
@@ -3178,56 +3505,56 @@
         <v>13</v>
       </c>
       <c r="F49" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G49" t="s">
         <v>265</v>
       </c>
       <c r="H49" t="s">
-        <v>10</v>
+        <v>266</v>
       </c>
       <c r="I49" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B50" t="s">
-        <v>18</v>
+        <v>103</v>
       </c>
       <c r="C50" t="s">
         <v>10</v>
       </c>
       <c r="D50" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E50" t="s">
         <v>13</v>
       </c>
       <c r="F50" t="s">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="G50" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H50" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="I50" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B51" t="s">
-        <v>273</v>
+        <v>10</v>
       </c>
       <c r="C51" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D51" t="s">
         <v>274</v>
@@ -3236,65 +3563,65 @@
         <v>13</v>
       </c>
       <c r="F51" t="s">
+        <v>14</v>
+      </c>
+      <c r="G51" t="s">
         <v>275</v>
       </c>
-      <c r="G51" t="s">
+      <c r="H51" t="s">
+        <v>10</v>
+      </c>
+      <c r="I51" t="s">
         <v>276</v>
-      </c>
-      <c r="H51" t="s">
-        <v>277</v>
-      </c>
-      <c r="I51" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>277</v>
+      </c>
+      <c r="B52" t="s">
+        <v>18</v>
+      </c>
+      <c r="C52" t="s">
+        <v>10</v>
+      </c>
+      <c r="D52" t="s">
+        <v>278</v>
+      </c>
+      <c r="E52" t="s">
+        <v>13</v>
+      </c>
+      <c r="F52" t="s">
+        <v>20</v>
+      </c>
+      <c r="G52" t="s">
         <v>279</v>
       </c>
-      <c r="B52" t="s">
-        <v>248</v>
-      </c>
-      <c r="C52" t="s">
-        <v>10</v>
-      </c>
-      <c r="D52" t="s">
+      <c r="H52" t="s">
         <v>280</v>
       </c>
-      <c r="E52" t="s">
-        <v>13</v>
-      </c>
-      <c r="F52" t="s">
-        <v>98</v>
-      </c>
-      <c r="G52" t="s">
+      <c r="I52" t="s">
         <v>281</v>
-      </c>
-      <c r="H52" t="s">
-        <v>282</v>
-      </c>
-      <c r="I52" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>282</v>
+      </c>
+      <c r="B53" t="s">
+        <v>283</v>
+      </c>
+      <c r="C53" t="s">
+        <v>10</v>
+      </c>
+      <c r="D53" t="s">
         <v>284</v>
       </c>
-      <c r="B53" t="s">
-        <v>36</v>
-      </c>
-      <c r="C53" t="s">
-        <v>10</v>
-      </c>
-      <c r="D53" t="s">
+      <c r="E53" t="s">
+        <v>13</v>
+      </c>
+      <c r="F53" t="s">
         <v>285</v>
-      </c>
-      <c r="E53" t="s">
-        <v>13</v>
-      </c>
-      <c r="F53" t="s">
-        <v>31</v>
       </c>
       <c r="G53" t="s">
         <v>286</v>
@@ -3311,7 +3638,7 @@
         <v>289</v>
       </c>
       <c r="B54" t="s">
-        <v>103</v>
+        <v>258</v>
       </c>
       <c r="C54" t="s">
         <v>10</v>
@@ -3352,7 +3679,7 @@
         <v>13</v>
       </c>
       <c r="F55" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="G55" t="s">
         <v>296</v>
@@ -3369,7 +3696,7 @@
         <v>299</v>
       </c>
       <c r="B56" t="s">
-        <v>36</v>
+        <v>103</v>
       </c>
       <c r="C56" t="s">
         <v>10</v>
@@ -3381,7 +3708,7 @@
         <v>13</v>
       </c>
       <c r="F56" t="s">
-        <v>31</v>
+        <v>98</v>
       </c>
       <c r="G56" t="s">
         <v>301</v>
@@ -3410,7 +3737,7 @@
         <v>13</v>
       </c>
       <c r="F57" t="s">
-        <v>31</v>
+        <v>98</v>
       </c>
       <c r="G57" t="s">
         <v>306</v>
@@ -3439,7 +3766,7 @@
         <v>13</v>
       </c>
       <c r="F58" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="G58" t="s">
         <v>311</v>
@@ -3456,10 +3783,10 @@
         <v>314</v>
       </c>
       <c r="B59" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C59" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D59" t="s">
         <v>315</v>
@@ -3468,137 +3795,137 @@
         <v>13</v>
       </c>
       <c r="F59" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G59" t="s">
         <v>316</v>
       </c>
       <c r="H59" t="s">
-        <v>10</v>
+        <v>317</v>
       </c>
       <c r="I59" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B60" t="s">
-        <v>90</v>
+        <v>36</v>
       </c>
       <c r="C60" t="s">
         <v>10</v>
       </c>
       <c r="D60" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E60" t="s">
         <v>13</v>
       </c>
       <c r="F60" t="s">
-        <v>31</v>
+        <v>98</v>
       </c>
       <c r="G60" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="H60" t="s">
-        <v>93</v>
+        <v>322</v>
       </c>
       <c r="I60" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B61" t="s">
-        <v>323</v>
+        <v>10</v>
       </c>
       <c r="C61" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D61" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E61" t="s">
         <v>13</v>
       </c>
       <c r="F61" t="s">
-        <v>325</v>
+        <v>14</v>
       </c>
       <c r="G61" t="s">
         <v>326</v>
       </c>
       <c r="H61" t="s">
+        <v>10</v>
+      </c>
+      <c r="I61" t="s">
         <v>327</v>
-      </c>
-      <c r="I61" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>328</v>
+      </c>
+      <c r="B62" t="s">
+        <v>90</v>
+      </c>
+      <c r="C62" t="s">
+        <v>10</v>
+      </c>
+      <c r="D62" t="s">
         <v>329</v>
       </c>
-      <c r="B62" t="s">
-        <v>96</v>
-      </c>
-      <c r="C62" t="s">
-        <v>10</v>
-      </c>
-      <c r="D62" t="s">
+      <c r="E62" t="s">
+        <v>13</v>
+      </c>
+      <c r="F62" t="s">
+        <v>31</v>
+      </c>
+      <c r="G62" t="s">
         <v>330</v>
       </c>
-      <c r="E62" t="s">
-        <v>13</v>
-      </c>
-      <c r="F62" t="s">
-        <v>98</v>
-      </c>
-      <c r="G62" t="s">
+      <c r="H62" t="s">
+        <v>93</v>
+      </c>
+      <c r="I62" t="s">
         <v>331</v>
-      </c>
-      <c r="H62" t="s">
-        <v>332</v>
-      </c>
-      <c r="I62" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>332</v>
+      </c>
+      <c r="B63" t="s">
+        <v>333</v>
+      </c>
+      <c r="C63" t="s">
+        <v>10</v>
+      </c>
+      <c r="D63" t="s">
         <v>334</v>
       </c>
-      <c r="B63" t="s">
+      <c r="E63" t="s">
+        <v>13</v>
+      </c>
+      <c r="F63" t="s">
         <v>335</v>
       </c>
-      <c r="C63" t="s">
-        <v>10</v>
-      </c>
-      <c r="D63" t="s">
+      <c r="G63" t="s">
         <v>336</v>
       </c>
-      <c r="E63" t="s">
-        <v>13</v>
-      </c>
-      <c r="F63" t="s">
-        <v>98</v>
-      </c>
-      <c r="G63" t="s">
+      <c r="H63" t="s">
         <v>337</v>
       </c>
-      <c r="H63" t="s">
+      <c r="I63" t="s">
         <v>338</v>
-      </c>
-      <c r="I63" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B64" t="s">
         <v>96</v>
@@ -3607,7 +3934,7 @@
         <v>10</v>
       </c>
       <c r="D64" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="E64" t="s">
         <v>13</v>
@@ -3616,21 +3943,21 @@
         <v>98</v>
       </c>
       <c r="G64" t="s">
+        <v>341</v>
+      </c>
+      <c r="H64" t="s">
         <v>342</v>
       </c>
-      <c r="H64" t="s">
+      <c r="I64" t="s">
         <v>343</v>
-      </c>
-      <c r="I64" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>344</v>
+      </c>
+      <c r="B65" t="s">
         <v>345</v>
-      </c>
-      <c r="B65" t="s">
-        <v>36</v>
       </c>
       <c r="C65" t="s">
         <v>10</v>
@@ -3659,7 +3986,7 @@
         <v>350</v>
       </c>
       <c r="B66" t="s">
-        <v>36</v>
+        <v>96</v>
       </c>
       <c r="C66" t="s">
         <v>10</v>
@@ -3688,7 +4015,7 @@
         <v>355</v>
       </c>
       <c r="B67" t="s">
-        <v>96</v>
+        <v>36</v>
       </c>
       <c r="C67" t="s">
         <v>10</v>
@@ -3746,33 +4073,33 @@
         <v>365</v>
       </c>
       <c r="B69" t="s">
+        <v>96</v>
+      </c>
+      <c r="C69" t="s">
+        <v>10</v>
+      </c>
+      <c r="D69" t="s">
         <v>366</v>
       </c>
-      <c r="C69" t="s">
-        <v>10</v>
-      </c>
-      <c r="D69" t="s">
+      <c r="E69" t="s">
+        <v>13</v>
+      </c>
+      <c r="F69" t="s">
+        <v>98</v>
+      </c>
+      <c r="G69" t="s">
         <v>367</v>
       </c>
-      <c r="E69" t="s">
-        <v>13</v>
-      </c>
-      <c r="F69" t="s">
+      <c r="H69" t="s">
         <v>368</v>
       </c>
-      <c r="G69" t="s">
+      <c r="I69" t="s">
         <v>369</v>
-      </c>
-      <c r="H69" t="s">
-        <v>370</v>
-      </c>
-      <c r="I69" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="B70" t="s">
         <v>36</v>
@@ -3781,94 +4108,94 @@
         <v>10</v>
       </c>
       <c r="D70" t="s">
+        <v>371</v>
+      </c>
+      <c r="E70" t="s">
+        <v>13</v>
+      </c>
+      <c r="F70" t="s">
+        <v>98</v>
+      </c>
+      <c r="G70" t="s">
+        <v>372</v>
+      </c>
+      <c r="H70" t="s">
         <v>373</v>
       </c>
-      <c r="E70" t="s">
-        <v>13</v>
-      </c>
-      <c r="F70" t="s">
-        <v>31</v>
-      </c>
-      <c r="G70" t="s">
+      <c r="I70" t="s">
         <v>374</v>
-      </c>
-      <c r="H70" t="s">
-        <v>375</v>
-      </c>
-      <c r="I70" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>375</v>
+      </c>
+      <c r="B71" t="s">
+        <v>376</v>
+      </c>
+      <c r="C71" t="s">
+        <v>10</v>
+      </c>
+      <c r="D71" t="s">
         <v>377</v>
       </c>
-      <c r="B71" t="s">
-        <v>10</v>
-      </c>
-      <c r="C71" t="s">
-        <v>11</v>
-      </c>
-      <c r="D71" t="s">
+      <c r="E71" t="s">
+        <v>13</v>
+      </c>
+      <c r="F71" t="s">
         <v>378</v>
-      </c>
-      <c r="E71" t="s">
-        <v>13</v>
-      </c>
-      <c r="F71" t="s">
-        <v>14</v>
       </c>
       <c r="G71" t="s">
         <v>379</v>
       </c>
       <c r="H71" t="s">
-        <v>10</v>
+        <v>380</v>
       </c>
       <c r="I71" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B72" t="s">
-        <v>18</v>
+        <v>36</v>
       </c>
       <c r="C72" t="s">
         <v>10</v>
       </c>
       <c r="D72" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E72" t="s">
         <v>13</v>
       </c>
       <c r="F72" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="G72" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="H72" t="s">
-        <v>270</v>
+        <v>385</v>
       </c>
       <c r="I72" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B73" t="s">
         <v>10</v>
       </c>
       <c r="C73" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D73" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="E73" t="s">
         <v>13</v>
@@ -3877,56 +4204,56 @@
         <v>14</v>
       </c>
       <c r="G73" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="H73" t="s">
         <v>10</v>
       </c>
       <c r="I73" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B74" t="s">
-        <v>390</v>
+        <v>18</v>
       </c>
       <c r="C74" t="s">
         <v>10</v>
       </c>
       <c r="D74" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E74" t="s">
         <v>13</v>
       </c>
       <c r="F74" t="s">
-        <v>392</v>
+        <v>20</v>
       </c>
       <c r="G74" t="s">
         <v>393</v>
       </c>
       <c r="H74" t="s">
+        <v>280</v>
+      </c>
+      <c r="I74" t="s">
         <v>394</v>
-      </c>
-      <c r="I74" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>395</v>
+      </c>
+      <c r="B75" t="s">
+        <v>10</v>
+      </c>
+      <c r="C75" t="s">
+        <v>14</v>
+      </c>
+      <c r="D75" t="s">
         <v>396</v>
-      </c>
-      <c r="B75" t="s">
-        <v>10</v>
-      </c>
-      <c r="C75" t="s">
-        <v>397</v>
-      </c>
-      <c r="D75" t="s">
-        <v>398</v>
       </c>
       <c r="E75" t="s">
         <v>13</v>
@@ -3935,33 +4262,33 @@
         <v>14</v>
       </c>
       <c r="G75" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="H75" t="s">
         <v>10</v>
       </c>
       <c r="I75" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>399</v>
+      </c>
+      <c r="B76" t="s">
+        <v>400</v>
+      </c>
+      <c r="C76" t="s">
+        <v>10</v>
+      </c>
+      <c r="D76" t="s">
         <v>401</v>
       </c>
-      <c r="B76" t="s">
-        <v>84</v>
-      </c>
-      <c r="C76" t="s">
-        <v>10</v>
-      </c>
-      <c r="D76" t="s">
+      <c r="E76" t="s">
+        <v>13</v>
+      </c>
+      <c r="F76" t="s">
         <v>402</v>
-      </c>
-      <c r="E76" t="s">
-        <v>13</v>
-      </c>
-      <c r="F76" t="s">
-        <v>31</v>
       </c>
       <c r="G76" t="s">
         <v>403</v>
@@ -3981,10 +4308,10 @@
         <v>10</v>
       </c>
       <c r="C77" t="s">
-        <v>397</v>
+        <v>407</v>
       </c>
       <c r="D77" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E77" t="s">
         <v>13</v>
@@ -3993,85 +4320,85 @@
         <v>14</v>
       </c>
       <c r="G77" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="H77" t="s">
         <v>10</v>
       </c>
       <c r="I77" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B78" t="s">
-        <v>84</v>
+        <v>412</v>
       </c>
       <c r="C78" t="s">
         <v>10</v>
       </c>
       <c r="D78" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="E78" t="s">
         <v>13</v>
       </c>
       <c r="F78" t="s">
-        <v>31</v>
+        <v>116</v>
       </c>
       <c r="G78" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="H78" t="s">
-        <v>404</v>
+        <v>415</v>
       </c>
       <c r="I78" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="B79" t="s">
-        <v>10</v>
+        <v>84</v>
       </c>
       <c r="C79" t="s">
-        <v>397</v>
+        <v>10</v>
       </c>
       <c r="D79" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="E79" t="s">
         <v>13</v>
       </c>
       <c r="F79" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G79" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="H79" t="s">
-        <v>10</v>
+        <v>420</v>
       </c>
       <c r="I79" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="B80" t="s">
         <v>10</v>
       </c>
       <c r="C80" t="s">
-        <v>397</v>
+        <v>407</v>
       </c>
       <c r="D80" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="E80" t="s">
         <v>13</v>
@@ -4080,97 +4407,97 @@
         <v>14</v>
       </c>
       <c r="G80" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="H80" t="s">
         <v>10</v>
       </c>
       <c r="I80" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="B81" t="s">
-        <v>423</v>
+        <v>36</v>
       </c>
       <c r="C81" t="s">
         <v>10</v>
       </c>
       <c r="D81" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="E81" t="s">
         <v>13</v>
       </c>
       <c r="F81" t="s">
-        <v>425</v>
+        <v>31</v>
       </c>
       <c r="G81" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="H81" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="I81" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B82" t="s">
-        <v>430</v>
+        <v>36</v>
       </c>
       <c r="C82" t="s">
         <v>10</v>
       </c>
       <c r="D82" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="E82" t="s">
         <v>13</v>
       </c>
       <c r="F82" t="s">
-        <v>432</v>
+        <v>31</v>
       </c>
       <c r="G82" t="s">
         <v>433</v>
       </c>
       <c r="H82" t="s">
-        <v>10</v>
+        <v>434</v>
       </c>
       <c r="I82" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="B83" t="s">
-        <v>84</v>
+        <v>412</v>
       </c>
       <c r="C83" t="s">
         <v>10</v>
       </c>
       <c r="D83" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E83" t="s">
         <v>13</v>
       </c>
       <c r="F83" t="s">
-        <v>31</v>
+        <v>116</v>
       </c>
       <c r="G83" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="H83" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="I83" t="s">
         <v>439</v>
@@ -4181,57 +4508,666 @@
         <v>440</v>
       </c>
       <c r="B84" t="s">
+        <v>84</v>
+      </c>
+      <c r="C84" t="s">
+        <v>10</v>
+      </c>
+      <c r="D84" t="s">
         <v>441</v>
       </c>
-      <c r="C84" t="s">
-        <v>10</v>
-      </c>
-      <c r="D84" t="s">
+      <c r="E84" t="s">
+        <v>13</v>
+      </c>
+      <c r="F84" t="s">
+        <v>31</v>
+      </c>
+      <c r="G84" t="s">
         <v>442</v>
       </c>
-      <c r="E84" t="s">
-        <v>13</v>
-      </c>
-      <c r="F84" t="s">
-        <v>425</v>
-      </c>
-      <c r="G84" t="s">
+      <c r="H84" t="s">
+        <v>420</v>
+      </c>
+      <c r="I84" t="s">
         <v>443</v>
-      </c>
-      <c r="H84" t="s">
-        <v>444</v>
-      </c>
-      <c r="I84" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>444</v>
+      </c>
+      <c r="B85" t="s">
+        <v>10</v>
+      </c>
+      <c r="C85" t="s">
+        <v>407</v>
+      </c>
+      <c r="D85" t="s">
+        <v>445</v>
+      </c>
+      <c r="E85" t="s">
+        <v>13</v>
+      </c>
+      <c r="F85" t="s">
+        <v>14</v>
+      </c>
+      <c r="G85" t="s">
         <v>446</v>
       </c>
-      <c r="B85" t="s">
+      <c r="H85" t="s">
+        <v>10</v>
+      </c>
+      <c r="I85" t="s">
         <v>447</v>
       </c>
-      <c r="C85" t="s">
-        <v>10</v>
-      </c>
-      <c r="D85" t="s">
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>448</v>
       </c>
-      <c r="E85" t="s">
-        <v>13</v>
-      </c>
-      <c r="F85" t="s">
+      <c r="B86" t="s">
+        <v>10</v>
+      </c>
+      <c r="C86" t="s">
+        <v>407</v>
+      </c>
+      <c r="D86" t="s">
         <v>449</v>
       </c>
-      <c r="G85" t="s">
+      <c r="E86" t="s">
+        <v>13</v>
+      </c>
+      <c r="F86" t="s">
+        <v>14</v>
+      </c>
+      <c r="G86" t="s">
         <v>450</v>
       </c>
-      <c r="H85" t="s">
+      <c r="H86" t="s">
+        <v>10</v>
+      </c>
+      <c r="I86" t="s">
         <v>451</v>
       </c>
-      <c r="I85" t="s">
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>452</v>
+      </c>
+      <c r="B87" t="s">
+        <v>453</v>
+      </c>
+      <c r="C87" t="s">
+        <v>10</v>
+      </c>
+      <c r="D87" t="s">
+        <v>454</v>
+      </c>
+      <c r="E87" t="s">
+        <v>13</v>
+      </c>
+      <c r="F87" t="s">
+        <v>455</v>
+      </c>
+      <c r="G87" t="s">
+        <v>456</v>
+      </c>
+      <c r="H87" t="s">
+        <v>457</v>
+      </c>
+      <c r="I87" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>459</v>
+      </c>
+      <c r="B88" t="s">
+        <v>460</v>
+      </c>
+      <c r="C88" t="s">
+        <v>10</v>
+      </c>
+      <c r="D88" t="s">
+        <v>461</v>
+      </c>
+      <c r="E88" t="s">
+        <v>13</v>
+      </c>
+      <c r="F88" t="s">
+        <v>116</v>
+      </c>
+      <c r="G88" t="s">
+        <v>462</v>
+      </c>
+      <c r="H88" t="s">
+        <v>463</v>
+      </c>
+      <c r="I88" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>465</v>
+      </c>
+      <c r="B89" t="s">
+        <v>460</v>
+      </c>
+      <c r="C89" t="s">
+        <v>10</v>
+      </c>
+      <c r="D89" t="s">
+        <v>466</v>
+      </c>
+      <c r="E89" t="s">
+        <v>13</v>
+      </c>
+      <c r="F89" t="s">
+        <v>116</v>
+      </c>
+      <c r="G89" t="s">
+        <v>467</v>
+      </c>
+      <c r="H89" t="s">
+        <v>468</v>
+      </c>
+      <c r="I89" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>470</v>
+      </c>
+      <c r="B90" t="s">
+        <v>471</v>
+      </c>
+      <c r="C90" t="s">
+        <v>10</v>
+      </c>
+      <c r="D90" t="s">
+        <v>472</v>
+      </c>
+      <c r="E90" t="s">
+        <v>13</v>
+      </c>
+      <c r="F90" t="s">
+        <v>473</v>
+      </c>
+      <c r="G90" t="s">
+        <v>474</v>
+      </c>
+      <c r="H90" t="s">
+        <v>10</v>
+      </c>
+      <c r="I90" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>476</v>
+      </c>
+      <c r="B91" t="s">
+        <v>36</v>
+      </c>
+      <c r="C91" t="s">
+        <v>10</v>
+      </c>
+      <c r="D91" t="s">
+        <v>477</v>
+      </c>
+      <c r="E91" t="s">
+        <v>13</v>
+      </c>
+      <c r="F91" t="s">
+        <v>31</v>
+      </c>
+      <c r="G91" t="s">
+        <v>478</v>
+      </c>
+      <c r="H91" t="s">
+        <v>479</v>
+      </c>
+      <c r="I91" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>481</v>
+      </c>
+      <c r="B92" t="s">
+        <v>90</v>
+      </c>
+      <c r="C92" t="s">
+        <v>10</v>
+      </c>
+      <c r="D92" t="s">
+        <v>482</v>
+      </c>
+      <c r="E92" t="s">
+        <v>13</v>
+      </c>
+      <c r="F92" t="s">
+        <v>31</v>
+      </c>
+      <c r="G92" t="s">
+        <v>483</v>
+      </c>
+      <c r="H92" t="s">
+        <v>484</v>
+      </c>
+      <c r="I92" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>486</v>
+      </c>
+      <c r="B93" t="s">
+        <v>36</v>
+      </c>
+      <c r="C93" t="s">
+        <v>10</v>
+      </c>
+      <c r="D93" t="s">
+        <v>487</v>
+      </c>
+      <c r="E93" t="s">
+        <v>13</v>
+      </c>
+      <c r="F93" t="s">
+        <v>31</v>
+      </c>
+      <c r="G93" t="s">
+        <v>488</v>
+      </c>
+      <c r="H93" t="s">
+        <v>489</v>
+      </c>
+      <c r="I93" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>491</v>
+      </c>
+      <c r="B94" t="s">
+        <v>36</v>
+      </c>
+      <c r="C94" t="s">
+        <v>10</v>
+      </c>
+      <c r="D94" t="s">
+        <v>492</v>
+      </c>
+      <c r="E94" t="s">
+        <v>13</v>
+      </c>
+      <c r="F94" t="s">
+        <v>31</v>
+      </c>
+      <c r="G94" t="s">
+        <v>493</v>
+      </c>
+      <c r="H94" t="s">
+        <v>494</v>
+      </c>
+      <c r="I94" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>496</v>
+      </c>
+      <c r="B95" t="s">
+        <v>84</v>
+      </c>
+      <c r="C95" t="s">
+        <v>10</v>
+      </c>
+      <c r="D95" t="s">
+        <v>497</v>
+      </c>
+      <c r="E95" t="s">
+        <v>13</v>
+      </c>
+      <c r="F95" t="s">
+        <v>31</v>
+      </c>
+      <c r="G95" t="s">
+        <v>498</v>
+      </c>
+      <c r="H95" t="s">
+        <v>499</v>
+      </c>
+      <c r="I95" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>501</v>
+      </c>
+      <c r="B96" t="s">
+        <v>502</v>
+      </c>
+      <c r="C96" t="s">
+        <v>10</v>
+      </c>
+      <c r="D96" t="s">
+        <v>503</v>
+      </c>
+      <c r="E96" t="s">
+        <v>13</v>
+      </c>
+      <c r="F96" t="s">
+        <v>31</v>
+      </c>
+      <c r="G96" t="s">
+        <v>504</v>
+      </c>
+      <c r="H96" t="s">
+        <v>505</v>
+      </c>
+      <c r="I96" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>507</v>
+      </c>
+      <c r="B97" t="s">
+        <v>84</v>
+      </c>
+      <c r="C97" t="s">
+        <v>10</v>
+      </c>
+      <c r="D97" t="s">
+        <v>508</v>
+      </c>
+      <c r="E97" t="s">
+        <v>13</v>
+      </c>
+      <c r="F97" t="s">
+        <v>31</v>
+      </c>
+      <c r="G97" t="s">
+        <v>509</v>
+      </c>
+      <c r="H97" t="s">
+        <v>510</v>
+      </c>
+      <c r="I97" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>512</v>
+      </c>
+      <c r="B98" t="s">
+        <v>84</v>
+      </c>
+      <c r="C98" t="s">
+        <v>10</v>
+      </c>
+      <c r="D98" t="s">
+        <v>513</v>
+      </c>
+      <c r="E98" t="s">
+        <v>13</v>
+      </c>
+      <c r="F98" t="s">
+        <v>31</v>
+      </c>
+      <c r="G98" t="s">
+        <v>514</v>
+      </c>
+      <c r="H98" t="s">
+        <v>515</v>
+      </c>
+      <c r="I98" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>517</v>
+      </c>
+      <c r="B99" t="s">
+        <v>36</v>
+      </c>
+      <c r="C99" t="s">
+        <v>10</v>
+      </c>
+      <c r="D99" t="s">
+        <v>518</v>
+      </c>
+      <c r="E99" t="s">
+        <v>13</v>
+      </c>
+      <c r="F99" t="s">
+        <v>31</v>
+      </c>
+      <c r="G99" t="s">
+        <v>519</v>
+      </c>
+      <c r="H99" t="s">
+        <v>520</v>
+      </c>
+      <c r="I99" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>522</v>
+      </c>
+      <c r="B100" t="s">
+        <v>36</v>
+      </c>
+      <c r="C100" t="s">
+        <v>10</v>
+      </c>
+      <c r="D100" t="s">
+        <v>523</v>
+      </c>
+      <c r="E100" t="s">
+        <v>13</v>
+      </c>
+      <c r="F100" t="s">
+        <v>31</v>
+      </c>
+      <c r="G100" t="s">
+        <v>524</v>
+      </c>
+      <c r="H100" t="s">
+        <v>525</v>
+      </c>
+      <c r="I100" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>527</v>
+      </c>
+      <c r="B101" t="s">
+        <v>84</v>
+      </c>
+      <c r="C101" t="s">
+        <v>10</v>
+      </c>
+      <c r="D101" t="s">
+        <v>528</v>
+      </c>
+      <c r="E101" t="s">
+        <v>13</v>
+      </c>
+      <c r="F101" t="s">
+        <v>31</v>
+      </c>
+      <c r="G101" t="s">
+        <v>529</v>
+      </c>
+      <c r="H101" t="s">
+        <v>530</v>
+      </c>
+      <c r="I101" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>532</v>
+      </c>
+      <c r="B102" t="s">
+        <v>533</v>
+      </c>
+      <c r="C102" t="s">
+        <v>10</v>
+      </c>
+      <c r="D102" t="s">
+        <v>534</v>
+      </c>
+      <c r="E102" t="s">
+        <v>13</v>
+      </c>
+      <c r="F102" t="s">
+        <v>31</v>
+      </c>
+      <c r="G102" t="s">
+        <v>535</v>
+      </c>
+      <c r="H102" t="s">
+        <v>536</v>
+      </c>
+      <c r="I102" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>538</v>
+      </c>
+      <c r="B103" t="s">
+        <v>539</v>
+      </c>
+      <c r="C103" t="s">
+        <v>10</v>
+      </c>
+      <c r="D103" t="s">
+        <v>540</v>
+      </c>
+      <c r="E103" t="s">
+        <v>13</v>
+      </c>
+      <c r="F103" t="s">
+        <v>31</v>
+      </c>
+      <c r="G103" t="s">
+        <v>541</v>
+      </c>
+      <c r="H103" t="s">
+        <v>542</v>
+      </c>
+      <c r="I103" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>544</v>
+      </c>
+      <c r="B104" t="s">
+        <v>84</v>
+      </c>
+      <c r="C104" t="s">
+        <v>10</v>
+      </c>
+      <c r="D104" t="s">
+        <v>545</v>
+      </c>
+      <c r="E104" t="s">
+        <v>13</v>
+      </c>
+      <c r="F104" t="s">
+        <v>31</v>
+      </c>
+      <c r="G104" t="s">
+        <v>546</v>
+      </c>
+      <c r="H104" t="s">
+        <v>547</v>
+      </c>
+      <c r="I104" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>549</v>
+      </c>
+      <c r="B105" t="s">
+        <v>550</v>
+      </c>
+      <c r="C105" t="s">
+        <v>10</v>
+      </c>
+      <c r="D105" t="s">
+        <v>551</v>
+      </c>
+      <c r="E105" t="s">
+        <v>13</v>
+      </c>
+      <c r="F105" t="s">
+        <v>455</v>
+      </c>
+      <c r="G105" t="s">
+        <v>552</v>
+      </c>
+      <c r="H105" t="s">
+        <v>553</v>
+      </c>
+      <c r="I105" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>555</v>
+      </c>
+      <c r="B106" t="s">
+        <v>556</v>
+      </c>
+      <c r="C106" t="s">
+        <v>10</v>
+      </c>
+      <c r="D106" t="s">
+        <v>557</v>
+      </c>
+      <c r="E106" t="s">
+        <v>13</v>
+      </c>
+      <c r="F106" t="s">
+        <v>558</v>
+      </c>
+      <c r="G106" t="s">
+        <v>559</v>
+      </c>
+      <c r="H106" t="s">
+        <v>560</v>
+      </c>
+      <c r="I106" t="s">
+        <v>561</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: section metadata placement, blob/data icon handling, AirCore typography, spacing, share links hidden, hero/lightbox parser fixes, date/price formats; re-imported 161 pages
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-info.report.xlsx
+++ b/tools/importer/reports/import-info.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1431" uniqueCount="827">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1575" uniqueCount="906">
   <si>
     <t>_reportFile</t>
   </si>
@@ -76,7 +76,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-10-21T18:23:02.162Z</t>
+    <t>2026-10-21T22:28:43.065Z</t>
   </si>
   <si>
     <t>Jetzt Flug buchen – mit Lufthansa zu über 200 Zielen reisen | Lufthansa</t>
@@ -109,7 +109,7 @@
     <t>info</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:02.890Z</t>
+    <t>2026-10-21T22:32:06.345Z</t>
   </si>
   <si>
     <t>Doctor on Board – Gut zu wissen | Lufthansa</t>
@@ -127,7 +127,7 @@
     <t>de/de/doctor-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:59.676Z</t>
+    <t>2026-10-21T22:32:01.082Z</t>
   </si>
   <si>
     <t>Doctor on Board | Lufthansa</t>
@@ -154,7 +154,7 @@
     <t>de/de/homepage</t>
   </si>
   <si>
-    <t>2026-10-21T18:22:56.557Z</t>
+    <t>2026-10-21T22:28:39.550Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/homepage</t>
@@ -166,7 +166,7 @@
     <t>de/de/kinder-an-bord</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:06.100Z</t>
+    <t>2026-10-21T22:31:25.780Z</t>
   </si>
   <si>
     <t>Mit Kindern und Babys an Bord | Lufthansa</t>
@@ -181,7 +181,7 @@
     <t>de/de/kindermenues-an-bord</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:08.100Z</t>
+    <t>2026-10-21T22:31:30.745Z</t>
   </si>
   <si>
     <t>Kindermenüs | Lufthansa</t>
@@ -196,7 +196,7 @@
     <t>de/de/lufthansa-first-class-entertainment</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:10.363Z</t>
+    <t>2026-10-21T22:34:02.541Z</t>
   </si>
   <si>
     <t>Entertainment Welt | Lufthansa</t>
@@ -211,7 +211,7 @@
     <t>de/de/lufthansa-first-class-komfort</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:07.683Z</t>
+    <t>2026-10-21T22:32:46.333Z</t>
   </si>
   <si>
     <t>Komfort an Bord der First Class | Lufthansa</t>
@@ -226,7 +226,7 @@
     <t>de/de/menues-auf-langstreckenfluegen</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:13.801Z</t>
+    <t>2026-10-21T22:34:20.948Z</t>
   </si>
   <si>
     <t>Menüs auf Langstreckenflügen | Lufthansa</t>
@@ -241,7 +241,7 @@
     <t>de/de/menues-reiseklassen</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:16.384Z</t>
+    <t>2026-10-21T22:34:25.475Z</t>
   </si>
   <si>
     <t>Menüs in unseren Reiseklassen | Lufthansa</t>
@@ -271,7 +271,7 @@
     <t>de/de/onboard-delights-faq</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:10.658Z</t>
+    <t>2026-10-21T22:32:11.489Z</t>
   </si>
   <si>
     <t>faq | Lufthansa</t>
@@ -289,7 +289,7 @@
     <t>de/de/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:18.569Z</t>
+    <t>2026-10-21T22:34:32.444Z</t>
   </si>
   <si>
     <t>Onboard Delights | Lufthansa</t>
@@ -310,7 +310,7 @@
     <t>hub</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:17.458Z</t>
+    <t>2026-10-21T22:29:36.688Z</t>
   </si>
   <si>
     <t>Services an Bord | Lufthansa</t>
@@ -328,7 +328,7 @@
     <t>de/de/speisen-und-getraenke</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:14.861Z</t>
+    <t>2026-10-21T22:29:10.255Z</t>
   </si>
   <si>
     <t>Menüs an Bord | Lufthansa</t>
@@ -343,7 +343,7 @@
     <t>de/de/unterhaltung-an-bord</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:12.411Z</t>
+    <t>2026-10-21T22:34:47.115Z</t>
   </si>
   <si>
     <t>Unterhaltung an Bord | Lufthansa</t>
@@ -403,7 +403,7 @@
     <t>de/en/accessible-travel</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:22.603Z</t>
+    <t>2026-10-21T22:29:47.559Z</t>
   </si>
   <si>
     <t>Accessible travel | Lufthansa</t>
@@ -418,7 +418,7 @@
     <t>de/en/add-sports-baggage</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:24.619Z</t>
+    <t>2026-10-21T22:29:49.905Z</t>
   </si>
   <si>
     <t>Add sports baggage | Lufthansa</t>
@@ -433,7 +433,7 @@
     <t>de/en/additional-services</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:31.376Z</t>
+    <t>2026-10-21T22:28:54.578Z</t>
   </si>
   <si>
     <t>Extra services | Lufthansa</t>
@@ -448,7 +448,7 @@
     <t>de/en/addresses-worldwide</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:26.855Z</t>
+    <t>2026-10-21T22:29:51.608Z</t>
   </si>
   <si>
     <t>Addresses worldwide | Lufthansa</t>
@@ -463,7 +463,7 @@
     <t>de/en/admission-rules</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:29.362Z</t>
+    <t>2026-10-21T22:29:53.742Z</t>
   </si>
   <si>
     <t>Access to our lounges | Lufthansa</t>
@@ -478,7 +478,7 @@
     <t>de/en/advance-seat-reservation</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:31.443Z</t>
+    <t>2026-10-21T22:29:57.170Z</t>
   </si>
   <si>
     <t>Advance seat reservation | Lufthansa</t>
@@ -496,7 +496,7 @@
     <t>de/en/advice-for-travellers-with-special-needs-to-and-from-the-usa</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:34.110Z</t>
+    <t>2026-10-21T22:29:59.570Z</t>
   </si>
   <si>
     <t>Information about accessible travel to the USA | Lufthansa</t>
@@ -511,7 +511,7 @@
     <t>de/en/affiliatemarketing</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:35.831Z</t>
+    <t>2026-10-21T22:30:02.705Z</t>
   </si>
   <si>
     <t>Affiliate marketing | Lufthansa</t>
@@ -526,7 +526,7 @@
     <t>de/en/airport-information</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:33.884Z</t>
+    <t>2026-10-21T22:28:57.157Z</t>
   </si>
   <si>
     <t>Airport information | Lufthansa</t>
@@ -541,7 +541,7 @@
     <t>de/en/all-check-in</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:37.770Z</t>
+    <t>2026-10-21T22:30:05.727Z</t>
   </si>
   <si>
     <t>All check-in options | Lufthansa</t>
@@ -556,7 +556,7 @@
     <t>de/en/arrival-services</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:39.836Z</t>
+    <t>2026-10-21T22:30:08.819Z</t>
   </si>
   <si>
     <t>Arrival services | Lufthansa</t>
@@ -571,7 +571,7 @@
     <t>de/en/assistenzhunde</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:42.444Z</t>
+    <t>2026-10-21T22:30:11.883Z</t>
   </si>
   <si>
     <t>Assistance dogs | Lufthansa</t>
@@ -586,7 +586,7 @@
     <t>de/en/automatic-check-in</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:44.459Z</t>
+    <t>2026-10-21T22:30:14.648Z</t>
   </si>
   <si>
     <t>Automated check-in | Lufthansa</t>
@@ -604,7 +604,7 @@
     <t>de/en/baggage-irregularities</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:46.494Z</t>
+    <t>2026-10-21T22:30:16.983Z</t>
   </si>
   <si>
     <t>Problems with baggage | Lufthansa</t>
@@ -622,7 +622,7 @@
     <t>de/en/baggage</t>
   </si>
   <si>
-    <t>2026-10-21T16:54:59.566Z</t>
+    <t>2026-10-21T22:28:51.748Z</t>
   </si>
   <si>
     <t>Baggage | Lufthansa</t>
@@ -637,7 +637,7 @@
     <t>de/en/bid-upgrade</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:48.493Z</t>
+    <t>2026-10-21T22:30:19.821Z</t>
   </si>
   <si>
     <t>Submit an offer for your upgrade | Lufthansa</t>
@@ -652,7 +652,7 @@
     <t>de/en/boarding</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:47.048Z</t>
+    <t>2026-10-21T22:30:22.222Z</t>
   </si>
   <si>
     <t>Boarding | Lufthansa</t>
@@ -667,7 +667,7 @@
     <t>de/en/business-class-on-short-and-medium-haul</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:06.858Z</t>
+    <t>2026-10-21T22:31:03.113Z</t>
   </si>
   <si>
     <t>Business Class on short and medium-haul routes | Lufthansa</t>
@@ -682,7 +682,7 @@
     <t>de/en/business-class</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:53.691Z</t>
+    <t>2026-10-21T22:31:00.658Z</t>
   </si>
   <si>
     <t>Business Class | Lufthansa</t>
@@ -697,7 +697,7 @@
     <t>de/en/business-services</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:09.743Z</t>
+    <t>2026-10-21T22:31:05.036Z</t>
   </si>
   <si>
     <t>Business Services | Lufthansa</t>
@@ -712,7 +712,7 @@
     <t>de/en/cancellations-and-refunds</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:11.729Z</t>
+    <t>2026-10-21T22:31:08.458Z</t>
   </si>
   <si>
     <t>Cancellation and refund | Lufthansa</t>
@@ -730,7 +730,7 @@
     <t>de/en/carry-on-baggage</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:14.342Z</t>
+    <t>2026-10-21T22:31:10.950Z</t>
   </si>
   <si>
     <t>Carry-on baggage | Lufthansa</t>
@@ -745,7 +745,7 @@
     <t>de/en/cash-and-miles</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:16.728Z</t>
+    <t>2026-10-21T22:31:14.017Z</t>
   </si>
   <si>
     <t>Cash &amp; Miles | Lufthansa</t>
@@ -760,7 +760,7 @@
     <t>de/en/check-in-baggage</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:18.964Z</t>
+    <t>2026-10-21T22:31:16.993Z</t>
   </si>
   <si>
     <t>Baggage drop | Lufthansa</t>
@@ -775,7 +775,7 @@
     <t>de/en/check-in-with-the-family</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:21.159Z</t>
+    <t>2026-10-21T22:31:18.810Z</t>
   </si>
   <si>
     <t>Online check-in with the whole family | Lufthansa</t>
@@ -790,7 +790,7 @@
     <t>de/en/child-restraint-systems</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:23.683Z</t>
+    <t>2026-10-21T22:31:20.992Z</t>
   </si>
   <si>
     <t>Safety for small children on board | Lufthansa</t>
@@ -805,7 +805,7 @@
     <t>de/en/children-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:50.216Z</t>
+    <t>2026-10-21T22:31:23.009Z</t>
   </si>
   <si>
     <t>On board with children and babies | Lufthansa</t>
@@ -820,7 +820,7 @@
     <t>de/en/childrens-menus-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:52.343Z</t>
+    <t>2026-10-21T22:31:28.164Z</t>
   </si>
   <si>
     <t>Children’s menus | Lufthansa</t>
@@ -835,7 +835,7 @@
     <t>de/en/dangerous-dogs</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:26.211Z</t>
+    <t>2026-10-21T22:31:34.059Z</t>
   </si>
   <si>
     <t>Fighting dog breeds and snub-nosed animals | Lufthansa</t>
@@ -850,7 +850,7 @@
     <t>de/en/digital-baggage-services</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:28.253Z</t>
+    <t>2026-10-21T22:31:36.282Z</t>
   </si>
   <si>
     <t>Digital baggage services | Lufthansa</t>
@@ -865,7 +865,7 @@
     <t>de/en/digital-self-services</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:36.360Z</t>
+    <t>2026-10-21T22:29:00.047Z</t>
   </si>
   <si>
     <t>Digital services | Lufthansa</t>
@@ -880,7 +880,7 @@
     <t>de/en/digital-travel-companion</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:30.083Z</t>
+    <t>2026-10-21T22:31:39.166Z</t>
   </si>
   <si>
     <t>Lufthansa app | Lufthansa</t>
@@ -895,7 +895,7 @@
     <t>de/en/doctor-on-board-news</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:46.896Z</t>
+    <t>2026-10-21T22:32:03.500Z</t>
   </si>
   <si>
     <t>Doctor on Board—good to know | Lufthansa</t>
@@ -910,7 +910,7 @@
     <t>de/en/doctor-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:44.039Z</t>
+    <t>2026-10-21T22:31:58.785Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/doctor-on-board</t>
@@ -922,7 +922,7 @@
     <t>de/en/economy-class</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:47.420Z</t>
+    <t>2026-10-21T22:32:21.285Z</t>
   </si>
   <si>
     <t>Economy Class | Lufthansa</t>
@@ -937,7 +937,7 @@
     <t>de/en/electronic-bag-tags</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:49.689Z</t>
+    <t>2026-10-21T22:32:23.940Z</t>
   </si>
   <si>
     <t>Electronic bag tags | Lufthansa</t>
@@ -952,7 +952,7 @@
     <t>de/en/entryprocesses</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:51.447Z</t>
+    <t>2026-10-21T22:32:26.708Z</t>
   </si>
   <si>
     <t>Entry regulations | Lufthansa</t>
@@ -967,7 +967,7 @@
     <t>de/en/europa-tarife-economy-class</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:53.242Z</t>
+    <t>2026-10-21T22:32:28.714Z</t>
   </si>
   <si>
     <t>Our Europe fares | Lufthansa</t>
@@ -982,7 +982,7 @@
     <t>de/en/europcar</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:55.653Z</t>
+    <t>2026-10-21T22:32:31.567Z</t>
   </si>
   <si>
     <t>Europcar | Lufthansa</t>
@@ -997,7 +997,7 @@
     <t>de/en/exclusive-charter</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:57.587Z</t>
+    <t>2026-10-21T22:32:33.293Z</t>
   </si>
   <si>
     <t>Lufthansa Charter | Lufthansa</t>
@@ -1012,7 +1012,7 @@
     <t>de/en/faq-ejournals</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:59.675Z</t>
+    <t>2026-10-21T22:32:35.654Z</t>
   </si>
   <si>
     <t>FAQs about eJournals | Lufthansa</t>
@@ -1048,7 +1048,7 @@
     <t>de/en/fia-valet-service</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:02.056Z</t>
+    <t>2026-10-21T22:32:38.408Z</t>
   </si>
   <si>
     <t>FIA Valet Service | Lufthansa</t>
@@ -1063,7 +1063,7 @@
     <t>de/en/first-class-comfort</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:51.510Z</t>
+    <t>2026-10-21T22:32:43.359Z</t>
   </si>
   <si>
     <t>Comfort on board First Class | Lufthansa</t>
@@ -1081,7 +1081,7 @@
     <t>de/en/first-class-lounges</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:07.253Z</t>
+    <t>2026-10-21T22:32:48.150Z</t>
   </si>
   <si>
     <t>First Class Lounges | Lufthansa</t>
@@ -1096,7 +1096,7 @@
     <t>de/en/first-class-personal-assistant</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:09.619Z</t>
+    <t>2026-10-21T22:32:49.855Z</t>
   </si>
   <si>
     <t>First Class personal assistant service | Lufthansa</t>
@@ -1111,7 +1111,7 @@
     <t>de/en/first-class-terminal</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:11.882Z</t>
+    <t>2026-10-21T22:32:52.460Z</t>
   </si>
   <si>
     <t>First Class Terminal | Lufthansa</t>
@@ -1126,7 +1126,7 @@
     <t>de/en/first-class-valet-parking-service</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:13.849Z</t>
+    <t>2026-10-21T22:32:55.683Z</t>
   </si>
   <si>
     <t>Valet parking service | Lufthansa</t>
@@ -1141,7 +1141,7 @@
     <t>de/en/first-class</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:04.433Z</t>
+    <t>2026-10-21T22:32:40.870Z</t>
   </si>
   <si>
     <t>Lufthansa First Class | Lufthansa</t>
@@ -1156,7 +1156,7 @@
     <t>de/en/fliegen-mit-baby</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:15.560Z</t>
+    <t>2026-10-21T22:32:58.220Z</t>
   </si>
   <si>
     <t>Flying with baby | Lufthansa</t>
@@ -1171,7 +1171,7 @@
     <t>de/en/flight-disruptions</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:17.617Z</t>
+    <t>2026-10-21T22:33:00.710Z</t>
   </si>
   <si>
     <t>Flights delayed and cancelled at short notice | Lufthansa</t>
@@ -1189,7 +1189,7 @@
     <t>de/en/flights</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:40.917Z</t>
+    <t>2026-10-21T22:29:04.966Z</t>
   </si>
   <si>
     <t>Flight offers and destinations worldwide | Lufthansa</t>
@@ -1204,7 +1204,7 @@
     <t>de/en/fly-more-sustainabl</t>
   </si>
   <si>
-    <t>2026-10-21T21:10:20.317Z</t>
+    <t>2026-10-21T22:33:02.743Z</t>
   </si>
   <si>
     <t>Fly more sustainably | Lufthansa</t>
@@ -1219,7 +1219,7 @@
     <t>de/en/flying-with-small-children</t>
   </si>
   <si>
-    <t>2026-10-21T17:01:18.757Z</t>
+    <t>2026-10-21T22:29:44.690Z</t>
   </si>
   <si>
     <t>Flying with small children | Lufthansa</t>
@@ -1234,7 +1234,7 @@
     <t>de/en/flynet</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:46.105Z</t>
+    <t>2026-10-21T22:33:05.112Z</t>
   </si>
   <si>
     <t>FlyNet® on board | Lufthansa</t>
@@ -1249,7 +1249,7 @@
     <t>de/en/fmg-valet-parking-service</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:48.875Z</t>
+    <t>2026-10-21T22:33:07.569Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/fmg-valet-parking-service</t>
@@ -1261,7 +1261,7 @@
     <t>de/en/food-and-beverages</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:43.683Z</t>
+    <t>2026-10-21T22:29:08.014Z</t>
   </si>
   <si>
     <t>Menus on board | Lufthansa</t>
@@ -1288,7 +1288,7 @@
     <t>de/en/free2move</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:51.672Z</t>
+    <t>2026-10-21T22:33:09.325Z</t>
   </si>
   <si>
     <t>Free2move carsharing | Lufthansa</t>
@@ -1303,7 +1303,7 @@
     <t>de/en/freigepaeck-regeln</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:53.913Z</t>
+    <t>2026-10-21T22:33:12.161Z</t>
   </si>
   <si>
     <t>Free baggage rules at Lufthansa | Lufthansa</t>
@@ -1318,7 +1318,7 @@
     <t>de/en/gefaehrliche-gegenstaende</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:57.010Z</t>
+    <t>2026-10-21T22:33:14.892Z</t>
   </si>
   <si>
     <t>Dangerous goods | Lufthansa</t>
@@ -1333,7 +1333,7 @@
     <t>de/en/green-fare</t>
   </si>
   <si>
-    <t>2026-10-21T21:17:59.988Z</t>
+    <t>2026-10-21T22:33:16.852Z</t>
   </si>
   <si>
     <t>Green Fares: More sustainable air travel | Lufthansa</t>
@@ -1348,7 +1348,7 @@
     <t>de/en/group-travel-and-charter</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:04.849Z</t>
+    <t>2026-10-21T22:33:21.847Z</t>
   </si>
   <si>
     <t>Group travel and Lufthansa Charter | Lufthansa</t>
@@ -1363,7 +1363,7 @@
     <t>de/en/group-travel</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:02.306Z</t>
+    <t>2026-10-21T22:33:19.066Z</t>
   </si>
   <si>
     <t>Group travel | Lufthansa</t>
@@ -1378,7 +1378,7 @@
     <t>de/en/hertz</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:07.686Z</t>
+    <t>2026-10-21T22:33:24.343Z</t>
   </si>
   <si>
     <t>Hertz | Lufthansa</t>
@@ -1393,7 +1393,7 @@
     <t>de/en/homepage</t>
   </si>
   <si>
-    <t>2026-10-21T17:01:12.172Z</t>
+    <t>2026-10-21T22:28:36.795Z</t>
   </si>
   <si>
     <t>Book your flight now - travel with Lufthansa to over 200 destinations | Lufthansa</t>
@@ -1408,7 +1408,7 @@
     <t>de/en/hotel-offers</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:10.223Z</t>
+    <t>2026-10-21T22:33:26.676Z</t>
   </si>
   <si>
     <t>Hotel offers | Lufthansa</t>
@@ -1444,7 +1444,7 @@
     <t>de/en/lh-rentalcar</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:12.065Z</t>
+    <t>2026-10-21T22:33:29.136Z</t>
   </si>
   <si>
     <t>Car rental partners | Lufthansa</t>
@@ -1459,7 +1459,7 @@
     <t>de/en/lounge-companions</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:14.309Z</t>
+    <t>2026-10-21T22:33:31.893Z</t>
   </si>
   <si>
     <t>Take your companions into the lounge with you | Lufthansa</t>
@@ -1474,7 +1474,7 @@
     <t>de/en/lounges</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:46.343Z</t>
+    <t>2026-10-21T22:29:12.311Z</t>
   </si>
   <si>
     <t>Lounges | Lufthansa</t>
@@ -1489,7 +1489,7 @@
     <t>de/en/lufthansa-am-flughafen-frankfurt</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:17.122Z</t>
+    <t>2026-10-21T22:33:33.693Z</t>
   </si>
   <si>
     <t>Lufthansa at Frankfurt Airport | Lufthansa</t>
@@ -1504,7 +1504,7 @@
     <t>de/en/lufthansa-at-berlin-airport</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:20.140Z</t>
+    <t>2026-10-21T22:33:36.028Z</t>
   </si>
   <si>
     <t>Lufthansa at Berlin Brandenburg Airport | Lufthansa</t>
@@ -1519,7 +1519,7 @@
     <t>de/en/lufthansa-at-duesseldorf-airport</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:21.964Z</t>
+    <t>2026-10-21T22:33:38.951Z</t>
   </si>
   <si>
     <t>Lufthansa at Dusseldorf Airport | Lufthansa</t>
@@ -1534,7 +1534,7 @@
     <t>de/en/lufthansa-at-vienna-airport</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:24.577Z</t>
+    <t>2026-10-21T22:33:41.420Z</t>
   </si>
   <si>
     <t>Lufthansa at Vienna Airport | Lufthansa</t>
@@ -1549,7 +1549,7 @@
     <t>de/en/lufthansa-at-zuerich-airport</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:26.731Z</t>
+    <t>2026-10-21T22:33:43.859Z</t>
   </si>
   <si>
     <t>Lufthansa at Zurich Airport | Lufthansa</t>
@@ -1564,7 +1564,7 @@
     <t>de/en/lufthansa-aviation-group</t>
   </si>
   <si>
-    <t>2026-10-21T21:18:29.559Z</t>
+    <t>2026-10-21T22:33:45.803Z</t>
   </si>
   <si>
     <t>Lufthansa Aviation Group | Lufthansa</t>
@@ -1573,13 +1573,88 @@
     <t>https://www.lufthansa.com/de/en/lufthansa-aviation-group</t>
   </si>
   <si>
+    <t>de/en/lufthansa-business-class-on-long-haul-routes.report.json</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-business-class-on-long-haul-routes</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:33:48.569Z</t>
+  </si>
+  <si>
+    <t>Business Class on long-haul routes | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/lufthansa-business-class-on-long-haul-routes</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-corporate-customers.report.json</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-corporate-customers</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:33:50.458Z</t>
+  </si>
+  <si>
+    <t>Lufthansa for corporate customers | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/lufthansa-corporate-customers</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-express-bus.report.json</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-express-bus</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:33:54.761Z</t>
+  </si>
+  <si>
+    <t>Lufthansa Express Bus | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/lufthansa-express-bus</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-express-rail.report.json</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-express-rail</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:33:56.987Z</t>
+  </si>
+  <si>
+    <t>Lufthansa Express Rail | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/lufthansa-express-rail</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-express.report.json</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-express</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:33:52.450Z</t>
+  </si>
+  <si>
+    <t>Airport arrival and departure – travel seamlessly | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/lufthansa-express</t>
+  </si>
+  <si>
     <t>de/en/lufthansa-first-class-entertainment.report.json</t>
   </si>
   <si>
     <t>de/en/lufthansa-first-class-entertainment</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:53.390Z</t>
+    <t>2026-10-21T22:34:00.424Z</t>
   </si>
   <si>
     <t>Entertainment world | Lufthansa</t>
@@ -1588,13 +1663,58 @@
     <t>https://www.lufthansa.com/de/en/lufthansa-first-class-entertainment</t>
   </si>
   <si>
+    <t>de/en/lufthansa-group-star-alliance-and-partner-airlines.report.json</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-group-star-alliance-and-partner-airlines</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:34:05.613Z</t>
+  </si>
+  <si>
+    <t>Lufthansa Group, Star Alliance and partner airlines | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/lufthansa-group-star-alliance-and-partner-airlines</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-guide-service.report.json</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-guide-service</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:34:07.304Z</t>
+  </si>
+  <si>
+    <t>Lufthansa Guide Service Munich | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/lufthansa-guide-service</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-terminal-muenchen.report.json</t>
+  </si>
+  <si>
+    <t>de/en/lufthansa-terminal-muenchen</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:34:10.267Z</t>
+  </si>
+  <si>
+    <t>Lufthansa at Munich Airport | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/lufthansa-terminal-muenchen</t>
+  </si>
+  <si>
     <t>de/en/lufthansa-travel-classes.report.json</t>
   </si>
   <si>
     <t>de/en/lufthansa-travel-classes</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:49.011Z</t>
+    <t>2026-10-21T22:29:15.410Z</t>
   </si>
   <si>
     <t>Our travel classes | Lufthansa</t>
@@ -1603,13 +1723,58 @@
     <t>https://www.lufthansa.com/de/en/lufthansa-travel-classes</t>
   </si>
   <si>
+    <t>de/en/medikamenten-transport.report.json</t>
+  </si>
+  <si>
+    <t>de/en/medikamenten-transport</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:34:13.158Z</t>
+  </si>
+  <si>
+    <t>Always at the right temperature | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/medikamenten-transport</t>
+  </si>
+  <si>
+    <t>de/en/meetings-and-events-delegates.report.json</t>
+  </si>
+  <si>
+    <t>de/en/meetings-and-events-delegates</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:34:15.050Z</t>
+  </si>
+  <si>
+    <t>Meetings &amp; Events: Information for organisers | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/meetings-and-events-delegates</t>
+  </si>
+  <si>
+    <t>de/en/meetings-and-events-organisers.report.json</t>
+  </si>
+  <si>
+    <t>de/en/meetings-and-events-organisers</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:34:16.965Z</t>
+  </si>
+  <si>
+    <t>Meeting &amp; Events: Information for organisers | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/meetings-and-events-organisers</t>
+  </si>
+  <si>
     <t>de/en/meetings-and-events.report.json</t>
   </si>
   <si>
     <t>de/en/meetings-and-events</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:51.766Z</t>
+    <t>2026-10-21T22:29:17.390Z</t>
   </si>
   <si>
     <t>Lufthansa Group Meetings &amp; Events | Lufthansa</t>
@@ -1624,7 +1789,7 @@
     <t>de/en/menus-on-long-haul-flights</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:56.509Z</t>
+    <t>2026-10-21T22:34:18.943Z</t>
   </si>
   <si>
     <t>Menus on long-haul flights | Lufthansa</t>
@@ -1639,7 +1804,7 @@
     <t>de/en/menus-travel-classes</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:58.485Z</t>
+    <t>2026-10-21T22:34:23.793Z</t>
   </si>
   <si>
     <t>Menus in our travel classes | Lufthansa</t>
@@ -1654,7 +1819,7 @@
     <t>de/en/miles-and-more</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:53.850Z</t>
+    <t>2026-10-21T22:29:19.875Z</t>
   </si>
   <si>
     <t>Miles &amp; More – Our frequent flyer programme | Lufthansa</t>
@@ -1663,6 +1828,21 @@
     <t>https://www.lufthansa.com/de/en/miles-and-more</t>
   </si>
   <si>
+    <t>de/en/mobility-partner-program-healthcare.report.json</t>
+  </si>
+  <si>
+    <t>de/en/mobility-partner-program-healthcare</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:34:27.573Z</t>
+  </si>
+  <si>
+    <t>Lufthansa Global Healthcare and Medical Services | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/mobility-partner-program-healthcare</t>
+  </si>
+  <si>
     <t>de/en/nav.report.json</t>
   </si>
   <si>
@@ -1681,12 +1861,27 @@
     <t>de/en/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-21T20:04:00.742Z</t>
+    <t>2026-10-21T22:34:30.374Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/onboard-delights</t>
   </si>
   <si>
+    <t>de/en/online-check-in-info.report.json</t>
+  </si>
+  <si>
+    <t>de/en/online-check-in-info</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:34:34.662Z</t>
+  </si>
+  <si>
+    <t>Online check-in information | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/online-check-in-info</t>
+  </si>
+  <si>
     <t>de/en/online-check-in.report.json</t>
   </si>
   <si>
@@ -1714,7 +1909,7 @@
     <t>de/en/overview-flights</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:55.609Z</t>
+    <t>2026-10-21T22:29:22.394Z</t>
   </si>
   <si>
     <t>Flights – your journey starts here | Lufthansa</t>
@@ -1732,7 +1927,7 @@
     <t>de/en/overview-manage</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:57.674Z</t>
+    <t>2026-10-21T22:29:24.956Z</t>
   </si>
   <si>
     <t>Manage your bookings | Lufthansa</t>
@@ -1747,7 +1942,7 @@
     <t>de/en/overview-special-request</t>
   </si>
   <si>
-    <t>2026-10-21T20:02:59.788Z</t>
+    <t>2026-10-21T22:29:26.725Z</t>
   </si>
   <si>
     <t>Special requests | Lufthansa</t>
@@ -1762,7 +1957,7 @@
     <t>de/en/overview-travel-information</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:02.269Z</t>
+    <t>2026-10-21T22:29:29.135Z</t>
   </si>
   <si>
     <t>Travel information – what you need to know | Lufthansa</t>
@@ -1771,13 +1966,58 @@
     <t>https://www.lufthansa.com/de/en/overview-travel-information</t>
   </si>
   <si>
+    <t>de/en/partner.report.json</t>
+  </si>
+  <si>
+    <t>de/en/partner</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:34:37.659Z</t>
+  </si>
+  <si>
+    <t>Partners | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/partner</t>
+  </si>
+  <si>
+    <t>de/en/passenger-receipt-90.report.json</t>
+  </si>
+  <si>
+    <t>de/en/passenger-receipt-90</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:34:39.755Z</t>
+  </si>
+  <si>
+    <t>Passenger receipt | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/passenger-receipt-90</t>
+  </si>
+  <si>
+    <t>de/en/passengers-using-wheelchairs.report.json</t>
+  </si>
+  <si>
+    <t>de/en/passengers-using-wheelchairs</t>
+  </si>
+  <si>
+    <t>2026-10-21T22:34:42.001Z</t>
+  </si>
+  <si>
+    <t>Passengers requiring wheelchairs | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/passengers-using-wheelchairs</t>
+  </si>
+  <si>
     <t>de/en/services-at-the-airport.report.json</t>
   </si>
   <si>
     <t>de/en/services-at-the-airport</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:04.410Z</t>
+    <t>2026-10-21T22:29:32.371Z</t>
   </si>
   <si>
     <t>Services at the airport | Lufthansa</t>
@@ -1792,7 +2032,7 @@
     <t>de/en/services-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:06.364Z</t>
+    <t>2026-10-21T22:29:34.558Z</t>
   </si>
   <si>
     <t>Services on board | Lufthansa</t>
@@ -1807,7 +2047,7 @@
     <t>de/en/special-needs</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:09.544Z</t>
+    <t>2026-10-21T22:29:39.318Z</t>
   </si>
   <si>
     <t>Register your assistance requirements online | Lufthansa</t>
@@ -1843,7 +2083,7 @@
     <t>de/en/unterhaltung-an-bord</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:55.435Z</t>
+    <t>2026-10-21T22:34:44.190Z</t>
   </si>
   <si>
     <t>Entertainment on board | Lufthansa</t>
@@ -1870,7 +2110,7 @@
     <t>gb/en/homepage</t>
   </si>
   <si>
-    <t>2026-10-21T18:23:07.976Z</t>
+    <t>2026-10-21T22:28:46.096Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/homepage</t>
@@ -1948,7 +2188,7 @@
     <t>de/de/during-your-trip/lhg-wifi</t>
   </si>
   <si>
-    <t>2026-10-21T20:18:04.970Z</t>
+    <t>2026-10-21T22:32:18.873Z</t>
   </si>
   <si>
     <t>Lufthansa Group Wi-Fi | Lufthansa</t>
@@ -1975,10 +2215,7 @@
     <t>de/en/book-and-manage/pax-receipt</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:40.390Z</t>
-  </si>
-  <si>
-    <t>Passenger receipt | Lufthansa</t>
+    <t>2026-10-21T22:30:46.923Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/book-and-manage/pax-receipt</t>
@@ -1990,7 +2227,7 @@
     <t>de/en/book-and-manage/rebook</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:46.117Z</t>
+    <t>2026-10-21T22:30:52.704Z</t>
   </si>
   <si>
     <t>Flight Rebooking | Lufthansa</t>
@@ -2005,7 +2242,7 @@
     <t>de/en/discover-lufthansa/flightreservation-priceguarantee</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:42.460Z</t>
+    <t>2026-10-21T22:31:51.511Z</t>
   </si>
   <si>
     <t>Reservation with price guarantee | Lufthansa</t>
@@ -2020,7 +2257,7 @@
     <t>de/en/discover-lufthansa/miles-and-more-credit-card</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:46.716Z</t>
+    <t>2026-10-21T22:31:56.206Z</t>
   </si>
   <si>
     <t>Miles &amp; More Credit Card | Lufthansa</t>
@@ -2047,7 +2284,7 @@
     <t>de/en/during-your-trip/internet-overview</t>
   </si>
   <si>
-    <t>2026-10-21T21:09:44.425Z</t>
+    <t>2026-10-21T22:32:14.040Z</t>
   </si>
   <si>
     <t>Internet | Lufthansa</t>
@@ -2062,7 +2299,7 @@
     <t>de/en/during-your-trip/lhg-wifi</t>
   </si>
   <si>
-    <t>2026-10-21T20:17:48.988Z</t>
+    <t>2026-10-21T22:32:16.809Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/during-your-trip/lhg-wifi</t>
@@ -2170,7 +2407,7 @@
     <t>de/en/book-and-manage/additional-services/get-your-guide</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:49.789Z</t>
+    <t>2026-10-21T22:30:23.858Z</t>
   </si>
   <si>
     <t>Unforgettable travel experiences—GetYourGuide | Lufthansa</t>
@@ -2185,7 +2422,7 @@
     <t>de/en/book-and-manage/additional-services/travel-insurances</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:51.782Z</t>
+    <t>2026-10-21T22:30:26.033Z</t>
   </si>
   <si>
     <t>Travel Care | Lufthansa</t>
@@ -2200,7 +2437,7 @@
     <t>de/en/book-and-manage/digital-self-services/airline-apps</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:54.185Z</t>
+    <t>2026-10-21T22:30:27.759Z</t>
   </si>
   <si>
     <t>Simply travel smarter | Lufthansa</t>
@@ -2215,7 +2452,7 @@
     <t>de/en/book-and-manage/flights/air-baltic</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:56.300Z</t>
+    <t>2026-10-21T22:30:30.294Z</t>
   </si>
   <si>
     <t>Your Lufthansa flight with airBaltic | Lufthansa</t>
@@ -2230,7 +2467,7 @@
     <t>de/en/book-and-manage/flights/ana</t>
   </si>
   <si>
-    <t>2026-10-21T20:41:58.144Z</t>
+    <t>2026-10-21T22:30:32.649Z</t>
   </si>
   <si>
     <t>ANA | Lufthansa</t>
@@ -2248,7 +2485,7 @@
     <t>de/en/book-and-manage/flights/giftvoucher</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:31.410Z</t>
+    <t>2026-10-21T22:30:37.799Z</t>
   </si>
   <si>
     <t>Buy a Lufthansa Gift Card &amp; give a flight as a gift | Lufthansa</t>
@@ -2263,7 +2500,7 @@
     <t>de/en/book-and-manage/flights/helvetic</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:33.522Z</t>
+    <t>2026-10-21T22:30:40.563Z</t>
   </si>
   <si>
     <t>Helvetic | Lufthansa</t>
@@ -2278,7 +2515,7 @@
     <t>de/en/book-and-manage/flights/lufthansa-voucher</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:35.591Z</t>
+    <t>2026-10-21T22:30:43.081Z</t>
   </si>
   <si>
     <t>Terms of use for the purchase of Gift Vouchers | Lufthansa</t>
@@ -2293,7 +2530,7 @@
     <t>de/en/book-and-manage/flights/wetlease-hub</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:37.711Z</t>
+    <t>2026-10-21T22:30:44.869Z</t>
   </si>
   <si>
     <t>Wet lease flights | Lufthansa</t>
@@ -2308,7 +2545,7 @@
     <t>de/en/book-and-manage/pax-receipt/invoices-different-countries</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:43.197Z</t>
+    <t>2026-10-21T22:30:49.989Z</t>
   </si>
   <si>
     <t>Invoices for different countries | Lufthansa</t>
@@ -2323,7 +2560,7 @@
     <t>de/en/book-and-manage/rebook/involuntary-rebooking</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:49.236Z</t>
+    <t>2026-10-21T22:30:55.679Z</t>
   </si>
   <si>
     <t>Flight cancellation | Lufthansa</t>
@@ -2338,7 +2575,7 @@
     <t>de/en/book-and-manage/rebook/voluntary-rebooking</t>
   </si>
   <si>
-    <t>2026-10-21T20:48:51.326Z</t>
+    <t>2026-10-21T22:30:57.574Z</t>
   </si>
   <si>
     <t>Change flight | Lufthansa</t>
@@ -2353,7 +2590,7 @@
     <t>de/en/discover-lufthansa/carbon-offsetting/climate-protection-projects</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:33.023Z</t>
+    <t>2026-10-21T22:31:42.262Z</t>
   </si>
   <si>
     <t>Climate protection projects | Lufthansa</t>
@@ -2368,7 +2605,7 @@
     <t>de/en/discover-lufthansa/carbon-offsetting/environmental-cost-surcharge</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:35.658Z</t>
+    <t>2026-10-21T22:31:44.526Z</t>
   </si>
   <si>
     <t>Environmental Cost Surcharge | Lufthansa</t>
@@ -2383,7 +2620,7 @@
     <t>de/en/discover-lufthansa/carbon-offsetting/faq-saf</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:37.765Z</t>
+    <t>2026-10-21T22:31:47.219Z</t>
   </si>
   <si>
     <t>FAQs Sustainable Aviation Fuel | Lufthansa</t>
@@ -2398,7 +2635,7 @@
     <t>de/en/discover-lufthansa/carbon-offsetting/saf</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:40.111Z</t>
+    <t>2026-10-21T22:31:49.735Z</t>
   </si>
   <si>
     <t>Why support the use of Sustainable Aviation Fuel? | Lufthansa</t>
@@ -2413,7 +2650,7 @@
     <t>de/en/discover-lufthansa/lufthansa-group-airlines/ita-airways</t>
   </si>
   <si>
-    <t>2026-10-21T21:00:44.302Z</t>
+    <t>2026-10-21T22:31:53.994Z</t>
   </si>
   <si>
     <t>ITA Airways | Lufthansa</t>
@@ -2431,7 +2668,7 @@
     <t>de/en/book-and-manage/flights/ana/faq</t>
   </si>
   <si>
-    <t>2026-10-21T20:42:00.121Z</t>
+    <t>2026-10-21T22:30:35.269Z</t>
   </si>
   <si>
     <t>FAQs on travel with Lufthansa and ANA | Lufthansa</t>
@@ -2446,7 +2683,7 @@
     <t>de/en/during-your-trip/food-and-beverages/onboard-delights/faq</t>
   </si>
   <si>
-    <t>2026-10-21T20:03:54.738Z</t>
+    <t>2026-10-21T22:32:08.618Z</t>
   </si>
   <si>
     <t>FAQs | Lufthansa</t>
@@ -2880,7 +3117,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I159"/>
+  <dimension ref="A1:I175"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
@@ -5796,7 +6033,7 @@
         <v>525</v>
       </c>
       <c r="B101" t="s">
-        <v>103</v>
+        <v>36</v>
       </c>
       <c r="C101" t="s">
         <v>10</v>
@@ -5808,7 +6045,7 @@
         <v>13</v>
       </c>
       <c r="F101" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="G101" t="s">
         <v>527</v>
@@ -5825,7 +6062,7 @@
         <v>530</v>
       </c>
       <c r="B102" t="s">
-        <v>36</v>
+        <v>237</v>
       </c>
       <c r="C102" t="s">
         <v>10</v>
@@ -5837,7 +6074,7 @@
         <v>13</v>
       </c>
       <c r="F102" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="G102" t="s">
         <v>532</v>
@@ -5854,7 +6091,7 @@
         <v>535</v>
       </c>
       <c r="B103" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="C103" t="s">
         <v>10</v>
@@ -5924,7 +6161,7 @@
         <v>13</v>
       </c>
       <c r="F105" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="G105" t="s">
         <v>547</v>
@@ -5941,10 +6178,10 @@
         <v>550</v>
       </c>
       <c r="B106" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C106" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="D106" t="s">
         <v>551</v>
@@ -5953,30 +6190,30 @@
         <v>13</v>
       </c>
       <c r="F106" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G106" t="s">
         <v>552</v>
       </c>
       <c r="H106" t="s">
-        <v>10</v>
+        <v>553</v>
       </c>
       <c r="I106" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B107" t="s">
-        <v>90</v>
+        <v>36</v>
       </c>
       <c r="C107" t="s">
         <v>10</v>
       </c>
       <c r="D107" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="E107" t="s">
         <v>13</v>
@@ -5985,33 +6222,33 @@
         <v>31</v>
       </c>
       <c r="G107" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="H107" t="s">
-        <v>93</v>
+        <v>558</v>
       </c>
       <c r="I107" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="B108" t="s">
-        <v>559</v>
+        <v>36</v>
       </c>
       <c r="C108" t="s">
         <v>10</v>
       </c>
       <c r="D108" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="E108" t="s">
         <v>13</v>
       </c>
       <c r="F108" t="s">
-        <v>561</v>
+        <v>31</v>
       </c>
       <c r="G108" t="s">
         <v>562</v>
@@ -6028,7 +6265,7 @@
         <v>565</v>
       </c>
       <c r="B109" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="C109" t="s">
         <v>10</v>
@@ -6057,62 +6294,62 @@
         <v>570</v>
       </c>
       <c r="B110" t="s">
+        <v>36</v>
+      </c>
+      <c r="C110" t="s">
+        <v>10</v>
+      </c>
+      <c r="D110" t="s">
         <v>571</v>
       </c>
-      <c r="C110" t="s">
-        <v>10</v>
-      </c>
-      <c r="D110" t="s">
+      <c r="E110" t="s">
+        <v>13</v>
+      </c>
+      <c r="F110" t="s">
+        <v>31</v>
+      </c>
+      <c r="G110" t="s">
         <v>572</v>
       </c>
-      <c r="E110" t="s">
-        <v>13</v>
-      </c>
-      <c r="F110" t="s">
-        <v>98</v>
-      </c>
-      <c r="G110" t="s">
+      <c r="H110" t="s">
         <v>573</v>
       </c>
-      <c r="H110" t="s">
+      <c r="I110" t="s">
         <v>574</v>
-      </c>
-      <c r="I110" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
+        <v>575</v>
+      </c>
+      <c r="B111" t="s">
+        <v>36</v>
+      </c>
+      <c r="C111" t="s">
+        <v>10</v>
+      </c>
+      <c r="D111" t="s">
         <v>576</v>
       </c>
-      <c r="B111" t="s">
-        <v>96</v>
-      </c>
-      <c r="C111" t="s">
-        <v>10</v>
-      </c>
-      <c r="D111" t="s">
+      <c r="E111" t="s">
+        <v>13</v>
+      </c>
+      <c r="F111" t="s">
+        <v>31</v>
+      </c>
+      <c r="G111" t="s">
         <v>577</v>
       </c>
-      <c r="E111" t="s">
-        <v>13</v>
-      </c>
-      <c r="F111" t="s">
-        <v>98</v>
-      </c>
-      <c r="G111" t="s">
+      <c r="H111" t="s">
         <v>578</v>
       </c>
-      <c r="H111" t="s">
+      <c r="I111" t="s">
         <v>579</v>
-      </c>
-      <c r="I111" t="s">
-        <v>580</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="B112" t="s">
         <v>36</v>
@@ -6121,27 +6358,27 @@
         <v>10</v>
       </c>
       <c r="D112" t="s">
+        <v>581</v>
+      </c>
+      <c r="E112" t="s">
+        <v>13</v>
+      </c>
+      <c r="F112" t="s">
+        <v>31</v>
+      </c>
+      <c r="G112" t="s">
         <v>582</v>
       </c>
-      <c r="E112" t="s">
-        <v>13</v>
-      </c>
-      <c r="F112" t="s">
-        <v>98</v>
-      </c>
-      <c r="G112" t="s">
+      <c r="H112" t="s">
         <v>583</v>
       </c>
-      <c r="H112" t="s">
+      <c r="I112" t="s">
         <v>584</v>
-      </c>
-      <c r="I112" t="s">
-        <v>585</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
       <c r="B113" t="s">
         <v>36</v>
@@ -6150,7 +6387,7 @@
         <v>10</v>
       </c>
       <c r="D113" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="E113" t="s">
         <v>13</v>
@@ -6159,47 +6396,47 @@
         <v>98</v>
       </c>
       <c r="G113" t="s">
+        <v>587</v>
+      </c>
+      <c r="H113" t="s">
         <v>588</v>
       </c>
-      <c r="H113" t="s">
+      <c r="I113" t="s">
         <v>589</v>
-      </c>
-      <c r="I113" t="s">
-        <v>590</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
+        <v>590</v>
+      </c>
+      <c r="B114" t="s">
+        <v>36</v>
+      </c>
+      <c r="C114" t="s">
+        <v>10</v>
+      </c>
+      <c r="D114" t="s">
         <v>591</v>
       </c>
-      <c r="B114" t="s">
-        <v>96</v>
-      </c>
-      <c r="C114" t="s">
-        <v>10</v>
-      </c>
-      <c r="D114" t="s">
+      <c r="E114" t="s">
+        <v>13</v>
+      </c>
+      <c r="F114" t="s">
+        <v>31</v>
+      </c>
+      <c r="G114" t="s">
         <v>592</v>
       </c>
-      <c r="E114" t="s">
-        <v>13</v>
-      </c>
-      <c r="F114" t="s">
-        <v>98</v>
-      </c>
-      <c r="G114" t="s">
+      <c r="H114" t="s">
         <v>593</v>
       </c>
-      <c r="H114" t="s">
+      <c r="I114" t="s">
         <v>594</v>
-      </c>
-      <c r="I114" t="s">
-        <v>595</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="B115" t="s">
         <v>36</v>
@@ -6208,56 +6445,56 @@
         <v>10</v>
       </c>
       <c r="D115" t="s">
+        <v>596</v>
+      </c>
+      <c r="E115" t="s">
+        <v>13</v>
+      </c>
+      <c r="F115" t="s">
+        <v>31</v>
+      </c>
+      <c r="G115" t="s">
         <v>597</v>
       </c>
-      <c r="E115" t="s">
-        <v>13</v>
-      </c>
-      <c r="F115" t="s">
-        <v>98</v>
-      </c>
-      <c r="G115" t="s">
+      <c r="H115" t="s">
         <v>598</v>
       </c>
-      <c r="H115" t="s">
+      <c r="I115" t="s">
         <v>599</v>
-      </c>
-      <c r="I115" t="s">
-        <v>600</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
+        <v>600</v>
+      </c>
+      <c r="B116" t="s">
+        <v>36</v>
+      </c>
+      <c r="C116" t="s">
+        <v>10</v>
+      </c>
+      <c r="D116" t="s">
         <v>601</v>
       </c>
-      <c r="B116" t="s">
+      <c r="E116" t="s">
+        <v>13</v>
+      </c>
+      <c r="F116" t="s">
+        <v>98</v>
+      </c>
+      <c r="G116" t="s">
         <v>602</v>
       </c>
-      <c r="C116" t="s">
-        <v>10</v>
-      </c>
-      <c r="D116" t="s">
+      <c r="H116" t="s">
         <v>603</v>
       </c>
-      <c r="E116" t="s">
-        <v>13</v>
-      </c>
-      <c r="F116" t="s">
+      <c r="I116" t="s">
         <v>604</v>
-      </c>
-      <c r="G116" t="s">
-        <v>605</v>
-      </c>
-      <c r="H116" t="s">
-        <v>606</v>
-      </c>
-      <c r="I116" t="s">
-        <v>607</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>608</v>
+        <v>605</v>
       </c>
       <c r="B117" t="s">
         <v>36</v>
@@ -6266,36 +6503,36 @@
         <v>10</v>
       </c>
       <c r="D117" t="s">
+        <v>606</v>
+      </c>
+      <c r="E117" t="s">
+        <v>13</v>
+      </c>
+      <c r="F117" t="s">
+        <v>31</v>
+      </c>
+      <c r="G117" t="s">
+        <v>607</v>
+      </c>
+      <c r="H117" t="s">
+        <v>608</v>
+      </c>
+      <c r="I117" t="s">
         <v>609</v>
-      </c>
-      <c r="E117" t="s">
-        <v>13</v>
-      </c>
-      <c r="F117" t="s">
-        <v>31</v>
-      </c>
-      <c r="G117" t="s">
-        <v>610</v>
-      </c>
-      <c r="H117" t="s">
-        <v>611</v>
-      </c>
-      <c r="I117" t="s">
-        <v>612</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>613</v>
+        <v>610</v>
       </c>
       <c r="B118" t="s">
         <v>10</v>
       </c>
       <c r="C118" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D118" t="s">
-        <v>614</v>
+        <v>611</v>
       </c>
       <c r="E118" t="s">
         <v>13</v>
@@ -6304,221 +6541,221 @@
         <v>14</v>
       </c>
       <c r="G118" t="s">
-        <v>615</v>
+        <v>612</v>
       </c>
       <c r="H118" t="s">
         <v>10</v>
       </c>
       <c r="I118" t="s">
-        <v>616</v>
+        <v>613</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
+        <v>614</v>
+      </c>
+      <c r="B119" t="s">
+        <v>90</v>
+      </c>
+      <c r="C119" t="s">
+        <v>10</v>
+      </c>
+      <c r="D119" t="s">
+        <v>615</v>
+      </c>
+      <c r="E119" t="s">
+        <v>13</v>
+      </c>
+      <c r="F119" t="s">
+        <v>31</v>
+      </c>
+      <c r="G119" t="s">
+        <v>616</v>
+      </c>
+      <c r="H119" t="s">
+        <v>93</v>
+      </c>
+      <c r="I119" t="s">
         <v>617</v>
-      </c>
-      <c r="B119" t="s">
-        <v>18</v>
-      </c>
-      <c r="C119" t="s">
-        <v>10</v>
-      </c>
-      <c r="D119" t="s">
-        <v>618</v>
-      </c>
-      <c r="E119" t="s">
-        <v>13</v>
-      </c>
-      <c r="F119" t="s">
-        <v>20</v>
-      </c>
-      <c r="G119" t="s">
-        <v>619</v>
-      </c>
-      <c r="H119" t="s">
-        <v>461</v>
-      </c>
-      <c r="I119" t="s">
-        <v>620</v>
       </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
+        <v>618</v>
+      </c>
+      <c r="B120" t="s">
+        <v>36</v>
+      </c>
+      <c r="C120" t="s">
+        <v>10</v>
+      </c>
+      <c r="D120" t="s">
+        <v>619</v>
+      </c>
+      <c r="E120" t="s">
+        <v>13</v>
+      </c>
+      <c r="F120" t="s">
+        <v>31</v>
+      </c>
+      <c r="G120" t="s">
+        <v>620</v>
+      </c>
+      <c r="H120" t="s">
         <v>621</v>
       </c>
-      <c r="B120" t="s">
-        <v>10</v>
-      </c>
-      <c r="C120" t="s">
-        <v>14</v>
-      </c>
-      <c r="D120" t="s">
+      <c r="I120" t="s">
         <v>622</v>
-      </c>
-      <c r="E120" t="s">
-        <v>13</v>
-      </c>
-      <c r="F120" t="s">
-        <v>14</v>
-      </c>
-      <c r="G120" t="s">
-        <v>623</v>
-      </c>
-      <c r="H120" t="s">
-        <v>10</v>
-      </c>
-      <c r="I120" t="s">
-        <v>624</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
+        <v>623</v>
+      </c>
+      <c r="B121" t="s">
+        <v>624</v>
+      </c>
+      <c r="C121" t="s">
+        <v>10</v>
+      </c>
+      <c r="D121" t="s">
         <v>625</v>
       </c>
-      <c r="B121" t="s">
+      <c r="E121" t="s">
+        <v>13</v>
+      </c>
+      <c r="F121" t="s">
         <v>626</v>
       </c>
-      <c r="C121" t="s">
-        <v>10</v>
-      </c>
-      <c r="D121" t="s">
+      <c r="G121" t="s">
         <v>627</v>
       </c>
-      <c r="E121" t="s">
-        <v>13</v>
-      </c>
-      <c r="F121" t="s">
+      <c r="H121" t="s">
         <v>628</v>
       </c>
-      <c r="G121" t="s">
+      <c r="I121" t="s">
         <v>629</v>
-      </c>
-      <c r="H121" t="s">
-        <v>630</v>
-      </c>
-      <c r="I121" t="s">
-        <v>631</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
+        <v>630</v>
+      </c>
+      <c r="B122" t="s">
+        <v>96</v>
+      </c>
+      <c r="C122" t="s">
+        <v>10</v>
+      </c>
+      <c r="D122" t="s">
+        <v>631</v>
+      </c>
+      <c r="E122" t="s">
+        <v>13</v>
+      </c>
+      <c r="F122" t="s">
+        <v>98</v>
+      </c>
+      <c r="G122" t="s">
         <v>632</v>
       </c>
-      <c r="B122" t="s">
-        <v>10</v>
-      </c>
-      <c r="C122" t="s">
+      <c r="H122" t="s">
         <v>633</v>
       </c>
-      <c r="D122" t="s">
+      <c r="I122" t="s">
         <v>634</v>
-      </c>
-      <c r="E122" t="s">
-        <v>13</v>
-      </c>
-      <c r="F122" t="s">
-        <v>14</v>
-      </c>
-      <c r="G122" t="s">
-        <v>635</v>
-      </c>
-      <c r="H122" t="s">
-        <v>10</v>
-      </c>
-      <c r="I122" t="s">
-        <v>636</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
+        <v>635</v>
+      </c>
+      <c r="B123" t="s">
+        <v>636</v>
+      </c>
+      <c r="C123" t="s">
+        <v>10</v>
+      </c>
+      <c r="D123" t="s">
         <v>637</v>
       </c>
-      <c r="B123" t="s">
+      <c r="E123" t="s">
+        <v>13</v>
+      </c>
+      <c r="F123" t="s">
+        <v>98</v>
+      </c>
+      <c r="G123" t="s">
         <v>638</v>
       </c>
-      <c r="C123" t="s">
-        <v>10</v>
-      </c>
-      <c r="D123" t="s">
+      <c r="H123" t="s">
         <v>639</v>
       </c>
-      <c r="E123" t="s">
-        <v>13</v>
-      </c>
-      <c r="F123" t="s">
-        <v>116</v>
-      </c>
-      <c r="G123" t="s">
+      <c r="I123" t="s">
         <v>640</v>
-      </c>
-      <c r="H123" t="s">
-        <v>641</v>
-      </c>
-      <c r="I123" t="s">
-        <v>642</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
+        <v>641</v>
+      </c>
+      <c r="B124" t="s">
+        <v>96</v>
+      </c>
+      <c r="C124" t="s">
+        <v>10</v>
+      </c>
+      <c r="D124" t="s">
+        <v>642</v>
+      </c>
+      <c r="E124" t="s">
+        <v>13</v>
+      </c>
+      <c r="F124" t="s">
+        <v>98</v>
+      </c>
+      <c r="G124" t="s">
         <v>643</v>
       </c>
-      <c r="B124" t="s">
-        <v>84</v>
-      </c>
-      <c r="C124" t="s">
-        <v>10</v>
-      </c>
-      <c r="D124" t="s">
+      <c r="H124" t="s">
         <v>644</v>
       </c>
-      <c r="E124" t="s">
-        <v>13</v>
-      </c>
-      <c r="F124" t="s">
-        <v>31</v>
-      </c>
-      <c r="G124" t="s">
+      <c r="I124" t="s">
         <v>645</v>
-      </c>
-      <c r="H124" t="s">
-        <v>646</v>
-      </c>
-      <c r="I124" t="s">
-        <v>647</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
+        <v>646</v>
+      </c>
+      <c r="B125" t="s">
+        <v>36</v>
+      </c>
+      <c r="C125" t="s">
+        <v>10</v>
+      </c>
+      <c r="D125" t="s">
+        <v>647</v>
+      </c>
+      <c r="E125" t="s">
+        <v>13</v>
+      </c>
+      <c r="F125" t="s">
+        <v>98</v>
+      </c>
+      <c r="G125" t="s">
         <v>648</v>
       </c>
-      <c r="B125" t="s">
-        <v>10</v>
-      </c>
-      <c r="C125" t="s">
-        <v>633</v>
-      </c>
-      <c r="D125" t="s">
+      <c r="H125" t="s">
         <v>649</v>
       </c>
-      <c r="E125" t="s">
-        <v>13</v>
-      </c>
-      <c r="F125" t="s">
-        <v>14</v>
-      </c>
-      <c r="G125" t="s">
+      <c r="I125" t="s">
         <v>650</v>
-      </c>
-      <c r="H125" t="s">
-        <v>10</v>
-      </c>
-      <c r="I125" t="s">
-        <v>651</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>652</v>
+        <v>651</v>
       </c>
       <c r="B126" t="s">
         <v>36</v>
@@ -6527,27 +6764,27 @@
         <v>10</v>
       </c>
       <c r="D126" t="s">
+        <v>652</v>
+      </c>
+      <c r="E126" t="s">
+        <v>13</v>
+      </c>
+      <c r="F126" t="s">
+        <v>31</v>
+      </c>
+      <c r="G126" t="s">
         <v>653</v>
       </c>
-      <c r="E126" t="s">
-        <v>13</v>
-      </c>
-      <c r="F126" t="s">
-        <v>31</v>
-      </c>
-      <c r="G126" t="s">
+      <c r="H126" t="s">
         <v>654</v>
       </c>
-      <c r="H126" t="s">
+      <c r="I126" t="s">
         <v>655</v>
-      </c>
-      <c r="I126" t="s">
-        <v>656</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="B127" t="s">
         <v>36</v>
@@ -6556,106 +6793,106 @@
         <v>10</v>
       </c>
       <c r="D127" t="s">
+        <v>657</v>
+      </c>
+      <c r="E127" t="s">
+        <v>13</v>
+      </c>
+      <c r="F127" t="s">
+        <v>31</v>
+      </c>
+      <c r="G127" t="s">
         <v>658</v>
       </c>
-      <c r="E127" t="s">
-        <v>13</v>
-      </c>
-      <c r="F127" t="s">
-        <v>31</v>
-      </c>
-      <c r="G127" t="s">
+      <c r="H127" t="s">
         <v>659</v>
       </c>
-      <c r="H127" t="s">
+      <c r="I127" t="s">
         <v>660</v>
-      </c>
-      <c r="I127" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
+        <v>661</v>
+      </c>
+      <c r="B128" t="s">
+        <v>237</v>
+      </c>
+      <c r="C128" t="s">
+        <v>10</v>
+      </c>
+      <c r="D128" t="s">
         <v>662</v>
       </c>
-      <c r="B128" t="s">
-        <v>84</v>
-      </c>
-      <c r="C128" t="s">
-        <v>10</v>
-      </c>
-      <c r="D128" t="s">
+      <c r="E128" t="s">
+        <v>13</v>
+      </c>
+      <c r="F128" t="s">
+        <v>31</v>
+      </c>
+      <c r="G128" t="s">
         <v>663</v>
       </c>
-      <c r="E128" t="s">
-        <v>13</v>
-      </c>
-      <c r="F128" t="s">
-        <v>31</v>
-      </c>
-      <c r="G128" t="s">
+      <c r="H128" t="s">
         <v>664</v>
       </c>
-      <c r="H128" t="s">
+      <c r="I128" t="s">
         <v>665</v>
-      </c>
-      <c r="I128" t="s">
-        <v>666</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
+        <v>666</v>
+      </c>
+      <c r="B129" t="s">
+        <v>36</v>
+      </c>
+      <c r="C129" t="s">
+        <v>10</v>
+      </c>
+      <c r="D129" t="s">
         <v>667</v>
       </c>
-      <c r="B129" t="s">
-        <v>84</v>
-      </c>
-      <c r="C129" t="s">
-        <v>10</v>
-      </c>
-      <c r="D129" t="s">
+      <c r="E129" t="s">
+        <v>13</v>
+      </c>
+      <c r="F129" t="s">
+        <v>98</v>
+      </c>
+      <c r="G129" t="s">
         <v>668</v>
       </c>
-      <c r="E129" t="s">
-        <v>13</v>
-      </c>
-      <c r="F129" t="s">
-        <v>31</v>
-      </c>
-      <c r="G129" t="s">
+      <c r="H129" t="s">
         <v>669</v>
       </c>
-      <c r="H129" t="s">
+      <c r="I129" t="s">
         <v>670</v>
-      </c>
-      <c r="I129" t="s">
-        <v>671</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
+        <v>671</v>
+      </c>
+      <c r="B130" t="s">
+        <v>96</v>
+      </c>
+      <c r="C130" t="s">
+        <v>10</v>
+      </c>
+      <c r="D130" t="s">
         <v>672</v>
       </c>
-      <c r="B130" t="s">
-        <v>638</v>
-      </c>
-      <c r="C130" t="s">
-        <v>10</v>
-      </c>
-      <c r="D130" t="s">
+      <c r="E130" t="s">
+        <v>13</v>
+      </c>
+      <c r="F130" t="s">
+        <v>98</v>
+      </c>
+      <c r="G130" t="s">
         <v>673</v>
       </c>
-      <c r="E130" t="s">
-        <v>13</v>
-      </c>
-      <c r="F130" t="s">
-        <v>116</v>
-      </c>
-      <c r="G130" t="s">
+      <c r="H130" t="s">
         <v>674</v>
-      </c>
-      <c r="H130" t="s">
-        <v>641</v>
       </c>
       <c r="I130" t="s">
         <v>675</v>
@@ -6678,7 +6915,7 @@
         <v>13</v>
       </c>
       <c r="F131" t="s">
-        <v>31</v>
+        <v>98</v>
       </c>
       <c r="G131" t="s">
         <v>678</v>
@@ -6695,71 +6932,71 @@
         <v>681</v>
       </c>
       <c r="B132" t="s">
-        <v>84</v>
+        <v>682</v>
       </c>
       <c r="C132" t="s">
         <v>10</v>
       </c>
       <c r="D132" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="E132" t="s">
         <v>13</v>
       </c>
       <c r="F132" t="s">
-        <v>31</v>
+        <v>684</v>
       </c>
       <c r="G132" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="H132" t="s">
-        <v>646</v>
+        <v>686</v>
       </c>
       <c r="I132" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="B133" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C133" t="s">
-        <v>633</v>
+        <v>10</v>
       </c>
       <c r="D133" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
       <c r="E133" t="s">
         <v>13</v>
       </c>
       <c r="F133" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G133" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="H133" t="s">
-        <v>10</v>
+        <v>691</v>
       </c>
       <c r="I133" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="B134" t="s">
         <v>10</v>
       </c>
       <c r="C134" t="s">
-        <v>633</v>
+        <v>11</v>
       </c>
       <c r="D134" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="E134" t="s">
         <v>13</v>
@@ -6768,53 +7005,53 @@
         <v>14</v>
       </c>
       <c r="G134" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="H134" t="s">
         <v>10</v>
       </c>
       <c r="I134" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="B135" t="s">
-        <v>694</v>
+        <v>18</v>
       </c>
       <c r="C135" t="s">
         <v>10</v>
       </c>
       <c r="D135" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="E135" t="s">
         <v>13</v>
       </c>
       <c r="F135" t="s">
-        <v>696</v>
+        <v>20</v>
       </c>
       <c r="G135" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="H135" t="s">
-        <v>698</v>
+        <v>461</v>
       </c>
       <c r="I135" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="B136" t="s">
-        <v>701</v>
+        <v>10</v>
       </c>
       <c r="C136" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="D136" t="s">
         <v>702</v>
@@ -6823,24 +7060,24 @@
         <v>13</v>
       </c>
       <c r="F136" t="s">
-        <v>116</v>
+        <v>14</v>
       </c>
       <c r="G136" t="s">
         <v>703</v>
       </c>
       <c r="H136" t="s">
+        <v>10</v>
+      </c>
+      <c r="I136" t="s">
         <v>704</v>
-      </c>
-      <c r="I136" t="s">
-        <v>705</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
+        <v>705</v>
+      </c>
+      <c r="B137" t="s">
         <v>706</v>
-      </c>
-      <c r="B137" t="s">
-        <v>701</v>
       </c>
       <c r="C137" t="s">
         <v>10</v>
@@ -6852,36 +7089,36 @@
         <v>13</v>
       </c>
       <c r="F137" t="s">
-        <v>116</v>
+        <v>708</v>
       </c>
       <c r="G137" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="H137" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="I137" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="B138" t="s">
-        <v>712</v>
+        <v>10</v>
       </c>
       <c r="C138" t="s">
-        <v>10</v>
+        <v>713</v>
       </c>
       <c r="D138" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="E138" t="s">
         <v>13</v>
       </c>
       <c r="F138" t="s">
-        <v>714</v>
+        <v>14</v>
       </c>
       <c r="G138" t="s">
         <v>715</v>
@@ -6898,42 +7135,42 @@
         <v>717</v>
       </c>
       <c r="B139" t="s">
-        <v>36</v>
+        <v>718</v>
       </c>
       <c r="C139" t="s">
         <v>10</v>
       </c>
       <c r="D139" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="E139" t="s">
         <v>13</v>
       </c>
       <c r="F139" t="s">
-        <v>31</v>
+        <v>116</v>
       </c>
       <c r="G139" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="H139" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="I139" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="B140" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C140" t="s">
         <v>10</v>
       </c>
       <c r="D140" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="E140" t="s">
         <v>13</v>
@@ -6942,39 +7179,39 @@
         <v>31</v>
       </c>
       <c r="G140" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="H140" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="I140" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="B141" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="C141" t="s">
-        <v>10</v>
+        <v>713</v>
       </c>
       <c r="D141" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="E141" t="s">
         <v>13</v>
       </c>
       <c r="F141" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G141" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="H141" t="s">
-        <v>730</v>
+        <v>10</v>
       </c>
       <c r="I141" t="s">
         <v>731</v>
@@ -7003,73 +7240,73 @@
         <v>734</v>
       </c>
       <c r="H142" t="s">
+        <v>659</v>
+      </c>
+      <c r="I142" t="s">
         <v>735</v>
-      </c>
-      <c r="I142" t="s">
-        <v>736</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
+        <v>736</v>
+      </c>
+      <c r="B143" t="s">
+        <v>36</v>
+      </c>
+      <c r="C143" t="s">
+        <v>10</v>
+      </c>
+      <c r="D143" t="s">
         <v>737</v>
       </c>
-      <c r="B143" t="s">
-        <v>84</v>
-      </c>
-      <c r="C143" t="s">
-        <v>10</v>
-      </c>
-      <c r="D143" t="s">
+      <c r="E143" t="s">
+        <v>13</v>
+      </c>
+      <c r="F143" t="s">
+        <v>31</v>
+      </c>
+      <c r="G143" t="s">
         <v>738</v>
       </c>
-      <c r="E143" t="s">
-        <v>13</v>
-      </c>
-      <c r="F143" t="s">
-        <v>31</v>
-      </c>
-      <c r="G143" t="s">
+      <c r="H143" t="s">
         <v>739</v>
       </c>
-      <c r="H143" t="s">
+      <c r="I143" t="s">
         <v>740</v>
-      </c>
-      <c r="I143" t="s">
-        <v>741</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
+        <v>741</v>
+      </c>
+      <c r="B144" t="s">
+        <v>84</v>
+      </c>
+      <c r="C144" t="s">
+        <v>10</v>
+      </c>
+      <c r="D144" t="s">
         <v>742</v>
       </c>
-      <c r="B144" t="s">
+      <c r="E144" t="s">
+        <v>13</v>
+      </c>
+      <c r="F144" t="s">
+        <v>31</v>
+      </c>
+      <c r="G144" t="s">
         <v>743</v>
       </c>
-      <c r="C144" t="s">
-        <v>10</v>
-      </c>
-      <c r="D144" t="s">
+      <c r="H144" t="s">
         <v>744</v>
       </c>
-      <c r="E144" t="s">
-        <v>13</v>
-      </c>
-      <c r="F144" t="s">
-        <v>31</v>
-      </c>
-      <c r="G144" t="s">
+      <c r="I144" t="s">
         <v>745</v>
-      </c>
-      <c r="H144" t="s">
-        <v>746</v>
-      </c>
-      <c r="I144" t="s">
-        <v>747</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="B145" t="s">
         <v>84</v>
@@ -7078,56 +7315,56 @@
         <v>10</v>
       </c>
       <c r="D145" t="s">
+        <v>747</v>
+      </c>
+      <c r="E145" t="s">
+        <v>13</v>
+      </c>
+      <c r="F145" t="s">
+        <v>31</v>
+      </c>
+      <c r="G145" t="s">
+        <v>748</v>
+      </c>
+      <c r="H145" t="s">
         <v>749</v>
       </c>
-      <c r="E145" t="s">
-        <v>13</v>
-      </c>
-      <c r="F145" t="s">
-        <v>31</v>
-      </c>
-      <c r="G145" t="s">
+      <c r="I145" t="s">
         <v>750</v>
-      </c>
-      <c r="H145" t="s">
-        <v>751</v>
-      </c>
-      <c r="I145" t="s">
-        <v>752</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
+        <v>751</v>
+      </c>
+      <c r="B146" t="s">
+        <v>718</v>
+      </c>
+      <c r="C146" t="s">
+        <v>10</v>
+      </c>
+      <c r="D146" t="s">
+        <v>752</v>
+      </c>
+      <c r="E146" t="s">
+        <v>13</v>
+      </c>
+      <c r="F146" t="s">
+        <v>116</v>
+      </c>
+      <c r="G146" t="s">
         <v>753</v>
       </c>
-      <c r="B146" t="s">
-        <v>84</v>
-      </c>
-      <c r="C146" t="s">
-        <v>10</v>
-      </c>
-      <c r="D146" t="s">
+      <c r="H146" t="s">
+        <v>721</v>
+      </c>
+      <c r="I146" t="s">
         <v>754</v>
-      </c>
-      <c r="E146" t="s">
-        <v>13</v>
-      </c>
-      <c r="F146" t="s">
-        <v>31</v>
-      </c>
-      <c r="G146" t="s">
-        <v>755</v>
-      </c>
-      <c r="H146" t="s">
-        <v>756</v>
-      </c>
-      <c r="I146" t="s">
-        <v>757</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="B147" t="s">
         <v>36</v>
@@ -7136,370 +7373,834 @@
         <v>10</v>
       </c>
       <c r="D147" t="s">
+        <v>756</v>
+      </c>
+      <c r="E147" t="s">
+        <v>13</v>
+      </c>
+      <c r="F147" t="s">
+        <v>31</v>
+      </c>
+      <c r="G147" t="s">
+        <v>757</v>
+      </c>
+      <c r="H147" t="s">
+        <v>758</v>
+      </c>
+      <c r="I147" t="s">
         <v>759</v>
-      </c>
-      <c r="E147" t="s">
-        <v>13</v>
-      </c>
-      <c r="F147" t="s">
-        <v>31</v>
-      </c>
-      <c r="G147" t="s">
-        <v>760</v>
-      </c>
-      <c r="H147" t="s">
-        <v>761</v>
-      </c>
-      <c r="I147" t="s">
-        <v>762</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
+        <v>760</v>
+      </c>
+      <c r="B148" t="s">
+        <v>84</v>
+      </c>
+      <c r="C148" t="s">
+        <v>10</v>
+      </c>
+      <c r="D148" t="s">
+        <v>761</v>
+      </c>
+      <c r="E148" t="s">
+        <v>13</v>
+      </c>
+      <c r="F148" t="s">
+        <v>31</v>
+      </c>
+      <c r="G148" t="s">
+        <v>762</v>
+      </c>
+      <c r="H148" t="s">
+        <v>726</v>
+      </c>
+      <c r="I148" t="s">
         <v>763</v>
-      </c>
-      <c r="B148" t="s">
-        <v>36</v>
-      </c>
-      <c r="C148" t="s">
-        <v>10</v>
-      </c>
-      <c r="D148" t="s">
-        <v>764</v>
-      </c>
-      <c r="E148" t="s">
-        <v>13</v>
-      </c>
-      <c r="F148" t="s">
-        <v>31</v>
-      </c>
-      <c r="G148" t="s">
-        <v>765</v>
-      </c>
-      <c r="H148" t="s">
-        <v>766</v>
-      </c>
-      <c r="I148" t="s">
-        <v>767</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="B149" t="s">
-        <v>84</v>
+        <v>10</v>
       </c>
       <c r="C149" t="s">
-        <v>10</v>
+        <v>713</v>
       </c>
       <c r="D149" t="s">
-        <v>769</v>
+        <v>765</v>
       </c>
       <c r="E149" t="s">
         <v>13</v>
       </c>
       <c r="F149" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G149" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="H149" t="s">
-        <v>771</v>
+        <v>10</v>
       </c>
       <c r="I149" t="s">
-        <v>772</v>
+        <v>767</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>773</v>
+        <v>768</v>
       </c>
       <c r="B150" t="s">
-        <v>237</v>
+        <v>10</v>
       </c>
       <c r="C150" t="s">
-        <v>10</v>
+        <v>713</v>
       </c>
       <c r="D150" t="s">
-        <v>774</v>
+        <v>769</v>
       </c>
       <c r="E150" t="s">
         <v>13</v>
       </c>
       <c r="F150" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G150" t="s">
-        <v>775</v>
+        <v>770</v>
       </c>
       <c r="H150" t="s">
-        <v>776</v>
+        <v>10</v>
       </c>
       <c r="I150" t="s">
-        <v>777</v>
+        <v>771</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
+        <v>772</v>
+      </c>
+      <c r="B151" t="s">
+        <v>773</v>
+      </c>
+      <c r="C151" t="s">
+        <v>10</v>
+      </c>
+      <c r="D151" t="s">
+        <v>774</v>
+      </c>
+      <c r="E151" t="s">
+        <v>13</v>
+      </c>
+      <c r="F151" t="s">
+        <v>775</v>
+      </c>
+      <c r="G151" t="s">
+        <v>776</v>
+      </c>
+      <c r="H151" t="s">
+        <v>777</v>
+      </c>
+      <c r="I151" t="s">
         <v>778</v>
-      </c>
-      <c r="B151" t="s">
-        <v>195</v>
-      </c>
-      <c r="C151" t="s">
-        <v>10</v>
-      </c>
-      <c r="D151" t="s">
-        <v>779</v>
-      </c>
-      <c r="E151" t="s">
-        <v>13</v>
-      </c>
-      <c r="F151" t="s">
-        <v>31</v>
-      </c>
-      <c r="G151" t="s">
-        <v>780</v>
-      </c>
-      <c r="H151" t="s">
-        <v>781</v>
-      </c>
-      <c r="I151" t="s">
-        <v>782</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
+        <v>779</v>
+      </c>
+      <c r="B152" t="s">
+        <v>780</v>
+      </c>
+      <c r="C152" t="s">
+        <v>10</v>
+      </c>
+      <c r="D152" t="s">
+        <v>781</v>
+      </c>
+      <c r="E152" t="s">
+        <v>13</v>
+      </c>
+      <c r="F152" t="s">
+        <v>116</v>
+      </c>
+      <c r="G152" t="s">
+        <v>782</v>
+      </c>
+      <c r="H152" t="s">
         <v>783</v>
       </c>
-      <c r="B152" t="s">
-        <v>36</v>
-      </c>
-      <c r="C152" t="s">
-        <v>10</v>
-      </c>
-      <c r="D152" t="s">
+      <c r="I152" t="s">
         <v>784</v>
-      </c>
-      <c r="E152" t="s">
-        <v>13</v>
-      </c>
-      <c r="F152" t="s">
-        <v>31</v>
-      </c>
-      <c r="G152" t="s">
-        <v>785</v>
-      </c>
-      <c r="H152" t="s">
-        <v>786</v>
-      </c>
-      <c r="I152" t="s">
-        <v>787</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
+        <v>785</v>
+      </c>
+      <c r="B153" t="s">
+        <v>780</v>
+      </c>
+      <c r="C153" t="s">
+        <v>10</v>
+      </c>
+      <c r="D153" t="s">
+        <v>786</v>
+      </c>
+      <c r="E153" t="s">
+        <v>13</v>
+      </c>
+      <c r="F153" t="s">
+        <v>116</v>
+      </c>
+      <c r="G153" t="s">
+        <v>787</v>
+      </c>
+      <c r="H153" t="s">
         <v>788</v>
       </c>
-      <c r="B153" t="s">
-        <v>84</v>
-      </c>
-      <c r="C153" t="s">
-        <v>10</v>
-      </c>
-      <c r="D153" t="s">
+      <c r="I153" t="s">
         <v>789</v>
-      </c>
-      <c r="E153" t="s">
-        <v>13</v>
-      </c>
-      <c r="F153" t="s">
-        <v>31</v>
-      </c>
-      <c r="G153" t="s">
-        <v>790</v>
-      </c>
-      <c r="H153" t="s">
-        <v>791</v>
-      </c>
-      <c r="I153" t="s">
-        <v>792</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
+        <v>790</v>
+      </c>
+      <c r="B154" t="s">
+        <v>791</v>
+      </c>
+      <c r="C154" t="s">
+        <v>10</v>
+      </c>
+      <c r="D154" t="s">
+        <v>792</v>
+      </c>
+      <c r="E154" t="s">
+        <v>13</v>
+      </c>
+      <c r="F154" t="s">
         <v>793</v>
       </c>
-      <c r="B154" t="s">
-        <v>36</v>
-      </c>
-      <c r="C154" t="s">
-        <v>10</v>
-      </c>
-      <c r="D154" t="s">
+      <c r="G154" t="s">
         <v>794</v>
       </c>
-      <c r="E154" t="s">
-        <v>13</v>
-      </c>
-      <c r="F154" t="s">
-        <v>31</v>
-      </c>
-      <c r="G154" t="s">
+      <c r="H154" t="s">
+        <v>10</v>
+      </c>
+      <c r="I154" t="s">
         <v>795</v>
-      </c>
-      <c r="H154" t="s">
-        <v>796</v>
-      </c>
-      <c r="I154" t="s">
-        <v>797</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
+        <v>796</v>
+      </c>
+      <c r="B155" t="s">
+        <v>36</v>
+      </c>
+      <c r="C155" t="s">
+        <v>10</v>
+      </c>
+      <c r="D155" t="s">
+        <v>797</v>
+      </c>
+      <c r="E155" t="s">
+        <v>13</v>
+      </c>
+      <c r="F155" t="s">
+        <v>31</v>
+      </c>
+      <c r="G155" t="s">
         <v>798</v>
       </c>
-      <c r="B155" t="s">
-        <v>84</v>
-      </c>
-      <c r="C155" t="s">
-        <v>10</v>
-      </c>
-      <c r="D155" t="s">
+      <c r="H155" t="s">
         <v>799</v>
       </c>
-      <c r="E155" t="s">
-        <v>13</v>
-      </c>
-      <c r="F155" t="s">
-        <v>31</v>
-      </c>
-      <c r="G155" t="s">
+      <c r="I155" t="s">
         <v>800</v>
-      </c>
-      <c r="H155" t="s">
-        <v>801</v>
-      </c>
-      <c r="I155" t="s">
-        <v>802</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
+        <v>801</v>
+      </c>
+      <c r="B156" t="s">
+        <v>90</v>
+      </c>
+      <c r="C156" t="s">
+        <v>10</v>
+      </c>
+      <c r="D156" t="s">
+        <v>802</v>
+      </c>
+      <c r="E156" t="s">
+        <v>13</v>
+      </c>
+      <c r="F156" t="s">
+        <v>31</v>
+      </c>
+      <c r="G156" t="s">
         <v>803</v>
       </c>
-      <c r="B156" t="s">
+      <c r="H156" t="s">
         <v>804</v>
       </c>
-      <c r="C156" t="s">
-        <v>10</v>
-      </c>
-      <c r="D156" t="s">
+      <c r="I156" t="s">
         <v>805</v>
-      </c>
-      <c r="E156" t="s">
-        <v>13</v>
-      </c>
-      <c r="F156" t="s">
-        <v>31</v>
-      </c>
-      <c r="G156" t="s">
-        <v>806</v>
-      </c>
-      <c r="H156" t="s">
-        <v>807</v>
-      </c>
-      <c r="I156" t="s">
-        <v>808</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
+        <v>806</v>
+      </c>
+      <c r="B157" t="s">
+        <v>36</v>
+      </c>
+      <c r="C157" t="s">
+        <v>10</v>
+      </c>
+      <c r="D157" t="s">
+        <v>807</v>
+      </c>
+      <c r="E157" t="s">
+        <v>13</v>
+      </c>
+      <c r="F157" t="s">
+        <v>31</v>
+      </c>
+      <c r="G157" t="s">
+        <v>808</v>
+      </c>
+      <c r="H157" t="s">
         <v>809</v>
       </c>
-      <c r="B157" t="s">
-        <v>84</v>
-      </c>
-      <c r="C157" t="s">
-        <v>10</v>
-      </c>
-      <c r="D157" t="s">
+      <c r="I157" t="s">
         <v>810</v>
-      </c>
-      <c r="E157" t="s">
-        <v>13</v>
-      </c>
-      <c r="F157" t="s">
-        <v>31</v>
-      </c>
-      <c r="G157" t="s">
-        <v>811</v>
-      </c>
-      <c r="H157" t="s">
-        <v>812</v>
-      </c>
-      <c r="I157" t="s">
-        <v>813</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
+        <v>811</v>
+      </c>
+      <c r="B158" t="s">
+        <v>36</v>
+      </c>
+      <c r="C158" t="s">
+        <v>10</v>
+      </c>
+      <c r="D158" t="s">
+        <v>812</v>
+      </c>
+      <c r="E158" t="s">
+        <v>13</v>
+      </c>
+      <c r="F158" t="s">
+        <v>31</v>
+      </c>
+      <c r="G158" t="s">
+        <v>813</v>
+      </c>
+      <c r="H158" t="s">
         <v>814</v>
       </c>
-      <c r="B158" t="s">
+      <c r="I158" t="s">
         <v>815</v>
-      </c>
-      <c r="C158" t="s">
-        <v>10</v>
-      </c>
-      <c r="D158" t="s">
-        <v>816</v>
-      </c>
-      <c r="E158" t="s">
-        <v>13</v>
-      </c>
-      <c r="F158" t="s">
-        <v>696</v>
-      </c>
-      <c r="G158" t="s">
-        <v>817</v>
-      </c>
-      <c r="H158" t="s">
-        <v>818</v>
-      </c>
-      <c r="I158" t="s">
-        <v>819</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
+        <v>816</v>
+      </c>
+      <c r="B159" t="s">
+        <v>84</v>
+      </c>
+      <c r="C159" t="s">
+        <v>10</v>
+      </c>
+      <c r="D159" t="s">
+        <v>817</v>
+      </c>
+      <c r="E159" t="s">
+        <v>13</v>
+      </c>
+      <c r="F159" t="s">
+        <v>31</v>
+      </c>
+      <c r="G159" t="s">
+        <v>818</v>
+      </c>
+      <c r="H159" t="s">
+        <v>819</v>
+      </c>
+      <c r="I159" t="s">
         <v>820</v>
       </c>
-      <c r="B159" t="s">
+    </row>
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
         <v>821</v>
       </c>
-      <c r="C159" t="s">
-        <v>10</v>
-      </c>
-      <c r="D159" t="s">
+      <c r="B160" t="s">
         <v>822</v>
       </c>
-      <c r="E159" t="s">
-        <v>13</v>
-      </c>
-      <c r="F159" t="s">
+      <c r="C160" t="s">
+        <v>10</v>
+      </c>
+      <c r="D160" t="s">
         <v>823</v>
       </c>
-      <c r="G159" t="s">
+      <c r="E160" t="s">
+        <v>13</v>
+      </c>
+      <c r="F160" t="s">
+        <v>31</v>
+      </c>
+      <c r="G160" t="s">
         <v>824</v>
       </c>
-      <c r="H159" t="s">
+      <c r="H160" t="s">
         <v>825</v>
       </c>
-      <c r="I159" t="s">
+      <c r="I160" t="s">
         <v>826</v>
+      </c>
+    </row>
+    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>827</v>
+      </c>
+      <c r="B161" t="s">
+        <v>84</v>
+      </c>
+      <c r="C161" t="s">
+        <v>10</v>
+      </c>
+      <c r="D161" t="s">
+        <v>828</v>
+      </c>
+      <c r="E161" t="s">
+        <v>13</v>
+      </c>
+      <c r="F161" t="s">
+        <v>31</v>
+      </c>
+      <c r="G161" t="s">
+        <v>829</v>
+      </c>
+      <c r="H161" t="s">
+        <v>830</v>
+      </c>
+      <c r="I161" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>832</v>
+      </c>
+      <c r="B162" t="s">
+        <v>84</v>
+      </c>
+      <c r="C162" t="s">
+        <v>10</v>
+      </c>
+      <c r="D162" t="s">
+        <v>833</v>
+      </c>
+      <c r="E162" t="s">
+        <v>13</v>
+      </c>
+      <c r="F162" t="s">
+        <v>31</v>
+      </c>
+      <c r="G162" t="s">
+        <v>834</v>
+      </c>
+      <c r="H162" t="s">
+        <v>835</v>
+      </c>
+      <c r="I162" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>837</v>
+      </c>
+      <c r="B163" t="s">
+        <v>36</v>
+      </c>
+      <c r="C163" t="s">
+        <v>10</v>
+      </c>
+      <c r="D163" t="s">
+        <v>838</v>
+      </c>
+      <c r="E163" t="s">
+        <v>13</v>
+      </c>
+      <c r="F163" t="s">
+        <v>31</v>
+      </c>
+      <c r="G163" t="s">
+        <v>839</v>
+      </c>
+      <c r="H163" t="s">
+        <v>840</v>
+      </c>
+      <c r="I163" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>842</v>
+      </c>
+      <c r="B164" t="s">
+        <v>36</v>
+      </c>
+      <c r="C164" t="s">
+        <v>10</v>
+      </c>
+      <c r="D164" t="s">
+        <v>843</v>
+      </c>
+      <c r="E164" t="s">
+        <v>13</v>
+      </c>
+      <c r="F164" t="s">
+        <v>31</v>
+      </c>
+      <c r="G164" t="s">
+        <v>844</v>
+      </c>
+      <c r="H164" t="s">
+        <v>845</v>
+      </c>
+      <c r="I164" t="s">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>847</v>
+      </c>
+      <c r="B165" t="s">
+        <v>84</v>
+      </c>
+      <c r="C165" t="s">
+        <v>10</v>
+      </c>
+      <c r="D165" t="s">
+        <v>848</v>
+      </c>
+      <c r="E165" t="s">
+        <v>13</v>
+      </c>
+      <c r="F165" t="s">
+        <v>31</v>
+      </c>
+      <c r="G165" t="s">
+        <v>849</v>
+      </c>
+      <c r="H165" t="s">
+        <v>850</v>
+      </c>
+      <c r="I165" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>852</v>
+      </c>
+      <c r="B166" t="s">
+        <v>237</v>
+      </c>
+      <c r="C166" t="s">
+        <v>10</v>
+      </c>
+      <c r="D166" t="s">
+        <v>853</v>
+      </c>
+      <c r="E166" t="s">
+        <v>13</v>
+      </c>
+      <c r="F166" t="s">
+        <v>31</v>
+      </c>
+      <c r="G166" t="s">
+        <v>854</v>
+      </c>
+      <c r="H166" t="s">
+        <v>855</v>
+      </c>
+      <c r="I166" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>857</v>
+      </c>
+      <c r="B167" t="s">
+        <v>195</v>
+      </c>
+      <c r="C167" t="s">
+        <v>10</v>
+      </c>
+      <c r="D167" t="s">
+        <v>858</v>
+      </c>
+      <c r="E167" t="s">
+        <v>13</v>
+      </c>
+      <c r="F167" t="s">
+        <v>31</v>
+      </c>
+      <c r="G167" t="s">
+        <v>859</v>
+      </c>
+      <c r="H167" t="s">
+        <v>860</v>
+      </c>
+      <c r="I167" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>862</v>
+      </c>
+      <c r="B168" t="s">
+        <v>36</v>
+      </c>
+      <c r="C168" t="s">
+        <v>10</v>
+      </c>
+      <c r="D168" t="s">
+        <v>863</v>
+      </c>
+      <c r="E168" t="s">
+        <v>13</v>
+      </c>
+      <c r="F168" t="s">
+        <v>31</v>
+      </c>
+      <c r="G168" t="s">
+        <v>864</v>
+      </c>
+      <c r="H168" t="s">
+        <v>865</v>
+      </c>
+      <c r="I168" t="s">
+        <v>866</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>867</v>
+      </c>
+      <c r="B169" t="s">
+        <v>84</v>
+      </c>
+      <c r="C169" t="s">
+        <v>10</v>
+      </c>
+      <c r="D169" t="s">
+        <v>868</v>
+      </c>
+      <c r="E169" t="s">
+        <v>13</v>
+      </c>
+      <c r="F169" t="s">
+        <v>31</v>
+      </c>
+      <c r="G169" t="s">
+        <v>869</v>
+      </c>
+      <c r="H169" t="s">
+        <v>870</v>
+      </c>
+      <c r="I169" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>872</v>
+      </c>
+      <c r="B170" t="s">
+        <v>36</v>
+      </c>
+      <c r="C170" t="s">
+        <v>10</v>
+      </c>
+      <c r="D170" t="s">
+        <v>873</v>
+      </c>
+      <c r="E170" t="s">
+        <v>13</v>
+      </c>
+      <c r="F170" t="s">
+        <v>31</v>
+      </c>
+      <c r="G170" t="s">
+        <v>874</v>
+      </c>
+      <c r="H170" t="s">
+        <v>875</v>
+      </c>
+      <c r="I170" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>877</v>
+      </c>
+      <c r="B171" t="s">
+        <v>84</v>
+      </c>
+      <c r="C171" t="s">
+        <v>10</v>
+      </c>
+      <c r="D171" t="s">
+        <v>878</v>
+      </c>
+      <c r="E171" t="s">
+        <v>13</v>
+      </c>
+      <c r="F171" t="s">
+        <v>31</v>
+      </c>
+      <c r="G171" t="s">
+        <v>879</v>
+      </c>
+      <c r="H171" t="s">
+        <v>880</v>
+      </c>
+      <c r="I171" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>882</v>
+      </c>
+      <c r="B172" t="s">
+        <v>883</v>
+      </c>
+      <c r="C172" t="s">
+        <v>10</v>
+      </c>
+      <c r="D172" t="s">
+        <v>884</v>
+      </c>
+      <c r="E172" t="s">
+        <v>13</v>
+      </c>
+      <c r="F172" t="s">
+        <v>31</v>
+      </c>
+      <c r="G172" t="s">
+        <v>885</v>
+      </c>
+      <c r="H172" t="s">
+        <v>886</v>
+      </c>
+      <c r="I172" t="s">
+        <v>887</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>888</v>
+      </c>
+      <c r="B173" t="s">
+        <v>84</v>
+      </c>
+      <c r="C173" t="s">
+        <v>10</v>
+      </c>
+      <c r="D173" t="s">
+        <v>889</v>
+      </c>
+      <c r="E173" t="s">
+        <v>13</v>
+      </c>
+      <c r="F173" t="s">
+        <v>31</v>
+      </c>
+      <c r="G173" t="s">
+        <v>890</v>
+      </c>
+      <c r="H173" t="s">
+        <v>891</v>
+      </c>
+      <c r="I173" t="s">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>893</v>
+      </c>
+      <c r="B174" t="s">
+        <v>894</v>
+      </c>
+      <c r="C174" t="s">
+        <v>10</v>
+      </c>
+      <c r="D174" t="s">
+        <v>895</v>
+      </c>
+      <c r="E174" t="s">
+        <v>13</v>
+      </c>
+      <c r="F174" t="s">
+        <v>775</v>
+      </c>
+      <c r="G174" t="s">
+        <v>896</v>
+      </c>
+      <c r="H174" t="s">
+        <v>897</v>
+      </c>
+      <c r="I174" t="s">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>899</v>
+      </c>
+      <c r="B175" t="s">
+        <v>900</v>
+      </c>
+      <c r="C175" t="s">
+        <v>10</v>
+      </c>
+      <c r="D175" t="s">
+        <v>901</v>
+      </c>
+      <c r="E175" t="s">
+        <v>13</v>
+      </c>
+      <c r="F175" t="s">
+        <v>902</v>
+      </c>
+      <c r="G175" t="s">
+        <v>903</v>
+      </c>
+      <c r="H175" t="s">
+        <v>904</v>
+      </c>
+      <c r="I175" t="s">
+        <v>905</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: checkpoint (capture/import/upload batches)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-info.report.xlsx
+++ b/tools/importer/reports/import-info.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1737" uniqueCount="997">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2088" uniqueCount="1191">
   <si>
     <t>_reportFile</t>
   </si>
@@ -364,7 +364,7 @@
     <t>campaign</t>
   </si>
   <si>
-    <t>2026-10-21T22:34:52.969Z</t>
+    <t>2026-10-22T00:11:17.425Z</t>
   </si>
   <si>
     <t>100 Years Lufthansa | Lufthansa</t>
@@ -385,7 +385,7 @@
     <t>fleet</t>
   </si>
   <si>
-    <t>2026-10-21T22:35:08.686Z</t>
+    <t>2026-10-22T00:11:32.785Z</t>
   </si>
   <si>
     <t>Airbus A350-900 | Lufthansa</t>
@@ -1033,7 +1033,7 @@
     <t>form</t>
   </si>
   <si>
-    <t>2026-10-21T22:35:24.617Z</t>
+    <t>2026-10-22T00:11:47.818Z</t>
   </si>
   <si>
     <t>Feedback and other contact forms | Lufthansa</t>
@@ -1429,7 +1429,7 @@
     <t>legal</t>
   </si>
   <si>
-    <t>2026-10-21T22:35:19.333Z</t>
+    <t>2026-10-22T00:11:42.520Z</t>
   </si>
   <si>
     <t>Legal notice | Lufthansa</t>
@@ -1897,7 +1897,7 @@
     <t>app-entry</t>
   </si>
   <si>
-    <t>2026-10-21T22:35:29.211Z</t>
+    <t>2026-10-22T00:11:53.146Z</t>
   </si>
   <si>
     <t>Online check-in | Lufthansa</t>
@@ -2059,6 +2059,123 @@
     <t>https://www.lufthansa.com/de/en/premium-economy-class</t>
   </si>
   <si>
+    <t>de/en/rail-and-fly.report.json</t>
+  </si>
+  <si>
+    <t>de/en/rail-and-fly</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:20.429Z</t>
+  </si>
+  <si>
+    <t>To your flight with Rail&amp;Fly | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/rail-and-fly</t>
+  </si>
+  <si>
+    <t>de/en/rechnungsbeleg.report.json</t>
+  </si>
+  <si>
+    <t>de/en/rechnungsbeleg</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:22.810Z</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/rechnungsbeleg</t>
+  </si>
+  <si>
+    <t>de/en/refund.report.json</t>
+  </si>
+  <si>
+    <t>de/en/refund</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:25.438Z</t>
+  </si>
+  <si>
+    <t>Refunds | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/refund</t>
+  </si>
+  <si>
+    <t>de/en/schengen.report.json</t>
+  </si>
+  <si>
+    <t>de/en/schengen</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:28.174Z</t>
+  </si>
+  <si>
+    <t>Entry into the Schengen Area | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/schengen</t>
+  </si>
+  <si>
+    <t>de/en/secure-flight.report.json</t>
+  </si>
+  <si>
+    <t>de/en/secure-flight</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:30.634Z</t>
+  </si>
+  <si>
+    <t>Secure Flight | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/secure-flight</t>
+  </si>
+  <si>
+    <t>de/en/security-check-time-slot.report.json</t>
+  </si>
+  <si>
+    <t>de/en/security-check-time-slot</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:33.554Z</t>
+  </si>
+  <si>
+    <t>Faster through security check | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/security-check-time-slot</t>
+  </si>
+  <si>
+    <t>de/en/security-fast-lanes.report.json</t>
+  </si>
+  <si>
+    <t>de/en/security-fast-lanes</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:35.541Z</t>
+  </si>
+  <si>
+    <t>Security Fast Lanes | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/security-fast-lanes</t>
+  </si>
+  <si>
+    <t>de/en/services-at-frankfurt-airport.report.json</t>
+  </si>
+  <si>
+    <t>de/en/services-at-frankfurt-airport</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:37.730Z</t>
+  </si>
+  <si>
+    <t>Services at Frankfurt Airport | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/services-at-frankfurt-airport</t>
+  </si>
+  <si>
     <t>de/en/services-at-the-airport.report.json</t>
   </si>
   <si>
@@ -2074,6 +2191,21 @@
     <t>https://www.lufthansa.com/de/en/services-at-the-airport</t>
   </si>
   <si>
+    <t>de/en/services-munich-airport.report.json</t>
+  </si>
+  <si>
+    <t>de/en/services-munich-airport</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:39.979Z</t>
+  </si>
+  <si>
+    <t>Services at Munich Airport | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/services-munich-airport</t>
+  </si>
+  <si>
     <t>de/en/services-on-board.report.json</t>
   </si>
   <si>
@@ -2089,6 +2221,51 @@
     <t>https://www.lufthansa.com/de/en/services-on-board</t>
   </si>
   <si>
+    <t>de/en/shopping.report.json</t>
+  </si>
+  <si>
+    <t>de/en/shopping</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:42.743Z</t>
+  </si>
+  <si>
+    <t>Inflight shopping, worldshop airport stores and online | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/shopping</t>
+  </si>
+  <si>
+    <t>de/en/sixt.report.json</t>
+  </si>
+  <si>
+    <t>de/en/sixt</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:45.864Z</t>
+  </si>
+  <si>
+    <t>Sixt | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/sixt</t>
+  </si>
+  <si>
+    <t>de/en/special-meals.report.json</t>
+  </si>
+  <si>
+    <t>de/en/special-meals</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:47.959Z</t>
+  </si>
+  <si>
+    <t>Special meals | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/special-meals</t>
+  </si>
+  <si>
     <t>de/en/special-needs.report.json</t>
   </si>
   <si>
@@ -2104,6 +2281,51 @@
     <t>https://www.lufthansa.com/de/en/special-needs</t>
   </si>
   <si>
+    <t>de/en/sports-baggage.report.json</t>
+  </si>
+  <si>
+    <t>de/en/sports-baggage</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:20.867Z</t>
+  </si>
+  <si>
+    <t>Sports baggage and special baggage | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/sports-baggage</t>
+  </si>
+  <si>
+    <t>de/en/tiere-als-handgepaeck.report.json</t>
+  </si>
+  <si>
+    <t>de/en/tiere-als-handgepaeck</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:27.322Z</t>
+  </si>
+  <si>
+    <t>Animals as additional carry-on baggage | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/tiere-als-handgepaeck</t>
+  </si>
+  <si>
+    <t>de/en/tiere-als-uebergepaeck.report.json</t>
+  </si>
+  <si>
+    <t>de/en/tiere-als-uebergepaeck</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:29.627Z</t>
+  </si>
+  <si>
+    <t>Animals as excess baggage | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/tiere-als-uebergepaeck</t>
+  </si>
+  <si>
     <t>de/en/timetable-and-flight-status.report.json</t>
   </si>
   <si>
@@ -2116,7 +2338,7 @@
     <t>flight-status</t>
   </si>
   <si>
-    <t>2026-10-21T22:35:34.539Z</t>
+    <t>2026-10-22T00:11:58.851Z</t>
   </si>
   <si>
     <t>Timetable &amp; flight status | Lufthansa</t>
@@ -2125,6 +2347,156 @@
     <t>https://www.lufthansa.com/de/en/timetable-and-flight-status</t>
   </si>
   <si>
+    <t>de/en/tips-senior-travellers.report.json</t>
+  </si>
+  <si>
+    <t>de/en/tips-senior-travellers</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:32.021Z</t>
+  </si>
+  <si>
+    <t>Older travellers | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/tips-senior-travellers</t>
+  </si>
+  <si>
+    <t>de/en/travel-agencies.report.json</t>
+  </si>
+  <si>
+    <t>de/en/travel-agencies</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:34.516Z</t>
+  </si>
+  <si>
+    <t>For travel agents | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/travel-agencies</t>
+  </si>
+  <si>
+    <t>de/en/travel-expense-management.report.json</t>
+  </si>
+  <si>
+    <t>de/en/travel-expense-management</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:37.710Z</t>
+  </si>
+  <si>
+    <t>Travel Expense Management | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/travel-expense-management</t>
+  </si>
+  <si>
+    <t>de/en/travelling-healthy.report.json</t>
+  </si>
+  <si>
+    <t>de/en/travelling-healthy</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:41.167Z</t>
+  </si>
+  <si>
+    <t>A healthy journey | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/travelling-healthy</t>
+  </si>
+  <si>
+    <t>de/en/travelling-with-animals.report.json</t>
+  </si>
+  <si>
+    <t>de/en/travelling-with-animals</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:43.834Z</t>
+  </si>
+  <si>
+    <t>Travelling with animals | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/travelling-with-animals</t>
+  </si>
+  <si>
+    <t>de/en/travelling-with-children.report.json</t>
+  </si>
+  <si>
+    <t>de/en/travelling-with-children</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:46.314Z</t>
+  </si>
+  <si>
+    <t>Flying with children: tips and information | Lufthansa | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/travelling-with-children</t>
+  </si>
+  <si>
+    <t>de/en/travelling-with-special-requirements.report.json</t>
+  </si>
+  <si>
+    <t>de/en/travelling-with-special-requirements</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:49.339Z</t>
+  </si>
+  <si>
+    <t>Travelling with assistance requirements | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/travelling-with-special-requirements</t>
+  </si>
+  <si>
+    <t>de/en/traveltricks.report.json</t>
+  </si>
+  <si>
+    <t>de/en/traveltricks</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:18.272Z</t>
+  </si>
+  <si>
+    <t>Lufthansa Traveltricks | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/traveltricks</t>
+  </si>
+  <si>
+    <t>de/en/uebergepaeck.report.json</t>
+  </si>
+  <si>
+    <t>de/en/uebergepaeck</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:21.465Z</t>
+  </si>
+  <si>
+    <t>Excess baggage | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/uebergepaeck</t>
+  </si>
+  <si>
+    <t>de/en/unaccompanied-minors.report.json</t>
+  </si>
+  <si>
+    <t>de/en/unaccompanied-minors</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:24.766Z</t>
+  </si>
+  <si>
+    <t>Unaccompanied children | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/unaccompanied-minors</t>
+  </si>
+  <si>
     <t>de/en/unterhaltung-an-bord.report.json</t>
   </si>
   <si>
@@ -2140,6 +2512,156 @@
     <t>https://www.lufthansa.com/de/en/unterhaltung-an-bord</t>
   </si>
   <si>
+    <t>de/en/upgrade-business-class-long-haul.report.json</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-business-class-long-haul</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:26.792Z</t>
+  </si>
+  <si>
+    <t>Upgrade to Lufthansa business class | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/upgrade-business-class-long-haul</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-first-class.report.json</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-first-class</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:29.510Z</t>
+  </si>
+  <si>
+    <t>Upgrade to Lufthansa first class | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/upgrade-first-class</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-info.report.json</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-info</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:32.210Z</t>
+  </si>
+  <si>
+    <t>General information about your upgrades | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/upgrade-info</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-options.report.json</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-options</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:35.160Z</t>
+  </si>
+  <si>
+    <t>Upgrade options | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/upgrade-options</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-premium-economy-class.report.json</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-premium-economy-class</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:37.318Z</t>
+  </si>
+  <si>
+    <t>A little luxury: the Premium Economy Class upgrade | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/upgrade-premium-economy-class</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-to-business-class.report.json</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-to-business-class</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:39.477Z</t>
+  </si>
+  <si>
+    <t>Upgrade to Lufthansa Business Class | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/upgrade-to-business-class</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-to-premium-economy-class.report.json</t>
+  </si>
+  <si>
+    <t>de/en/upgrade-to-premium-economy-class</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:41.681Z</t>
+  </si>
+  <si>
+    <t>Premium Economy Class – your upgrade options | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/upgrade-to-premium-economy-class</t>
+  </si>
+  <si>
+    <t>de/en/upgrades-at-online-check-in.report.json</t>
+  </si>
+  <si>
+    <t>de/en/upgrades-at-online-check-in</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:44.370Z</t>
+  </si>
+  <si>
+    <t>Fixed price upgrades when you check in online | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/upgrades-at-online-check-in</t>
+  </si>
+  <si>
+    <t>de/en/wheelchair-batteries.report.json</t>
+  </si>
+  <si>
+    <t>de/en/wheelchair-batteries</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:47.294Z</t>
+  </si>
+  <si>
+    <t>Conditions for the carriage of wheelchair batteries | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/wheelchair-batteries</t>
+  </si>
+  <si>
+    <t>de/en/with-children-at-the-airport.report.json</t>
+  </si>
+  <si>
+    <t>de/en/with-children-at-the-airport</t>
+  </si>
+  <si>
+    <t>2026-10-22T01:00:49.659Z</t>
+  </si>
+  <si>
+    <t>At the airport with children | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/with-children-at-the-airport</t>
+  </si>
+  <si>
     <t>gb/en/footer.report.json</t>
   </si>
   <si>
@@ -2188,7 +2710,7 @@
     <t>aircore-destination-overview</t>
   </si>
   <si>
-    <t>2026-10-21T22:35:43.227Z</t>
+    <t>2026-10-22T00:12:06.910Z</t>
   </si>
   <si>
     <t>Book flights to destinations all over the world | Lufthansa</t>
@@ -2221,7 +2743,7 @@
     <t>de/de/discover-lufthansa/new-onboard-experience</t>
   </si>
   <si>
-    <t>2026-10-21T22:35:03.116Z</t>
+    <t>2026-10-22T00:11:27.425Z</t>
   </si>
   <si>
     <t>New Onboard Experience | Lufthansa</t>
@@ -2320,7 +2842,7 @@
     <t>de/en/discover-lufthansa/new-onboard-experience</t>
   </si>
   <si>
-    <t>2026-10-21T22:34:59.894Z</t>
+    <t>2026-10-22T00:11:22.313Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/discover-lufthansa/new-onboard-experience</t>
@@ -2380,6 +2902,21 @@
     <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/current-travel-information</t>
   </si>
   <si>
+    <t>de/en/support/feedback-and-contact-airlines.report.json</t>
+  </si>
+  <si>
+    <t>de/en/support/feedback-and-contact-airlines</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:25.366Z</t>
+  </si>
+  <si>
+    <t>Contact &amp; Feedback Hub | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/support/feedback-and-contact-airlines</t>
+  </si>
+  <si>
     <t>gb/en/fragments/payment-social.report.json</t>
   </si>
   <si>
@@ -2422,7 +2959,7 @@
     <t>de/de/100-years/history/menu-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T22:34:57.145Z</t>
+    <t>2026-10-22T00:11:24.603Z</t>
   </si>
   <si>
     <t>Menüs an Board | Lufthansa</t>
@@ -2437,7 +2974,7 @@
     <t>de/en/100-years/history/menu-on-board</t>
   </si>
   <si>
-    <t>2026-10-21T22:34:54.910Z</t>
+    <t>2026-10-22T00:11:20.013Z</t>
   </si>
   <si>
     <t>Menus on Board | Lufthansa</t>
@@ -2458,7 +2995,7 @@
     <t>insights</t>
   </si>
   <si>
-    <t>2026-10-21T22:35:13.632Z</t>
+    <t>2026-10-22T00:11:37.732Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/articles/explore-the-world/eat-see-do-berlin</t>
@@ -2812,6 +3349,51 @@
     <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/travel-classes/economy-basic</t>
   </si>
   <si>
+    <t>de/en/prepare-for-your-trip/travelling-with-children/child-in-businessclass.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/travelling-with-children/child-in-businessclass</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:15.709Z</t>
+  </si>
+  <si>
+    <t>Children in Allegris Business Class | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/travelling-with-children/child-in-businessclass</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/travelling-with-children/planning-with-kids.report.json</t>
+  </si>
+  <si>
+    <t>de/en/prepare-for-your-trip/travelling-with-children/planning-with-kids</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:42:17.565Z</t>
+  </si>
+  <si>
+    <t>Planning a trip with children | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/prepare-for-your-trip/travelling-with-children/planning-with-kids</t>
+  </si>
+  <si>
+    <t>de/en/support/contact/passenger-duty-united-kingdom.report.json</t>
+  </si>
+  <si>
+    <t>de/en/support/contact/passenger-duty-united-kingdom</t>
+  </si>
+  <si>
+    <t>2026-10-22T00:51:22.939Z</t>
+  </si>
+  <si>
+    <t>UK Air Passenger Duty (APD) | Lufthansa</t>
+  </si>
+  <si>
+    <t>https://www.lufthansa.com/de/en/support/contact/passenger-duty-united-kingdom</t>
+  </si>
+  <si>
     <t>de/en/book-and-manage/flights/ana/faq.report.json</t>
   </si>
   <si>
@@ -2974,7 +3556,7 @@
     <t>lhg/de/en/dest/cy/new-york</t>
   </si>
   <si>
-    <t>2026-10-21T22:35:49.019Z</t>
+    <t>2026-10-22T00:12:13.013Z</t>
   </si>
   <si>
     <t>Flight to New York (NYC) | Lufthansa</t>
@@ -2995,7 +3577,7 @@
     <t>aircore-route</t>
   </si>
   <si>
-    <t>2026-10-21T22:35:55.034Z</t>
+    <t>2026-10-22T00:12:17.775Z</t>
   </si>
   <si>
     <t>Flights from Germany to USA | Lufthansa</t>
@@ -3390,7 +3972,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I193"/>
+  <dimension ref="A1:I232"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
@@ -7205,7 +7787,7 @@
         <v>682</v>
       </c>
       <c r="B132" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="C132" t="s">
         <v>10</v>
@@ -7217,7 +7799,7 @@
         <v>13</v>
       </c>
       <c r="F132" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="G132" t="s">
         <v>684</v>
@@ -7234,7 +7816,7 @@
         <v>687</v>
       </c>
       <c r="B133" t="s">
-        <v>96</v>
+        <v>36</v>
       </c>
       <c r="C133" t="s">
         <v>10</v>
@@ -7246,187 +7828,187 @@
         <v>13</v>
       </c>
       <c r="F133" t="s">
-        <v>98</v>
+        <v>31</v>
       </c>
       <c r="G133" t="s">
         <v>689</v>
       </c>
       <c r="H133" t="s">
+        <v>660</v>
+      </c>
+      <c r="I133" t="s">
         <v>690</v>
-      </c>
-      <c r="I133" t="s">
-        <v>691</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
+        <v>691</v>
+      </c>
+      <c r="B134" t="s">
+        <v>36</v>
+      </c>
+      <c r="C134" t="s">
+        <v>10</v>
+      </c>
+      <c r="D134" t="s">
         <v>692</v>
       </c>
-      <c r="B134" t="s">
-        <v>36</v>
-      </c>
-      <c r="C134" t="s">
-        <v>10</v>
-      </c>
-      <c r="D134" t="s">
+      <c r="E134" t="s">
+        <v>13</v>
+      </c>
+      <c r="F134" t="s">
+        <v>31</v>
+      </c>
+      <c r="G134" t="s">
         <v>693</v>
       </c>
-      <c r="E134" t="s">
-        <v>13</v>
-      </c>
-      <c r="F134" t="s">
-        <v>98</v>
-      </c>
-      <c r="G134" t="s">
+      <c r="H134" t="s">
         <v>694</v>
       </c>
-      <c r="H134" t="s">
+      <c r="I134" t="s">
         <v>695</v>
-      </c>
-      <c r="I134" t="s">
-        <v>696</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
+        <v>696</v>
+      </c>
+      <c r="B135" t="s">
+        <v>36</v>
+      </c>
+      <c r="C135" t="s">
+        <v>10</v>
+      </c>
+      <c r="D135" t="s">
         <v>697</v>
       </c>
-      <c r="B135" t="s">
+      <c r="E135" t="s">
+        <v>13</v>
+      </c>
+      <c r="F135" t="s">
+        <v>31</v>
+      </c>
+      <c r="G135" t="s">
         <v>698</v>
       </c>
-      <c r="C135" t="s">
-        <v>10</v>
-      </c>
-      <c r="D135" t="s">
+      <c r="H135" t="s">
         <v>699</v>
       </c>
-      <c r="E135" t="s">
-        <v>13</v>
-      </c>
-      <c r="F135" t="s">
+      <c r="I135" t="s">
         <v>700</v>
-      </c>
-      <c r="G135" t="s">
-        <v>701</v>
-      </c>
-      <c r="H135" t="s">
-        <v>702</v>
-      </c>
-      <c r="I135" t="s">
-        <v>703</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
+        <v>701</v>
+      </c>
+      <c r="B136" t="s">
+        <v>36</v>
+      </c>
+      <c r="C136" t="s">
+        <v>10</v>
+      </c>
+      <c r="D136" t="s">
+        <v>702</v>
+      </c>
+      <c r="E136" t="s">
+        <v>13</v>
+      </c>
+      <c r="F136" t="s">
+        <v>31</v>
+      </c>
+      <c r="G136" t="s">
+        <v>703</v>
+      </c>
+      <c r="H136" t="s">
         <v>704</v>
       </c>
-      <c r="B136" t="s">
-        <v>36</v>
-      </c>
-      <c r="C136" t="s">
-        <v>10</v>
-      </c>
-      <c r="D136" t="s">
+      <c r="I136" t="s">
         <v>705</v>
-      </c>
-      <c r="E136" t="s">
-        <v>13</v>
-      </c>
-      <c r="F136" t="s">
-        <v>31</v>
-      </c>
-      <c r="G136" t="s">
-        <v>706</v>
-      </c>
-      <c r="H136" t="s">
-        <v>707</v>
-      </c>
-      <c r="I136" t="s">
-        <v>708</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
+        <v>706</v>
+      </c>
+      <c r="B137" t="s">
+        <v>36</v>
+      </c>
+      <c r="C137" t="s">
+        <v>10</v>
+      </c>
+      <c r="D137" t="s">
+        <v>707</v>
+      </c>
+      <c r="E137" t="s">
+        <v>13</v>
+      </c>
+      <c r="F137" t="s">
+        <v>31</v>
+      </c>
+      <c r="G137" t="s">
+        <v>708</v>
+      </c>
+      <c r="H137" t="s">
         <v>709</v>
       </c>
-      <c r="B137" t="s">
-        <v>10</v>
-      </c>
-      <c r="C137" t="s">
-        <v>11</v>
-      </c>
-      <c r="D137" t="s">
+      <c r="I137" t="s">
         <v>710</v>
-      </c>
-      <c r="E137" t="s">
-        <v>13</v>
-      </c>
-      <c r="F137" t="s">
-        <v>14</v>
-      </c>
-      <c r="G137" t="s">
-        <v>711</v>
-      </c>
-      <c r="H137" t="s">
-        <v>10</v>
-      </c>
-      <c r="I137" t="s">
-        <v>712</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
+        <v>711</v>
+      </c>
+      <c r="B138" t="s">
+        <v>354</v>
+      </c>
+      <c r="C138" t="s">
+        <v>10</v>
+      </c>
+      <c r="D138" t="s">
+        <v>712</v>
+      </c>
+      <c r="E138" t="s">
+        <v>13</v>
+      </c>
+      <c r="F138" t="s">
+        <v>31</v>
+      </c>
+      <c r="G138" t="s">
         <v>713</v>
       </c>
-      <c r="B138" t="s">
-        <v>18</v>
-      </c>
-      <c r="C138" t="s">
-        <v>10</v>
-      </c>
-      <c r="D138" t="s">
+      <c r="H138" t="s">
         <v>714</v>
       </c>
-      <c r="E138" t="s">
-        <v>13</v>
-      </c>
-      <c r="F138" t="s">
-        <v>20</v>
-      </c>
-      <c r="G138" t="s">
+      <c r="I138" t="s">
         <v>715</v>
-      </c>
-      <c r="H138" t="s">
-        <v>461</v>
-      </c>
-      <c r="I138" t="s">
-        <v>716</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
+        <v>716</v>
+      </c>
+      <c r="B139" t="s">
+        <v>84</v>
+      </c>
+      <c r="C139" t="s">
+        <v>10</v>
+      </c>
+      <c r="D139" t="s">
         <v>717</v>
       </c>
-      <c r="B139" t="s">
-        <v>10</v>
-      </c>
-      <c r="C139" t="s">
-        <v>14</v>
-      </c>
-      <c r="D139" t="s">
+      <c r="E139" t="s">
+        <v>13</v>
+      </c>
+      <c r="F139" t="s">
+        <v>31</v>
+      </c>
+      <c r="G139" t="s">
         <v>718</v>
       </c>
-      <c r="E139" t="s">
-        <v>13</v>
-      </c>
-      <c r="F139" t="s">
-        <v>14</v>
-      </c>
-      <c r="G139" t="s">
+      <c r="H139" t="s">
         <v>719</v>
-      </c>
-      <c r="H139" t="s">
-        <v>10</v>
       </c>
       <c r="I139" t="s">
         <v>720</v>
@@ -7437,286 +8019,286 @@
         <v>721</v>
       </c>
       <c r="B140" t="s">
+        <v>36</v>
+      </c>
+      <c r="C140" t="s">
+        <v>10</v>
+      </c>
+      <c r="D140" t="s">
         <v>722</v>
       </c>
-      <c r="C140" t="s">
-        <v>10</v>
-      </c>
-      <c r="D140" t="s">
+      <c r="E140" t="s">
+        <v>13</v>
+      </c>
+      <c r="F140" t="s">
+        <v>98</v>
+      </c>
+      <c r="G140" t="s">
         <v>723</v>
       </c>
-      <c r="E140" t="s">
-        <v>13</v>
-      </c>
-      <c r="F140" t="s">
+      <c r="H140" t="s">
         <v>724</v>
       </c>
-      <c r="G140" t="s">
+      <c r="I140" t="s">
         <v>725</v>
-      </c>
-      <c r="H140" t="s">
-        <v>726</v>
-      </c>
-      <c r="I140" t="s">
-        <v>727</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
+        <v>726</v>
+      </c>
+      <c r="B141" t="s">
+        <v>84</v>
+      </c>
+      <c r="C141" t="s">
+        <v>10</v>
+      </c>
+      <c r="D141" t="s">
+        <v>727</v>
+      </c>
+      <c r="E141" t="s">
+        <v>13</v>
+      </c>
+      <c r="F141" t="s">
+        <v>31</v>
+      </c>
+      <c r="G141" t="s">
         <v>728</v>
       </c>
-      <c r="B141" t="s">
-        <v>10</v>
-      </c>
-      <c r="C141" t="s">
+      <c r="H141" t="s">
         <v>729</v>
       </c>
-      <c r="D141" t="s">
+      <c r="I141" t="s">
         <v>730</v>
-      </c>
-      <c r="E141" t="s">
-        <v>13</v>
-      </c>
-      <c r="F141" t="s">
-        <v>14</v>
-      </c>
-      <c r="G141" t="s">
-        <v>731</v>
-      </c>
-      <c r="H141" t="s">
-        <v>10</v>
-      </c>
-      <c r="I141" t="s">
-        <v>732</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
+        <v>731</v>
+      </c>
+      <c r="B142" t="s">
+        <v>96</v>
+      </c>
+      <c r="C142" t="s">
+        <v>10</v>
+      </c>
+      <c r="D142" t="s">
+        <v>732</v>
+      </c>
+      <c r="E142" t="s">
+        <v>13</v>
+      </c>
+      <c r="F142" t="s">
+        <v>98</v>
+      </c>
+      <c r="G142" t="s">
         <v>733</v>
       </c>
-      <c r="B142" t="s">
+      <c r="H142" t="s">
         <v>734</v>
       </c>
-      <c r="C142" t="s">
-        <v>10</v>
-      </c>
-      <c r="D142" t="s">
+      <c r="I142" t="s">
         <v>735</v>
-      </c>
-      <c r="E142" t="s">
-        <v>13</v>
-      </c>
-      <c r="F142" t="s">
-        <v>116</v>
-      </c>
-      <c r="G142" t="s">
-        <v>736</v>
-      </c>
-      <c r="H142" t="s">
-        <v>737</v>
-      </c>
-      <c r="I142" t="s">
-        <v>738</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
+        <v>736</v>
+      </c>
+      <c r="B143" t="s">
+        <v>36</v>
+      </c>
+      <c r="C143" t="s">
+        <v>10</v>
+      </c>
+      <c r="D143" t="s">
+        <v>737</v>
+      </c>
+      <c r="E143" t="s">
+        <v>13</v>
+      </c>
+      <c r="F143" t="s">
+        <v>31</v>
+      </c>
+      <c r="G143" t="s">
+        <v>738</v>
+      </c>
+      <c r="H143" t="s">
         <v>739</v>
       </c>
-      <c r="B143" t="s">
-        <v>84</v>
-      </c>
-      <c r="C143" t="s">
-        <v>10</v>
-      </c>
-      <c r="D143" t="s">
+      <c r="I143" t="s">
         <v>740</v>
-      </c>
-      <c r="E143" t="s">
-        <v>13</v>
-      </c>
-      <c r="F143" t="s">
-        <v>31</v>
-      </c>
-      <c r="G143" t="s">
-        <v>741</v>
-      </c>
-      <c r="H143" t="s">
-        <v>742</v>
-      </c>
-      <c r="I143" t="s">
-        <v>743</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
+        <v>741</v>
+      </c>
+      <c r="B144" t="s">
+        <v>36</v>
+      </c>
+      <c r="C144" t="s">
+        <v>10</v>
+      </c>
+      <c r="D144" t="s">
+        <v>742</v>
+      </c>
+      <c r="E144" t="s">
+        <v>13</v>
+      </c>
+      <c r="F144" t="s">
+        <v>31</v>
+      </c>
+      <c r="G144" t="s">
+        <v>743</v>
+      </c>
+      <c r="H144" t="s">
         <v>744</v>
       </c>
-      <c r="B144" t="s">
-        <v>10</v>
-      </c>
-      <c r="C144" t="s">
-        <v>729</v>
-      </c>
-      <c r="D144" t="s">
+      <c r="I144" t="s">
         <v>745</v>
-      </c>
-      <c r="E144" t="s">
-        <v>13</v>
-      </c>
-      <c r="F144" t="s">
-        <v>14</v>
-      </c>
-      <c r="G144" t="s">
-        <v>746</v>
-      </c>
-      <c r="H144" t="s">
-        <v>10</v>
-      </c>
-      <c r="I144" t="s">
-        <v>747</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
+        <v>746</v>
+      </c>
+      <c r="B145" t="s">
+        <v>36</v>
+      </c>
+      <c r="C145" t="s">
+        <v>10</v>
+      </c>
+      <c r="D145" t="s">
+        <v>747</v>
+      </c>
+      <c r="E145" t="s">
+        <v>13</v>
+      </c>
+      <c r="F145" t="s">
+        <v>31</v>
+      </c>
+      <c r="G145" t="s">
         <v>748</v>
       </c>
-      <c r="B145" t="s">
-        <v>36</v>
-      </c>
-      <c r="C145" t="s">
-        <v>10</v>
-      </c>
-      <c r="D145" t="s">
+      <c r="H145" t="s">
         <v>749</v>
       </c>
-      <c r="E145" t="s">
-        <v>13</v>
-      </c>
-      <c r="F145" t="s">
-        <v>31</v>
-      </c>
-      <c r="G145" t="s">
+      <c r="I145" t="s">
         <v>750</v>
-      </c>
-      <c r="H145" t="s">
-        <v>660</v>
-      </c>
-      <c r="I145" t="s">
-        <v>751</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
+        <v>751</v>
+      </c>
+      <c r="B146" t="s">
+        <v>36</v>
+      </c>
+      <c r="C146" t="s">
+        <v>10</v>
+      </c>
+      <c r="D146" t="s">
         <v>752</v>
       </c>
-      <c r="B146" t="s">
-        <v>36</v>
-      </c>
-      <c r="C146" t="s">
-        <v>10</v>
-      </c>
-      <c r="D146" t="s">
+      <c r="E146" t="s">
+        <v>13</v>
+      </c>
+      <c r="F146" t="s">
+        <v>98</v>
+      </c>
+      <c r="G146" t="s">
         <v>753</v>
       </c>
-      <c r="E146" t="s">
-        <v>13</v>
-      </c>
-      <c r="F146" t="s">
-        <v>31</v>
-      </c>
-      <c r="G146" t="s">
+      <c r="H146" t="s">
         <v>754</v>
       </c>
-      <c r="H146" t="s">
+      <c r="I146" t="s">
         <v>755</v>
-      </c>
-      <c r="I146" t="s">
-        <v>756</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
+        <v>756</v>
+      </c>
+      <c r="B147" t="s">
+        <v>195</v>
+      </c>
+      <c r="C147" t="s">
+        <v>10</v>
+      </c>
+      <c r="D147" t="s">
         <v>757</v>
       </c>
-      <c r="B147" t="s">
-        <v>84</v>
-      </c>
-      <c r="C147" t="s">
-        <v>10</v>
-      </c>
-      <c r="D147" t="s">
+      <c r="E147" t="s">
+        <v>13</v>
+      </c>
+      <c r="F147" t="s">
+        <v>31</v>
+      </c>
+      <c r="G147" t="s">
         <v>758</v>
       </c>
-      <c r="E147" t="s">
-        <v>13</v>
-      </c>
-      <c r="F147" t="s">
-        <v>31</v>
-      </c>
-      <c r="G147" t="s">
+      <c r="H147" t="s">
         <v>759</v>
       </c>
-      <c r="H147" t="s">
+      <c r="I147" t="s">
         <v>760</v>
-      </c>
-      <c r="I147" t="s">
-        <v>761</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
+        <v>761</v>
+      </c>
+      <c r="B148" t="s">
+        <v>237</v>
+      </c>
+      <c r="C148" t="s">
+        <v>10</v>
+      </c>
+      <c r="D148" t="s">
         <v>762</v>
       </c>
-      <c r="B148" t="s">
-        <v>84</v>
-      </c>
-      <c r="C148" t="s">
-        <v>10</v>
-      </c>
-      <c r="D148" t="s">
+      <c r="E148" t="s">
+        <v>13</v>
+      </c>
+      <c r="F148" t="s">
+        <v>31</v>
+      </c>
+      <c r="G148" t="s">
         <v>763</v>
       </c>
-      <c r="E148" t="s">
-        <v>13</v>
-      </c>
-      <c r="F148" t="s">
-        <v>31</v>
-      </c>
-      <c r="G148" t="s">
+      <c r="H148" t="s">
         <v>764</v>
       </c>
-      <c r="H148" t="s">
+      <c r="I148" t="s">
         <v>765</v>
-      </c>
-      <c r="I148" t="s">
-        <v>766</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
+        <v>766</v>
+      </c>
+      <c r="B149" t="s">
+        <v>237</v>
+      </c>
+      <c r="C149" t="s">
+        <v>10</v>
+      </c>
+      <c r="D149" t="s">
         <v>767</v>
       </c>
-      <c r="B149" t="s">
-        <v>734</v>
-      </c>
-      <c r="C149" t="s">
-        <v>10</v>
-      </c>
-      <c r="D149" t="s">
+      <c r="E149" t="s">
+        <v>13</v>
+      </c>
+      <c r="F149" t="s">
+        <v>31</v>
+      </c>
+      <c r="G149" t="s">
         <v>768</v>
       </c>
-      <c r="E149" t="s">
-        <v>13</v>
-      </c>
-      <c r="F149" t="s">
-        <v>116</v>
-      </c>
-      <c r="G149" t="s">
+      <c r="H149" t="s">
         <v>769</v>
-      </c>
-      <c r="H149" t="s">
-        <v>737</v>
       </c>
       <c r="I149" t="s">
         <v>770</v>
@@ -7727,42 +8309,42 @@
         <v>771</v>
       </c>
       <c r="B150" t="s">
-        <v>36</v>
+        <v>772</v>
       </c>
       <c r="C150" t="s">
         <v>10</v>
       </c>
       <c r="D150" t="s">
-        <v>772</v>
+        <v>773</v>
       </c>
       <c r="E150" t="s">
         <v>13</v>
       </c>
       <c r="F150" t="s">
-        <v>31</v>
+        <v>774</v>
       </c>
       <c r="G150" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="H150" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="I150" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="B151" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="C151" t="s">
         <v>10</v>
       </c>
       <c r="D151" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="E151" t="s">
         <v>13</v>
@@ -7771,56 +8353,56 @@
         <v>31</v>
       </c>
       <c r="G151" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="H151" t="s">
-        <v>742</v>
+        <v>781</v>
       </c>
       <c r="I151" t="s">
-        <v>779</v>
+        <v>782</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>780</v>
+        <v>783</v>
       </c>
       <c r="B152" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="C152" t="s">
-        <v>729</v>
+        <v>10</v>
       </c>
       <c r="D152" t="s">
-        <v>781</v>
+        <v>784</v>
       </c>
       <c r="E152" t="s">
         <v>13</v>
       </c>
       <c r="F152" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G152" t="s">
-        <v>782</v>
+        <v>785</v>
       </c>
       <c r="H152" t="s">
-        <v>10</v>
+        <v>786</v>
       </c>
       <c r="I152" t="s">
-        <v>783</v>
+        <v>787</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>784</v>
+        <v>788</v>
       </c>
       <c r="B153" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="C153" t="s">
         <v>10</v>
       </c>
       <c r="D153" t="s">
-        <v>785</v>
+        <v>789</v>
       </c>
       <c r="E153" t="s">
         <v>13</v>
@@ -7829,172 +8411,172 @@
         <v>31</v>
       </c>
       <c r="G153" t="s">
-        <v>786</v>
+        <v>790</v>
       </c>
       <c r="H153" t="s">
-        <v>787</v>
+        <v>791</v>
       </c>
       <c r="I153" t="s">
-        <v>788</v>
+        <v>792</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>789</v>
+        <v>793</v>
       </c>
       <c r="B154" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="C154" t="s">
-        <v>729</v>
+        <v>10</v>
       </c>
       <c r="D154" t="s">
-        <v>790</v>
+        <v>794</v>
       </c>
       <c r="E154" t="s">
         <v>13</v>
       </c>
       <c r="F154" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G154" t="s">
-        <v>791</v>
+        <v>795</v>
       </c>
       <c r="H154" t="s">
-        <v>10</v>
+        <v>796</v>
       </c>
       <c r="I154" t="s">
-        <v>792</v>
+        <v>797</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>793</v>
+        <v>798</v>
       </c>
       <c r="B155" t="s">
-        <v>794</v>
+        <v>237</v>
       </c>
       <c r="C155" t="s">
         <v>10</v>
       </c>
       <c r="D155" t="s">
-        <v>795</v>
+        <v>799</v>
       </c>
       <c r="E155" t="s">
         <v>13</v>
       </c>
       <c r="F155" t="s">
-        <v>796</v>
+        <v>31</v>
       </c>
       <c r="G155" t="s">
-        <v>797</v>
+        <v>800</v>
       </c>
       <c r="H155" t="s">
-        <v>798</v>
+        <v>801</v>
       </c>
       <c r="I155" t="s">
-        <v>799</v>
+        <v>802</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>800</v>
+        <v>803</v>
       </c>
       <c r="B156" t="s">
-        <v>801</v>
+        <v>36</v>
       </c>
       <c r="C156" t="s">
         <v>10</v>
       </c>
       <c r="D156" t="s">
-        <v>802</v>
+        <v>804</v>
       </c>
       <c r="E156" t="s">
         <v>13</v>
       </c>
       <c r="F156" t="s">
-        <v>116</v>
+        <v>31</v>
       </c>
       <c r="G156" t="s">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="H156" t="s">
-        <v>804</v>
+        <v>806</v>
       </c>
       <c r="I156" t="s">
-        <v>805</v>
+        <v>807</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>806</v>
+        <v>808</v>
       </c>
       <c r="B157" t="s">
-        <v>801</v>
+        <v>36</v>
       </c>
       <c r="C157" t="s">
         <v>10</v>
       </c>
       <c r="D157" t="s">
-        <v>807</v>
+        <v>809</v>
       </c>
       <c r="E157" t="s">
         <v>13</v>
       </c>
       <c r="F157" t="s">
-        <v>116</v>
+        <v>31</v>
       </c>
       <c r="G157" t="s">
-        <v>808</v>
+        <v>810</v>
       </c>
       <c r="H157" t="s">
-        <v>809</v>
+        <v>811</v>
       </c>
       <c r="I157" t="s">
-        <v>810</v>
+        <v>812</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>811</v>
+        <v>813</v>
       </c>
       <c r="B158" t="s">
-        <v>812</v>
+        <v>36</v>
       </c>
       <c r="C158" t="s">
         <v>10</v>
       </c>
       <c r="D158" t="s">
-        <v>813</v>
+        <v>814</v>
       </c>
       <c r="E158" t="s">
         <v>13</v>
       </c>
       <c r="F158" t="s">
-        <v>814</v>
+        <v>31</v>
       </c>
       <c r="G158" t="s">
         <v>815</v>
       </c>
       <c r="H158" t="s">
-        <v>10</v>
+        <v>816</v>
       </c>
       <c r="I158" t="s">
-        <v>816</v>
+        <v>817</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>817</v>
+        <v>818</v>
       </c>
       <c r="B159" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="C159" t="s">
         <v>10</v>
       </c>
       <c r="D159" t="s">
-        <v>818</v>
+        <v>819</v>
       </c>
       <c r="E159" t="s">
         <v>13</v>
@@ -8003,27 +8585,27 @@
         <v>31</v>
       </c>
       <c r="G159" t="s">
-        <v>819</v>
+        <v>820</v>
       </c>
       <c r="H159" t="s">
-        <v>820</v>
+        <v>821</v>
       </c>
       <c r="I159" t="s">
-        <v>821</v>
+        <v>822</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>822</v>
+        <v>823</v>
       </c>
       <c r="B160" t="s">
-        <v>90</v>
+        <v>36</v>
       </c>
       <c r="C160" t="s">
         <v>10</v>
       </c>
       <c r="D160" t="s">
-        <v>823</v>
+        <v>824</v>
       </c>
       <c r="E160" t="s">
         <v>13</v>
@@ -8032,18 +8614,18 @@
         <v>31</v>
       </c>
       <c r="G160" t="s">
-        <v>824</v>
+        <v>825</v>
       </c>
       <c r="H160" t="s">
-        <v>825</v>
+        <v>826</v>
       </c>
       <c r="I160" t="s">
-        <v>826</v>
+        <v>827</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>827</v>
+        <v>828</v>
       </c>
       <c r="B161" t="s">
         <v>36</v>
@@ -8052,7 +8634,7 @@
         <v>10</v>
       </c>
       <c r="D161" t="s">
-        <v>828</v>
+        <v>829</v>
       </c>
       <c r="E161" t="s">
         <v>13</v>
@@ -8061,27 +8643,27 @@
         <v>31</v>
       </c>
       <c r="G161" t="s">
-        <v>829</v>
+        <v>830</v>
       </c>
       <c r="H161" t="s">
-        <v>830</v>
+        <v>831</v>
       </c>
       <c r="I161" t="s">
-        <v>831</v>
+        <v>832</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>832</v>
+        <v>833</v>
       </c>
       <c r="B162" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="C162" t="s">
         <v>10</v>
       </c>
       <c r="D162" t="s">
-        <v>833</v>
+        <v>834</v>
       </c>
       <c r="E162" t="s">
         <v>13</v>
@@ -8090,18 +8672,18 @@
         <v>31</v>
       </c>
       <c r="G162" t="s">
-        <v>834</v>
+        <v>835</v>
       </c>
       <c r="H162" t="s">
-        <v>835</v>
+        <v>836</v>
       </c>
       <c r="I162" t="s">
-        <v>836</v>
+        <v>837</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="B163" t="s">
         <v>84</v>
@@ -8110,7 +8692,7 @@
         <v>10</v>
       </c>
       <c r="D163" t="s">
-        <v>838</v>
+        <v>839</v>
       </c>
       <c r="E163" t="s">
         <v>13</v>
@@ -8119,21 +8701,21 @@
         <v>31</v>
       </c>
       <c r="G163" t="s">
-        <v>839</v>
+        <v>840</v>
       </c>
       <c r="H163" t="s">
-        <v>840</v>
+        <v>841</v>
       </c>
       <c r="I163" t="s">
-        <v>841</v>
+        <v>842</v>
       </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>842</v>
+        <v>843</v>
       </c>
       <c r="B164" t="s">
-        <v>843</v>
+        <v>36</v>
       </c>
       <c r="C164" t="s">
         <v>10</v>
@@ -8162,7 +8744,7 @@
         <v>848</v>
       </c>
       <c r="B165" t="s">
-        <v>84</v>
+        <v>36</v>
       </c>
       <c r="C165" t="s">
         <v>10</v>
@@ -8220,7 +8802,7 @@
         <v>858</v>
       </c>
       <c r="B167" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="C167" t="s">
         <v>10</v>
@@ -8307,7 +8889,7 @@
         <v>873</v>
       </c>
       <c r="B170" t="s">
-        <v>237</v>
+        <v>36</v>
       </c>
       <c r="C170" t="s">
         <v>10</v>
@@ -8336,7 +8918,7 @@
         <v>878</v>
       </c>
       <c r="B171" t="s">
-        <v>195</v>
+        <v>36</v>
       </c>
       <c r="C171" t="s">
         <v>10</v>
@@ -8365,10 +8947,10 @@
         <v>883</v>
       </c>
       <c r="B172" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="C172" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D172" t="s">
         <v>884</v>
@@ -8377,114 +8959,114 @@
         <v>13</v>
       </c>
       <c r="F172" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G172" t="s">
         <v>885</v>
       </c>
       <c r="H172" t="s">
+        <v>10</v>
+      </c>
+      <c r="I172" t="s">
         <v>886</v>
-      </c>
-      <c r="I172" t="s">
-        <v>887</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
+        <v>887</v>
+      </c>
+      <c r="B173" t="s">
+        <v>18</v>
+      </c>
+      <c r="C173" t="s">
+        <v>10</v>
+      </c>
+      <c r="D173" t="s">
         <v>888</v>
       </c>
-      <c r="B173" t="s">
-        <v>84</v>
-      </c>
-      <c r="C173" t="s">
-        <v>10</v>
-      </c>
-      <c r="D173" t="s">
+      <c r="E173" t="s">
+        <v>13</v>
+      </c>
+      <c r="F173" t="s">
+        <v>20</v>
+      </c>
+      <c r="G173" t="s">
         <v>889</v>
       </c>
-      <c r="E173" t="s">
-        <v>13</v>
-      </c>
-      <c r="F173" t="s">
-        <v>31</v>
-      </c>
-      <c r="G173" t="s">
+      <c r="H173" t="s">
+        <v>461</v>
+      </c>
+      <c r="I173" t="s">
         <v>890</v>
-      </c>
-      <c r="H173" t="s">
-        <v>891</v>
-      </c>
-      <c r="I173" t="s">
-        <v>892</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
+        <v>891</v>
+      </c>
+      <c r="B174" t="s">
+        <v>10</v>
+      </c>
+      <c r="C174" t="s">
+        <v>14</v>
+      </c>
+      <c r="D174" t="s">
+        <v>892</v>
+      </c>
+      <c r="E174" t="s">
+        <v>13</v>
+      </c>
+      <c r="F174" t="s">
+        <v>14</v>
+      </c>
+      <c r="G174" t="s">
         <v>893</v>
       </c>
-      <c r="B174" t="s">
-        <v>36</v>
-      </c>
-      <c r="C174" t="s">
-        <v>10</v>
-      </c>
-      <c r="D174" t="s">
+      <c r="H174" t="s">
+        <v>10</v>
+      </c>
+      <c r="I174" t="s">
         <v>894</v>
-      </c>
-      <c r="E174" t="s">
-        <v>13</v>
-      </c>
-      <c r="F174" t="s">
-        <v>31</v>
-      </c>
-      <c r="G174" t="s">
-        <v>895</v>
-      </c>
-      <c r="H174" t="s">
-        <v>896</v>
-      </c>
-      <c r="I174" t="s">
-        <v>897</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
+        <v>895</v>
+      </c>
+      <c r="B175" t="s">
+        <v>896</v>
+      </c>
+      <c r="C175" t="s">
+        <v>10</v>
+      </c>
+      <c r="D175" t="s">
+        <v>897</v>
+      </c>
+      <c r="E175" t="s">
+        <v>13</v>
+      </c>
+      <c r="F175" t="s">
         <v>898</v>
       </c>
-      <c r="B175" t="s">
-        <v>84</v>
-      </c>
-      <c r="C175" t="s">
-        <v>10</v>
-      </c>
-      <c r="D175" t="s">
+      <c r="G175" t="s">
         <v>899</v>
       </c>
-      <c r="E175" t="s">
-        <v>13</v>
-      </c>
-      <c r="F175" t="s">
-        <v>31</v>
-      </c>
-      <c r="G175" t="s">
+      <c r="H175" t="s">
         <v>900</v>
       </c>
-      <c r="H175" t="s">
+      <c r="I175" t="s">
         <v>901</v>
-      </c>
-      <c r="I175" t="s">
-        <v>902</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
+        <v>902</v>
+      </c>
+      <c r="B176" t="s">
+        <v>10</v>
+      </c>
+      <c r="C176" t="s">
         <v>903</v>
-      </c>
-      <c r="B176" t="s">
-        <v>29</v>
-      </c>
-      <c r="C176" t="s">
-        <v>10</v>
       </c>
       <c r="D176" t="s">
         <v>904</v>
@@ -8493,24 +9075,24 @@
         <v>13</v>
       </c>
       <c r="F176" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G176" t="s">
         <v>905</v>
       </c>
       <c r="H176" t="s">
+        <v>10</v>
+      </c>
+      <c r="I176" t="s">
         <v>906</v>
-      </c>
-      <c r="I176" t="s">
-        <v>907</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
+        <v>907</v>
+      </c>
+      <c r="B177" t="s">
         <v>908</v>
-      </c>
-      <c r="B177" t="s">
-        <v>36</v>
       </c>
       <c r="C177" t="s">
         <v>10</v>
@@ -8522,7 +9104,7 @@
         <v>13</v>
       </c>
       <c r="F177" t="s">
-        <v>31</v>
+        <v>116</v>
       </c>
       <c r="G177" t="s">
         <v>910</v>
@@ -8539,7 +9121,7 @@
         <v>913</v>
       </c>
       <c r="B178" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="C178" t="s">
         <v>10</v>
@@ -8568,10 +9150,10 @@
         <v>918</v>
       </c>
       <c r="B179" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="C179" t="s">
-        <v>10</v>
+        <v>903</v>
       </c>
       <c r="D179" t="s">
         <v>919</v>
@@ -8580,108 +9162,108 @@
         <v>13</v>
       </c>
       <c r="F179" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G179" t="s">
         <v>920</v>
       </c>
       <c r="H179" t="s">
+        <v>10</v>
+      </c>
+      <c r="I179" t="s">
         <v>921</v>
-      </c>
-      <c r="I179" t="s">
-        <v>922</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
+        <v>922</v>
+      </c>
+      <c r="B180" t="s">
+        <v>36</v>
+      </c>
+      <c r="C180" t="s">
+        <v>10</v>
+      </c>
+      <c r="D180" t="s">
         <v>923</v>
       </c>
-      <c r="B180" t="s">
-        <v>90</v>
-      </c>
-      <c r="C180" t="s">
-        <v>10</v>
-      </c>
-      <c r="D180" t="s">
+      <c r="E180" t="s">
+        <v>13</v>
+      </c>
+      <c r="F180" t="s">
+        <v>31</v>
+      </c>
+      <c r="G180" t="s">
         <v>924</v>
       </c>
-      <c r="E180" t="s">
-        <v>13</v>
-      </c>
-      <c r="F180" t="s">
-        <v>31</v>
-      </c>
-      <c r="G180" t="s">
+      <c r="H180" t="s">
+        <v>660</v>
+      </c>
+      <c r="I180" t="s">
         <v>925</v>
-      </c>
-      <c r="H180" t="s">
-        <v>926</v>
-      </c>
-      <c r="I180" t="s">
-        <v>927</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
+        <v>926</v>
+      </c>
+      <c r="B181" t="s">
+        <v>36</v>
+      </c>
+      <c r="C181" t="s">
+        <v>10</v>
+      </c>
+      <c r="D181" t="s">
+        <v>927</v>
+      </c>
+      <c r="E181" t="s">
+        <v>13</v>
+      </c>
+      <c r="F181" t="s">
+        <v>31</v>
+      </c>
+      <c r="G181" t="s">
         <v>928</v>
       </c>
-      <c r="B181" t="s">
-        <v>84</v>
-      </c>
-      <c r="C181" t="s">
-        <v>10</v>
-      </c>
-      <c r="D181" t="s">
+      <c r="H181" t="s">
         <v>929</v>
       </c>
-      <c r="E181" t="s">
-        <v>13</v>
-      </c>
-      <c r="F181" t="s">
-        <v>31</v>
-      </c>
-      <c r="G181" t="s">
+      <c r="I181" t="s">
         <v>930</v>
-      </c>
-      <c r="H181" t="s">
-        <v>931</v>
-      </c>
-      <c r="I181" t="s">
-        <v>932</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
+        <v>931</v>
+      </c>
+      <c r="B182" t="s">
+        <v>84</v>
+      </c>
+      <c r="C182" t="s">
+        <v>10</v>
+      </c>
+      <c r="D182" t="s">
+        <v>932</v>
+      </c>
+      <c r="E182" t="s">
+        <v>13</v>
+      </c>
+      <c r="F182" t="s">
+        <v>31</v>
+      </c>
+      <c r="G182" t="s">
         <v>933</v>
       </c>
-      <c r="B182" t="s">
+      <c r="H182" t="s">
         <v>934</v>
       </c>
-      <c r="C182" t="s">
-        <v>10</v>
-      </c>
-      <c r="D182" t="s">
+      <c r="I182" t="s">
         <v>935</v>
-      </c>
-      <c r="E182" t="s">
-        <v>13</v>
-      </c>
-      <c r="F182" t="s">
-        <v>31</v>
-      </c>
-      <c r="G182" t="s">
-        <v>936</v>
-      </c>
-      <c r="H182" t="s">
-        <v>937</v>
-      </c>
-      <c r="I182" t="s">
-        <v>938</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
-        <v>939</v>
+        <v>936</v>
       </c>
       <c r="B183" t="s">
         <v>84</v>
@@ -8690,94 +9272,94 @@
         <v>10</v>
       </c>
       <c r="D183" t="s">
+        <v>937</v>
+      </c>
+      <c r="E183" t="s">
+        <v>13</v>
+      </c>
+      <c r="F183" t="s">
+        <v>31</v>
+      </c>
+      <c r="G183" t="s">
+        <v>938</v>
+      </c>
+      <c r="H183" t="s">
+        <v>939</v>
+      </c>
+      <c r="I183" t="s">
         <v>940</v>
-      </c>
-      <c r="E183" t="s">
-        <v>13</v>
-      </c>
-      <c r="F183" t="s">
-        <v>31</v>
-      </c>
-      <c r="G183" t="s">
-        <v>941</v>
-      </c>
-      <c r="H183" t="s">
-        <v>942</v>
-      </c>
-      <c r="I183" t="s">
-        <v>943</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
+        <v>941</v>
+      </c>
+      <c r="B184" t="s">
+        <v>908</v>
+      </c>
+      <c r="C184" t="s">
+        <v>10</v>
+      </c>
+      <c r="D184" t="s">
+        <v>942</v>
+      </c>
+      <c r="E184" t="s">
+        <v>13</v>
+      </c>
+      <c r="F184" t="s">
+        <v>116</v>
+      </c>
+      <c r="G184" t="s">
+        <v>943</v>
+      </c>
+      <c r="H184" t="s">
+        <v>911</v>
+      </c>
+      <c r="I184" t="s">
         <v>944</v>
-      </c>
-      <c r="B184" t="s">
-        <v>36</v>
-      </c>
-      <c r="C184" t="s">
-        <v>10</v>
-      </c>
-      <c r="D184" t="s">
-        <v>945</v>
-      </c>
-      <c r="E184" t="s">
-        <v>13</v>
-      </c>
-      <c r="F184" t="s">
-        <v>31</v>
-      </c>
-      <c r="G184" t="s">
-        <v>946</v>
-      </c>
-      <c r="H184" t="s">
-        <v>947</v>
-      </c>
-      <c r="I184" t="s">
-        <v>948</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
+        <v>945</v>
+      </c>
+      <c r="B185" t="s">
+        <v>36</v>
+      </c>
+      <c r="C185" t="s">
+        <v>10</v>
+      </c>
+      <c r="D185" t="s">
+        <v>946</v>
+      </c>
+      <c r="E185" t="s">
+        <v>13</v>
+      </c>
+      <c r="F185" t="s">
+        <v>31</v>
+      </c>
+      <c r="G185" t="s">
+        <v>947</v>
+      </c>
+      <c r="H185" t="s">
+        <v>948</v>
+      </c>
+      <c r="I185" t="s">
         <v>949</v>
-      </c>
-      <c r="B185" t="s">
-        <v>934</v>
-      </c>
-      <c r="C185" t="s">
-        <v>10</v>
-      </c>
-      <c r="D185" t="s">
-        <v>950</v>
-      </c>
-      <c r="E185" t="s">
-        <v>13</v>
-      </c>
-      <c r="F185" t="s">
-        <v>31</v>
-      </c>
-      <c r="G185" t="s">
-        <v>951</v>
-      </c>
-      <c r="H185" t="s">
-        <v>952</v>
-      </c>
-      <c r="I185" t="s">
-        <v>953</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
-        <v>954</v>
+        <v>950</v>
       </c>
       <c r="B186" t="s">
-        <v>195</v>
+        <v>84</v>
       </c>
       <c r="C186" t="s">
         <v>10</v>
       </c>
       <c r="D186" t="s">
-        <v>955</v>
+        <v>951</v>
       </c>
       <c r="E186" t="s">
         <v>13</v>
@@ -8786,56 +9368,56 @@
         <v>31</v>
       </c>
       <c r="G186" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
       <c r="H186" t="s">
-        <v>957</v>
+        <v>916</v>
       </c>
       <c r="I186" t="s">
-        <v>958</v>
+        <v>953</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
-        <v>959</v>
+        <v>954</v>
       </c>
       <c r="B187" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="C187" t="s">
-        <v>10</v>
+        <v>903</v>
       </c>
       <c r="D187" t="s">
-        <v>960</v>
+        <v>955</v>
       </c>
       <c r="E187" t="s">
         <v>13</v>
       </c>
       <c r="F187" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G187" t="s">
-        <v>961</v>
+        <v>956</v>
       </c>
       <c r="H187" t="s">
-        <v>962</v>
+        <v>10</v>
       </c>
       <c r="I187" t="s">
-        <v>963</v>
+        <v>957</v>
       </c>
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
-        <v>964</v>
+        <v>958</v>
       </c>
       <c r="B188" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="C188" t="s">
         <v>10</v>
       </c>
       <c r="D188" t="s">
-        <v>965</v>
+        <v>959</v>
       </c>
       <c r="E188" t="s">
         <v>13</v>
@@ -8844,18 +9426,18 @@
         <v>31</v>
       </c>
       <c r="G188" t="s">
-        <v>966</v>
+        <v>960</v>
       </c>
       <c r="H188" t="s">
-        <v>967</v>
+        <v>961</v>
       </c>
       <c r="I188" t="s">
-        <v>968</v>
+        <v>962</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
-        <v>969</v>
+        <v>963</v>
       </c>
       <c r="B189" t="s">
         <v>36</v>
@@ -8864,7 +9446,7 @@
         <v>10</v>
       </c>
       <c r="D189" t="s">
-        <v>970</v>
+        <v>964</v>
       </c>
       <c r="E189" t="s">
         <v>13</v>
@@ -8873,129 +9455,1260 @@
         <v>31</v>
       </c>
       <c r="G189" t="s">
-        <v>971</v>
+        <v>965</v>
       </c>
       <c r="H189" t="s">
-        <v>972</v>
+        <v>966</v>
       </c>
       <c r="I189" t="s">
-        <v>973</v>
+        <v>967</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
-        <v>974</v>
+        <v>968</v>
       </c>
       <c r="B190" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="C190" t="s">
-        <v>10</v>
+        <v>903</v>
       </c>
       <c r="D190" t="s">
-        <v>975</v>
+        <v>969</v>
       </c>
       <c r="E190" t="s">
         <v>13</v>
       </c>
       <c r="F190" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G190" t="s">
-        <v>976</v>
+        <v>970</v>
       </c>
       <c r="H190" t="s">
-        <v>977</v>
+        <v>10</v>
       </c>
       <c r="I190" t="s">
-        <v>978</v>
+        <v>971</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
-        <v>979</v>
+        <v>972</v>
       </c>
       <c r="B191" t="s">
-        <v>36</v>
+        <v>973</v>
       </c>
       <c r="C191" t="s">
         <v>10</v>
       </c>
       <c r="D191" t="s">
-        <v>980</v>
+        <v>974</v>
       </c>
       <c r="E191" t="s">
         <v>13</v>
       </c>
       <c r="F191" t="s">
-        <v>31</v>
+        <v>975</v>
       </c>
       <c r="G191" t="s">
-        <v>981</v>
+        <v>976</v>
       </c>
       <c r="H191" t="s">
-        <v>982</v>
+        <v>977</v>
       </c>
       <c r="I191" t="s">
-        <v>983</v>
+        <v>978</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
+        <v>979</v>
+      </c>
+      <c r="B192" t="s">
+        <v>980</v>
+      </c>
+      <c r="C192" t="s">
+        <v>10</v>
+      </c>
+      <c r="D192" t="s">
+        <v>981</v>
+      </c>
+      <c r="E192" t="s">
+        <v>13</v>
+      </c>
+      <c r="F192" t="s">
+        <v>116</v>
+      </c>
+      <c r="G192" t="s">
+        <v>982</v>
+      </c>
+      <c r="H192" t="s">
+        <v>983</v>
+      </c>
+      <c r="I192" t="s">
         <v>984</v>
-      </c>
-      <c r="B192" t="s">
-        <v>985</v>
-      </c>
-      <c r="C192" t="s">
-        <v>10</v>
-      </c>
-      <c r="D192" t="s">
-        <v>986</v>
-      </c>
-      <c r="E192" t="s">
-        <v>13</v>
-      </c>
-      <c r="F192" t="s">
-        <v>796</v>
-      </c>
-      <c r="G192" t="s">
-        <v>987</v>
-      </c>
-      <c r="H192" t="s">
-        <v>988</v>
-      </c>
-      <c r="I192" t="s">
-        <v>989</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
+        <v>985</v>
+      </c>
+      <c r="B193" t="s">
+        <v>980</v>
+      </c>
+      <c r="C193" t="s">
+        <v>10</v>
+      </c>
+      <c r="D193" t="s">
+        <v>986</v>
+      </c>
+      <c r="E193" t="s">
+        <v>13</v>
+      </c>
+      <c r="F193" t="s">
+        <v>116</v>
+      </c>
+      <c r="G193" t="s">
+        <v>987</v>
+      </c>
+      <c r="H193" t="s">
+        <v>988</v>
+      </c>
+      <c r="I193" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
         <v>990</v>
       </c>
-      <c r="B193" t="s">
+      <c r="B194" t="s">
         <v>991</v>
       </c>
-      <c r="C193" t="s">
-        <v>10</v>
-      </c>
-      <c r="D193" t="s">
+      <c r="C194" t="s">
+        <v>10</v>
+      </c>
+      <c r="D194" t="s">
         <v>992</v>
       </c>
-      <c r="E193" t="s">
-        <v>13</v>
-      </c>
-      <c r="F193" t="s">
+      <c r="E194" t="s">
+        <v>13</v>
+      </c>
+      <c r="F194" t="s">
         <v>993</v>
       </c>
-      <c r="G193" t="s">
+      <c r="G194" t="s">
         <v>994</v>
       </c>
-      <c r="H193" t="s">
+      <c r="H194" t="s">
+        <v>10</v>
+      </c>
+      <c r="I194" t="s">
         <v>995</v>
       </c>
-      <c r="I193" t="s">
+    </row>
+    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
         <v>996</v>
+      </c>
+      <c r="B195" t="s">
+        <v>36</v>
+      </c>
+      <c r="C195" t="s">
+        <v>10</v>
+      </c>
+      <c r="D195" t="s">
+        <v>997</v>
+      </c>
+      <c r="E195" t="s">
+        <v>13</v>
+      </c>
+      <c r="F195" t="s">
+        <v>31</v>
+      </c>
+      <c r="G195" t="s">
+        <v>998</v>
+      </c>
+      <c r="H195" t="s">
+        <v>999</v>
+      </c>
+      <c r="I195" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B196" t="s">
+        <v>90</v>
+      </c>
+      <c r="C196" t="s">
+        <v>10</v>
+      </c>
+      <c r="D196" t="s">
+        <v>1002</v>
+      </c>
+      <c r="E196" t="s">
+        <v>13</v>
+      </c>
+      <c r="F196" t="s">
+        <v>31</v>
+      </c>
+      <c r="G196" t="s">
+        <v>1003</v>
+      </c>
+      <c r="H196" t="s">
+        <v>1004</v>
+      </c>
+      <c r="I196" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>1006</v>
+      </c>
+      <c r="B197" t="s">
+        <v>36</v>
+      </c>
+      <c r="C197" t="s">
+        <v>10</v>
+      </c>
+      <c r="D197" t="s">
+        <v>1007</v>
+      </c>
+      <c r="E197" t="s">
+        <v>13</v>
+      </c>
+      <c r="F197" t="s">
+        <v>31</v>
+      </c>
+      <c r="G197" t="s">
+        <v>1008</v>
+      </c>
+      <c r="H197" t="s">
+        <v>1009</v>
+      </c>
+      <c r="I197" t="s">
+        <v>1010</v>
+      </c>
+    </row>
+    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>1011</v>
+      </c>
+      <c r="B198" t="s">
+        <v>36</v>
+      </c>
+      <c r="C198" t="s">
+        <v>10</v>
+      </c>
+      <c r="D198" t="s">
+        <v>1012</v>
+      </c>
+      <c r="E198" t="s">
+        <v>13</v>
+      </c>
+      <c r="F198" t="s">
+        <v>31</v>
+      </c>
+      <c r="G198" t="s">
+        <v>1013</v>
+      </c>
+      <c r="H198" t="s">
+        <v>1014</v>
+      </c>
+      <c r="I198" t="s">
+        <v>1015</v>
+      </c>
+    </row>
+    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B199" t="s">
+        <v>84</v>
+      </c>
+      <c r="C199" t="s">
+        <v>10</v>
+      </c>
+      <c r="D199" t="s">
+        <v>1017</v>
+      </c>
+      <c r="E199" t="s">
+        <v>13</v>
+      </c>
+      <c r="F199" t="s">
+        <v>31</v>
+      </c>
+      <c r="G199" t="s">
+        <v>1018</v>
+      </c>
+      <c r="H199" t="s">
+        <v>1019</v>
+      </c>
+      <c r="I199" t="s">
+        <v>1020</v>
+      </c>
+    </row>
+    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B200" t="s">
+        <v>1022</v>
+      </c>
+      <c r="C200" t="s">
+        <v>10</v>
+      </c>
+      <c r="D200" t="s">
+        <v>1023</v>
+      </c>
+      <c r="E200" t="s">
+        <v>13</v>
+      </c>
+      <c r="F200" t="s">
+        <v>31</v>
+      </c>
+      <c r="G200" t="s">
+        <v>1024</v>
+      </c>
+      <c r="H200" t="s">
+        <v>1025</v>
+      </c>
+      <c r="I200" t="s">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B201" t="s">
+        <v>84</v>
+      </c>
+      <c r="C201" t="s">
+        <v>10</v>
+      </c>
+      <c r="D201" t="s">
+        <v>1028</v>
+      </c>
+      <c r="E201" t="s">
+        <v>13</v>
+      </c>
+      <c r="F201" t="s">
+        <v>31</v>
+      </c>
+      <c r="G201" t="s">
+        <v>1029</v>
+      </c>
+      <c r="H201" t="s">
+        <v>1030</v>
+      </c>
+      <c r="I201" t="s">
+        <v>1031</v>
+      </c>
+    </row>
+    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B202" t="s">
+        <v>84</v>
+      </c>
+      <c r="C202" t="s">
+        <v>10</v>
+      </c>
+      <c r="D202" t="s">
+        <v>1033</v>
+      </c>
+      <c r="E202" t="s">
+        <v>13</v>
+      </c>
+      <c r="F202" t="s">
+        <v>31</v>
+      </c>
+      <c r="G202" t="s">
+        <v>1034</v>
+      </c>
+      <c r="H202" t="s">
+        <v>1035</v>
+      </c>
+      <c r="I202" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B203" t="s">
+        <v>36</v>
+      </c>
+      <c r="C203" t="s">
+        <v>10</v>
+      </c>
+      <c r="D203" t="s">
+        <v>1038</v>
+      </c>
+      <c r="E203" t="s">
+        <v>13</v>
+      </c>
+      <c r="F203" t="s">
+        <v>31</v>
+      </c>
+      <c r="G203" t="s">
+        <v>1039</v>
+      </c>
+      <c r="H203" t="s">
+        <v>1040</v>
+      </c>
+      <c r="I203" t="s">
+        <v>1041</v>
+      </c>
+    </row>
+    <row r="204" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>1042</v>
+      </c>
+      <c r="B204" t="s">
+        <v>36</v>
+      </c>
+      <c r="C204" t="s">
+        <v>10</v>
+      </c>
+      <c r="D204" t="s">
+        <v>1043</v>
+      </c>
+      <c r="E204" t="s">
+        <v>13</v>
+      </c>
+      <c r="F204" t="s">
+        <v>31</v>
+      </c>
+      <c r="G204" t="s">
+        <v>1044</v>
+      </c>
+      <c r="H204" t="s">
+        <v>1045</v>
+      </c>
+      <c r="I204" t="s">
+        <v>1046</v>
+      </c>
+    </row>
+    <row r="205" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>1047</v>
+      </c>
+      <c r="B205" t="s">
+        <v>84</v>
+      </c>
+      <c r="C205" t="s">
+        <v>10</v>
+      </c>
+      <c r="D205" t="s">
+        <v>1048</v>
+      </c>
+      <c r="E205" t="s">
+        <v>13</v>
+      </c>
+      <c r="F205" t="s">
+        <v>31</v>
+      </c>
+      <c r="G205" t="s">
+        <v>1049</v>
+      </c>
+      <c r="H205" t="s">
+        <v>1050</v>
+      </c>
+      <c r="I205" t="s">
+        <v>1051</v>
+      </c>
+    </row>
+    <row r="206" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>1052</v>
+      </c>
+      <c r="B206" t="s">
+        <v>237</v>
+      </c>
+      <c r="C206" t="s">
+        <v>10</v>
+      </c>
+      <c r="D206" t="s">
+        <v>1053</v>
+      </c>
+      <c r="E206" t="s">
+        <v>13</v>
+      </c>
+      <c r="F206" t="s">
+        <v>31</v>
+      </c>
+      <c r="G206" t="s">
+        <v>1054</v>
+      </c>
+      <c r="H206" t="s">
+        <v>1055</v>
+      </c>
+      <c r="I206" t="s">
+        <v>1056</v>
+      </c>
+    </row>
+    <row r="207" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>1057</v>
+      </c>
+      <c r="B207" t="s">
+        <v>195</v>
+      </c>
+      <c r="C207" t="s">
+        <v>10</v>
+      </c>
+      <c r="D207" t="s">
+        <v>1058</v>
+      </c>
+      <c r="E207" t="s">
+        <v>13</v>
+      </c>
+      <c r="F207" t="s">
+        <v>31</v>
+      </c>
+      <c r="G207" t="s">
+        <v>1059</v>
+      </c>
+      <c r="H207" t="s">
+        <v>1060</v>
+      </c>
+      <c r="I207" t="s">
+        <v>1061</v>
+      </c>
+    </row>
+    <row r="208" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>1062</v>
+      </c>
+      <c r="B208" t="s">
+        <v>36</v>
+      </c>
+      <c r="C208" t="s">
+        <v>10</v>
+      </c>
+      <c r="D208" t="s">
+        <v>1063</v>
+      </c>
+      <c r="E208" t="s">
+        <v>13</v>
+      </c>
+      <c r="F208" t="s">
+        <v>31</v>
+      </c>
+      <c r="G208" t="s">
+        <v>1064</v>
+      </c>
+      <c r="H208" t="s">
+        <v>1065</v>
+      </c>
+      <c r="I208" t="s">
+        <v>1066</v>
+      </c>
+    </row>
+    <row r="209" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B209" t="s">
+        <v>84</v>
+      </c>
+      <c r="C209" t="s">
+        <v>10</v>
+      </c>
+      <c r="D209" t="s">
+        <v>1068</v>
+      </c>
+      <c r="E209" t="s">
+        <v>13</v>
+      </c>
+      <c r="F209" t="s">
+        <v>31</v>
+      </c>
+      <c r="G209" t="s">
+        <v>1069</v>
+      </c>
+      <c r="H209" t="s">
+        <v>1070</v>
+      </c>
+      <c r="I209" t="s">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="210" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>1072</v>
+      </c>
+      <c r="B210" t="s">
+        <v>36</v>
+      </c>
+      <c r="C210" t="s">
+        <v>10</v>
+      </c>
+      <c r="D210" t="s">
+        <v>1073</v>
+      </c>
+      <c r="E210" t="s">
+        <v>13</v>
+      </c>
+      <c r="F210" t="s">
+        <v>31</v>
+      </c>
+      <c r="G210" t="s">
+        <v>1074</v>
+      </c>
+      <c r="H210" t="s">
+        <v>1075</v>
+      </c>
+      <c r="I210" t="s">
+        <v>1076</v>
+      </c>
+    </row>
+    <row r="211" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B211" t="s">
+        <v>84</v>
+      </c>
+      <c r="C211" t="s">
+        <v>10</v>
+      </c>
+      <c r="D211" t="s">
+        <v>1078</v>
+      </c>
+      <c r="E211" t="s">
+        <v>13</v>
+      </c>
+      <c r="F211" t="s">
+        <v>31</v>
+      </c>
+      <c r="G211" t="s">
+        <v>1079</v>
+      </c>
+      <c r="H211" t="s">
+        <v>1080</v>
+      </c>
+      <c r="I211" t="s">
+        <v>1081</v>
+      </c>
+    </row>
+    <row r="212" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>1082</v>
+      </c>
+      <c r="B212" t="s">
+        <v>29</v>
+      </c>
+      <c r="C212" t="s">
+        <v>10</v>
+      </c>
+      <c r="D212" t="s">
+        <v>1083</v>
+      </c>
+      <c r="E212" t="s">
+        <v>13</v>
+      </c>
+      <c r="F212" t="s">
+        <v>31</v>
+      </c>
+      <c r="G212" t="s">
+        <v>1084</v>
+      </c>
+      <c r="H212" t="s">
+        <v>1085</v>
+      </c>
+      <c r="I212" t="s">
+        <v>1086</v>
+      </c>
+    </row>
+    <row r="213" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B213" t="s">
+        <v>36</v>
+      </c>
+      <c r="C213" t="s">
+        <v>10</v>
+      </c>
+      <c r="D213" t="s">
+        <v>1088</v>
+      </c>
+      <c r="E213" t="s">
+        <v>13</v>
+      </c>
+      <c r="F213" t="s">
+        <v>31</v>
+      </c>
+      <c r="G213" t="s">
+        <v>1089</v>
+      </c>
+      <c r="H213" t="s">
+        <v>1090</v>
+      </c>
+      <c r="I213" t="s">
+        <v>1091</v>
+      </c>
+    </row>
+    <row r="214" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>1092</v>
+      </c>
+      <c r="B214" t="s">
+        <v>36</v>
+      </c>
+      <c r="C214" t="s">
+        <v>10</v>
+      </c>
+      <c r="D214" t="s">
+        <v>1093</v>
+      </c>
+      <c r="E214" t="s">
+        <v>13</v>
+      </c>
+      <c r="F214" t="s">
+        <v>31</v>
+      </c>
+      <c r="G214" t="s">
+        <v>1094</v>
+      </c>
+      <c r="H214" t="s">
+        <v>1095</v>
+      </c>
+      <c r="I214" t="s">
+        <v>1096</v>
+      </c>
+    </row>
+    <row r="215" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>1097</v>
+      </c>
+      <c r="B215" t="s">
+        <v>36</v>
+      </c>
+      <c r="C215" t="s">
+        <v>10</v>
+      </c>
+      <c r="D215" t="s">
+        <v>1098</v>
+      </c>
+      <c r="E215" t="s">
+        <v>13</v>
+      </c>
+      <c r="F215" t="s">
+        <v>31</v>
+      </c>
+      <c r="G215" t="s">
+        <v>1099</v>
+      </c>
+      <c r="H215" t="s">
+        <v>1100</v>
+      </c>
+      <c r="I215" t="s">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="216" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>1102</v>
+      </c>
+      <c r="B216" t="s">
+        <v>90</v>
+      </c>
+      <c r="C216" t="s">
+        <v>10</v>
+      </c>
+      <c r="D216" t="s">
+        <v>1103</v>
+      </c>
+      <c r="E216" t="s">
+        <v>13</v>
+      </c>
+      <c r="F216" t="s">
+        <v>31</v>
+      </c>
+      <c r="G216" t="s">
+        <v>1104</v>
+      </c>
+      <c r="H216" t="s">
+        <v>1105</v>
+      </c>
+      <c r="I216" t="s">
+        <v>1106</v>
+      </c>
+    </row>
+    <row r="217" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>1107</v>
+      </c>
+      <c r="B217" t="s">
+        <v>84</v>
+      </c>
+      <c r="C217" t="s">
+        <v>10</v>
+      </c>
+      <c r="D217" t="s">
+        <v>1108</v>
+      </c>
+      <c r="E217" t="s">
+        <v>13</v>
+      </c>
+      <c r="F217" t="s">
+        <v>31</v>
+      </c>
+      <c r="G217" t="s">
+        <v>1109</v>
+      </c>
+      <c r="H217" t="s">
+        <v>1110</v>
+      </c>
+      <c r="I217" t="s">
+        <v>1111</v>
+      </c>
+    </row>
+    <row r="218" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>1112</v>
+      </c>
+      <c r="B218" t="s">
+        <v>36</v>
+      </c>
+      <c r="C218" t="s">
+        <v>10</v>
+      </c>
+      <c r="D218" t="s">
+        <v>1113</v>
+      </c>
+      <c r="E218" t="s">
+        <v>13</v>
+      </c>
+      <c r="F218" t="s">
+        <v>31</v>
+      </c>
+      <c r="G218" t="s">
+        <v>1114</v>
+      </c>
+      <c r="H218" t="s">
+        <v>1115</v>
+      </c>
+      <c r="I218" t="s">
+        <v>1116</v>
+      </c>
+    </row>
+    <row r="219" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>1117</v>
+      </c>
+      <c r="B219" t="s">
+        <v>36</v>
+      </c>
+      <c r="C219" t="s">
+        <v>10</v>
+      </c>
+      <c r="D219" t="s">
+        <v>1118</v>
+      </c>
+      <c r="E219" t="s">
+        <v>13</v>
+      </c>
+      <c r="F219" t="s">
+        <v>31</v>
+      </c>
+      <c r="G219" t="s">
+        <v>1119</v>
+      </c>
+      <c r="H219" t="s">
+        <v>1120</v>
+      </c>
+      <c r="I219" t="s">
+        <v>1121</v>
+      </c>
+    </row>
+    <row r="220" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>1122</v>
+      </c>
+      <c r="B220" t="s">
+        <v>36</v>
+      </c>
+      <c r="C220" t="s">
+        <v>10</v>
+      </c>
+      <c r="D220" t="s">
+        <v>1123</v>
+      </c>
+      <c r="E220" t="s">
+        <v>13</v>
+      </c>
+      <c r="F220" t="s">
+        <v>31</v>
+      </c>
+      <c r="G220" t="s">
+        <v>1124</v>
+      </c>
+      <c r="H220" t="s">
+        <v>1125</v>
+      </c>
+      <c r="I220" t="s">
+        <v>1126</v>
+      </c>
+    </row>
+    <row r="221" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>1127</v>
+      </c>
+      <c r="B221" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C221" t="s">
+        <v>10</v>
+      </c>
+      <c r="D221" t="s">
+        <v>1129</v>
+      </c>
+      <c r="E221" t="s">
+        <v>13</v>
+      </c>
+      <c r="F221" t="s">
+        <v>31</v>
+      </c>
+      <c r="G221" t="s">
+        <v>1130</v>
+      </c>
+      <c r="H221" t="s">
+        <v>1131</v>
+      </c>
+      <c r="I221" t="s">
+        <v>1132</v>
+      </c>
+    </row>
+    <row r="222" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>1133</v>
+      </c>
+      <c r="B222" t="s">
+        <v>84</v>
+      </c>
+      <c r="C222" t="s">
+        <v>10</v>
+      </c>
+      <c r="D222" t="s">
+        <v>1134</v>
+      </c>
+      <c r="E222" t="s">
+        <v>13</v>
+      </c>
+      <c r="F222" t="s">
+        <v>31</v>
+      </c>
+      <c r="G222" t="s">
+        <v>1135</v>
+      </c>
+      <c r="H222" t="s">
+        <v>1136</v>
+      </c>
+      <c r="I222" t="s">
+        <v>1137</v>
+      </c>
+    </row>
+    <row r="223" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>1138</v>
+      </c>
+      <c r="B223" t="s">
+        <v>36</v>
+      </c>
+      <c r="C223" t="s">
+        <v>10</v>
+      </c>
+      <c r="D223" t="s">
+        <v>1139</v>
+      </c>
+      <c r="E223" t="s">
+        <v>13</v>
+      </c>
+      <c r="F223" t="s">
+        <v>31</v>
+      </c>
+      <c r="G223" t="s">
+        <v>1140</v>
+      </c>
+      <c r="H223" t="s">
+        <v>1141</v>
+      </c>
+      <c r="I223" t="s">
+        <v>1142</v>
+      </c>
+    </row>
+    <row r="224" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>1143</v>
+      </c>
+      <c r="B224" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C224" t="s">
+        <v>10</v>
+      </c>
+      <c r="D224" t="s">
+        <v>1144</v>
+      </c>
+      <c r="E224" t="s">
+        <v>13</v>
+      </c>
+      <c r="F224" t="s">
+        <v>31</v>
+      </c>
+      <c r="G224" t="s">
+        <v>1145</v>
+      </c>
+      <c r="H224" t="s">
+        <v>1146</v>
+      </c>
+      <c r="I224" t="s">
+        <v>1147</v>
+      </c>
+    </row>
+    <row r="225" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>1148</v>
+      </c>
+      <c r="B225" t="s">
+        <v>195</v>
+      </c>
+      <c r="C225" t="s">
+        <v>10</v>
+      </c>
+      <c r="D225" t="s">
+        <v>1149</v>
+      </c>
+      <c r="E225" t="s">
+        <v>13</v>
+      </c>
+      <c r="F225" t="s">
+        <v>31</v>
+      </c>
+      <c r="G225" t="s">
+        <v>1150</v>
+      </c>
+      <c r="H225" t="s">
+        <v>1151</v>
+      </c>
+      <c r="I225" t="s">
+        <v>1152</v>
+      </c>
+    </row>
+    <row r="226" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>1153</v>
+      </c>
+      <c r="B226" t="s">
+        <v>29</v>
+      </c>
+      <c r="C226" t="s">
+        <v>10</v>
+      </c>
+      <c r="D226" t="s">
+        <v>1154</v>
+      </c>
+      <c r="E226" t="s">
+        <v>13</v>
+      </c>
+      <c r="F226" t="s">
+        <v>31</v>
+      </c>
+      <c r="G226" t="s">
+        <v>1155</v>
+      </c>
+      <c r="H226" t="s">
+        <v>1156</v>
+      </c>
+      <c r="I226" t="s">
+        <v>1157</v>
+      </c>
+    </row>
+    <row r="227" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>1158</v>
+      </c>
+      <c r="B227" t="s">
+        <v>36</v>
+      </c>
+      <c r="C227" t="s">
+        <v>10</v>
+      </c>
+      <c r="D227" t="s">
+        <v>1159</v>
+      </c>
+      <c r="E227" t="s">
+        <v>13</v>
+      </c>
+      <c r="F227" t="s">
+        <v>31</v>
+      </c>
+      <c r="G227" t="s">
+        <v>1160</v>
+      </c>
+      <c r="H227" t="s">
+        <v>1161</v>
+      </c>
+      <c r="I227" t="s">
+        <v>1162</v>
+      </c>
+    </row>
+    <row r="228" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>1163</v>
+      </c>
+      <c r="B228" t="s">
+        <v>36</v>
+      </c>
+      <c r="C228" t="s">
+        <v>10</v>
+      </c>
+      <c r="D228" t="s">
+        <v>1164</v>
+      </c>
+      <c r="E228" t="s">
+        <v>13</v>
+      </c>
+      <c r="F228" t="s">
+        <v>31</v>
+      </c>
+      <c r="G228" t="s">
+        <v>1165</v>
+      </c>
+      <c r="H228" t="s">
+        <v>1166</v>
+      </c>
+      <c r="I228" t="s">
+        <v>1167</v>
+      </c>
+    </row>
+    <row r="229" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B229" t="s">
+        <v>36</v>
+      </c>
+      <c r="C229" t="s">
+        <v>10</v>
+      </c>
+      <c r="D229" t="s">
+        <v>1169</v>
+      </c>
+      <c r="E229" t="s">
+        <v>13</v>
+      </c>
+      <c r="F229" t="s">
+        <v>31</v>
+      </c>
+      <c r="G229" t="s">
+        <v>1170</v>
+      </c>
+      <c r="H229" t="s">
+        <v>1171</v>
+      </c>
+      <c r="I229" t="s">
+        <v>1172</v>
+      </c>
+    </row>
+    <row r="230" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
+        <v>1173</v>
+      </c>
+      <c r="B230" t="s">
+        <v>36</v>
+      </c>
+      <c r="C230" t="s">
+        <v>10</v>
+      </c>
+      <c r="D230" t="s">
+        <v>1174</v>
+      </c>
+      <c r="E230" t="s">
+        <v>13</v>
+      </c>
+      <c r="F230" t="s">
+        <v>31</v>
+      </c>
+      <c r="G230" t="s">
+        <v>1175</v>
+      </c>
+      <c r="H230" t="s">
+        <v>1176</v>
+      </c>
+      <c r="I230" t="s">
+        <v>1177</v>
+      </c>
+    </row>
+    <row r="231" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
+        <v>1178</v>
+      </c>
+      <c r="B231" t="s">
+        <v>1179</v>
+      </c>
+      <c r="C231" t="s">
+        <v>10</v>
+      </c>
+      <c r="D231" t="s">
+        <v>1180</v>
+      </c>
+      <c r="E231" t="s">
+        <v>13</v>
+      </c>
+      <c r="F231" t="s">
+        <v>975</v>
+      </c>
+      <c r="G231" t="s">
+        <v>1181</v>
+      </c>
+      <c r="H231" t="s">
+        <v>1182</v>
+      </c>
+      <c r="I231" t="s">
+        <v>1183</v>
+      </c>
+    </row>
+    <row r="232" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>1184</v>
+      </c>
+      <c r="B232" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C232" t="s">
+        <v>10</v>
+      </c>
+      <c r="D232" t="s">
+        <v>1186</v>
+      </c>
+      <c r="E232" t="s">
+        <v>13</v>
+      </c>
+      <c r="F232" t="s">
+        <v>1187</v>
+      </c>
+      <c r="G232" t="s">
+        <v>1188</v>
+      </c>
+      <c r="H232" t="s">
+        <v>1189</v>
+      </c>
+      <c r="I232" t="s">
+        <v>1190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(import): C2-4 (100-years x4) and onboard-delights (x4) re-imported with the rebuilt bundles, uploaded and previewed; spot-checks, fixes.json entries, report rows
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-info.report.xlsx
+++ b/tools/importer/reports/import-info.report.xlsx
@@ -58,7 +58,7 @@
     <t>campaign</t>
   </si>
   <si>
-    <t>2026-10-24T00:59:50.514Z</t>
+    <t>2026-10-24T06:15:40.361Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/100-years</t>
@@ -1840,13 +1840,13 @@
     <t>at/de/onboard-delights.report.json</t>
   </si>
   <si>
-    <t>["hero-campaign","carousel-cards","columns-media","columns-media","columns-media","columns-media"]</t>
+    <t>["profile-tabs","hero-campaign","carousel-cards","columns-media","columns-media","columns-media","columns-media","columns-media"]</t>
   </si>
   <si>
     <t>at/de/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-24T02:45:36.734Z</t>
+    <t>2026-10-24T06:16:17.650Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/onboard-delights</t>
@@ -2626,7 +2626,7 @@
     <t>de/de/100-years</t>
   </si>
   <si>
-    <t>2026-10-24T01:00:35.189Z</t>
+    <t>2026-10-24T06:15:37.900Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/100-years</t>
@@ -4180,7 +4180,7 @@
     <t>de/de/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-24T02:58:13.713Z</t>
+    <t>2026-10-24T06:16:14.552Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/onboard-delights</t>
@@ -4903,7 +4903,7 @@
     <t>de/en/100-years</t>
   </si>
   <si>
-    <t>2026-10-24T01:01:44.043Z</t>
+    <t>2026-10-24T06:15:35.815Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/100-years</t>
@@ -6403,7 +6403,7 @@
     <t>de/en/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-24T03:12:07.501Z</t>
+    <t>2026-10-24T06:16:11.748Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/onboard-delights</t>
@@ -7177,7 +7177,7 @@
     <t>gb/en/100-years</t>
   </si>
   <si>
-    <t>2026-10-24T01:02:23.558Z</t>
+    <t>2026-10-24T06:15:43.344Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/100-years</t>
@@ -8665,7 +8665,7 @@
     <t>gb/en/onboard-delights</t>
   </si>
   <si>
-    <t>2026-10-24T03:25:07.015Z</t>
+    <t>2026-10-24T06:16:20.392Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/onboard-delights</t>

</xml_diff>

<commit_message>
feat(ejournals): .ejournals > .dcep-ejournals mapped in info (new parser: one empty ejournals block after the Login heading instead of the Loading... paragraph); unterhaltung-an-bord x4 re-imported, uploaded and previewed; spot-check, fixes.json entry, report rows
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-info.report.xlsx
+++ b/tools/importer/reports/import-info.report.xlsx
@@ -2485,13 +2485,13 @@
     <t>at/de/unterhaltung-an-bord.report.json</t>
   </si>
   <si>
-    <t>["table-striped","embed"]</t>
+    <t>["table-striped","embed","ejournals"]</t>
   </si>
   <si>
     <t>at/de/unterhaltung-an-bord</t>
   </si>
   <si>
-    <t>2026-10-24T11:14:46.858Z</t>
+    <t>2026-10-25T04:55:17.080Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/unterhaltung-an-bord</t>
@@ -4768,7 +4768,7 @@
     <t>de/de/unterhaltung-an-bord</t>
   </si>
   <si>
-    <t>2026-10-24T11:14:43.900Z</t>
+    <t>2026-10-25T04:55:11.570Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/unterhaltung-an-bord</t>
@@ -7039,7 +7039,7 @@
     <t>de/en/unterhaltung-an-bord</t>
   </si>
   <si>
-    <t>2026-10-24T11:14:40.705Z</t>
+    <t>2026-10-25T04:55:14.363Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/unterhaltung-an-bord</t>
@@ -9295,7 +9295,7 @@
     <t>gb/en/unterhaltung-an-bord</t>
   </si>
   <si>
-    <t>2026-10-24T11:14:49.545Z</t>
+    <t>2026-10-25T04:55:20.097Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/unterhaltung-an-bord</t>

</xml_diff>

<commit_message>
fix(local-pages): flight search over a background image (data-dcep backgroundImageL/S -> Background image rows, full-width 500px band, card at its bottom), the authored destination code shown by name (Cape Town), partner icon teasers in info -> cards-icon-text partner, text-only four-up teaser cards four per row with the teaser card look; the 7 local promotion/event pages re-imported, uploaded and previewed; parity jobs for the 10 market-only pages (build-jobs reads /content/lh/markets)
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-info.report.xlsx
+++ b/tools/importer/reports/import-info.report.xlsx
@@ -9835,7 +9835,7 @@
     <t>at/de/event/esorics-2027</t>
   </si>
   <si>
-    <t>2026-10-25T05:49:11.537Z</t>
+    <t>2026-10-25T06:13:22.603Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/event/esorics-2027</t>
@@ -9895,7 +9895,7 @@
     <t>at/de/local-page/black-friday</t>
   </si>
   <si>
-    <t>2026-10-25T05:49:09.065Z</t>
+    <t>2026-10-25T06:13:20.232Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/local-page/black-friday</t>
@@ -10234,7 +10234,7 @@
     <t>de/de/event/dghm-2026</t>
   </si>
   <si>
-    <t>2026-10-25T05:49:06.296Z</t>
+    <t>2026-10-25T06:13:17.662Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/event/dghm-2026</t>
@@ -10279,13 +10279,13 @@
     <t>de/de/local-page/south-africa-winter-promotion.report.json</t>
   </si>
   <si>
-    <t>["flight-search","hero-campaign","accordion-columns","carousel-cards","carousel-cards","carousel-cards"]</t>
+    <t>["flight-search","hero-campaign","accordion-columns","cards-icon-text","carousel-cards","carousel-cards","carousel-cards"]</t>
   </si>
   <si>
     <t>de/de/local-page/south-africa-winter-promotion</t>
   </si>
   <si>
-    <t>2026-10-25T05:49:00.321Z</t>
+    <t>2026-10-25T06:13:12.675Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/local-page/south-africa-winter-promotion</t>
@@ -10627,7 +10627,7 @@
     <t>de/en/event/dghm-2026</t>
   </si>
   <si>
-    <t>2026-10-25T05:49:03.954Z</t>
+    <t>2026-10-25T06:13:15.060Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/event/dghm-2026</t>
@@ -10675,7 +10675,7 @@
     <t>de/en/local-page/south-africa-winter-promotion</t>
   </si>
   <si>
-    <t>2026-10-25T05:48:57.791Z</t>
+    <t>2026-10-25T06:13:10.276Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/local-page/south-africa-winter-promotion</t>
@@ -11050,7 +11050,7 @@
     <t>gb/en/local-page/ski-campaign-2026</t>
   </si>
   <si>
-    <t>2026-10-25T05:49:13.725Z</t>
+    <t>2026-10-25T06:13:25.732Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/local-page/ski-campaign-2026</t>

</xml_diff>

<commit_message>
fix(importer): a live title that repeats the site suffix ("Help & Contact | Lufthansa | Lufthansa") is imported with one; support/support, travel-briefing and travelling-with-children / fliegen-mit-kindern (all four locales, 12 documents) re-imported, uploaded and previewed; compare-solo reads the alias notes always
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-info.report.xlsx
+++ b/tools/importer/reports/import-info.report.xlsx
@@ -955,7 +955,7 @@
     <t>at/de/fliegen-mit-kindern</t>
   </si>
   <si>
-    <t>2026-10-24T02:41:40.709Z</t>
+    <t>2026-10-25T20:27:06.292Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/fliegen-mit-kindern</t>
@@ -2440,7 +2440,7 @@
     <t>at/de/travel-briefing</t>
   </si>
   <si>
-    <t>2026-10-25T18:49:52.000Z</t>
+    <t>2026-10-25T20:27:09.372Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/travel-briefing</t>
@@ -3409,7 +3409,7 @@
     <t>de/de/fliegen-mit-kindern</t>
   </si>
   <si>
-    <t>2026-10-24T02:55:34.467Z</t>
+    <t>2026-10-25T20:26:55.229Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/fliegen-mit-kindern</t>
@@ -4747,7 +4747,7 @@
     <t>de/de/travel-briefing</t>
   </si>
   <si>
-    <t>2026-10-25T18:49:40.717Z</t>
+    <t>2026-10-25T20:26:58.154Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/travel-briefing</t>
@@ -6994,7 +6994,7 @@
     <t>de/en/travel-briefing</t>
   </si>
   <si>
-    <t>2026-10-25T18:49:30.045Z</t>
+    <t>2026-10-25T20:27:03.008Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/travel-briefing</t>
@@ -7054,7 +7054,7 @@
     <t>de/en/travelling-with-children</t>
   </si>
   <si>
-    <t>2026-10-24T03:15:09.690Z</t>
+    <t>2026-10-25T20:27:00.925Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/travelling-with-children</t>
@@ -9274,7 +9274,7 @@
     <t>gb/en/travel-briefing</t>
   </si>
   <si>
-    <t>2026-10-25T18:50:02.158Z</t>
+    <t>2026-10-25T20:27:13.773Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/travel-briefing</t>
@@ -9334,7 +9334,7 @@
     <t>gb/en/travelling-with-children</t>
   </si>
   <si>
-    <t>2026-10-24T03:29:07.203Z</t>
+    <t>2026-10-25T20:27:11.962Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/travelling-with-children</t>
@@ -10096,7 +10096,7 @@
     <t>at/de/support/support</t>
   </si>
   <si>
-    <t>2026-10-25T19:00:25.961Z</t>
+    <t>2026-10-25T20:27:20.320Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/at/de/support/support</t>
@@ -10522,7 +10522,7 @@
     <t>de/de/support/support</t>
   </si>
   <si>
-    <t>2026-10-25T19:00:23.133Z</t>
+    <t>2026-10-25T20:27:15.757Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/de/support/support</t>
@@ -10948,7 +10948,7 @@
     <t>de/en/support/support</t>
   </si>
   <si>
-    <t>2026-10-25T19:00:20.391Z</t>
+    <t>2026-10-25T20:27:17.894Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/de/en/support/support</t>
@@ -11359,7 +11359,7 @@
     <t>gb/en/support/support</t>
   </si>
   <si>
-    <t>2026-10-25T19:00:28.126Z</t>
+    <t>2026-10-25T20:27:23.033Z</t>
   </si>
   <si>
     <t>https://www.lufthansa.com/gb/en/support/support</t>

</xml_diff>